<commit_message>
fix: update course modules spreadsheet and day 1 presentation slides
</commit_message>
<xml_diff>
--- a/AIASD-311-CourseModules.xlsx
+++ b/AIASD-311-CourseModules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\AIASD\AI-Assisted-Software-Development-Course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AE6F30E-8C88-4D4B-8D46-8A1209F263F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89C0966-987C-4BB2-95CC-E998A62ED176}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="5" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
+    <workbookView xWindow="4583" yWindow="16103" windowWidth="21795" windowHeight="13875" activeTab="6" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
   </bookViews>
   <sheets>
     <sheet name="monday" sheetId="2" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="thursday" sheetId="6" r:id="rId4"/>
     <sheet name="friday" sheetId="7" r:id="rId5"/>
     <sheet name="totals" sheetId="8" r:id="rId6"/>
+    <sheet name="GE Mods" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="210">
   <si>
     <t>CI/CD Pipeline Creation</t>
   </si>
@@ -623,6 +624,54 @@
   </si>
   <si>
     <t>Once the Claude, Visual Studio, and AzDO specific content is created, building any of these permutations would be straight forward.</t>
+  </si>
+  <si>
+    <t>MFC --&gt; WPF</t>
+  </si>
+  <si>
+    <t>C++ --&gt; EF + SQL</t>
+  </si>
+  <si>
+    <t>VS Code UI Tour</t>
+  </si>
+  <si>
+    <t>Day 1 Mods</t>
+  </si>
+  <si>
+    <t>Day 2 Mods</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>Column3</t>
+  </si>
+  <si>
+    <t>Section</t>
+  </si>
+  <si>
+    <t>Hours</t>
+  </si>
+  <si>
+    <t>These are estimates for modifications requested by GE</t>
+  </si>
+  <si>
+    <t>Create a Visual Studio version of this content</t>
+  </si>
+  <si>
+    <t>Investigate support for this feature in Visual Studio and create a Visual Studio version of this content if it is</t>
+  </si>
+  <si>
+    <t>Create content showing how to create a simple MCP server</t>
+  </si>
+  <si>
+    <t>Create an exercise to create a simple MCP server</t>
+  </si>
+  <si>
+    <t>Create slides and exercises for AI assisted dialog transformation</t>
+  </si>
+  <si>
+    <t>Create slides and exercises for AI assisted SQL string to EF transformation</t>
   </si>
 </sst>
 </file>
@@ -822,8 +871,8 @@
       </extLst>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -831,7 +880,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
@@ -846,7 +895,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="115">
+  <dxfs count="116">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
@@ -858,6 +910,38 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+        <bottom/>
+      </border>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <font>
@@ -908,7 +992,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
@@ -972,7 +1056,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
@@ -1036,7 +1120,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
@@ -1111,7 +1195,39 @@
       </border>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="1"/>
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="double">
+          <color theme="4"/>
+        </top>
+        <bottom/>
+      </border>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
         </ext>
       </extLst>
     </dxf>
@@ -1164,7 +1280,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="1" formatCode="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
@@ -1228,7 +1344,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="1" formatCode="0"/>
       <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
@@ -1269,11 +1385,6 @@
         </top>
         <bottom/>
       </border>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <font>
@@ -1303,9 +1414,29 @@
       </border>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
+          <xfpb:DXFComplement i="1"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="double">
+          <color theme="4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1324,256 +1455,18 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="double">
-          <color theme="4"/>
-        </top>
-        <bottom/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
       </border>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="double">
-          <color theme="4"/>
-        </top>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <font>
@@ -1601,33 +1494,6 @@
       </fill>
     </dxf>
     <dxf>
-      <border outline="0">
-        <top style="double">
-          <color theme="4"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <right style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </right>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1636,6 +1502,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1644,6 +1518,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1652,6 +1534,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1660,6 +1550,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1668,6 +1566,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1676,6 +1582,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1685,28 +1599,26 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -1722,6 +1634,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1730,6 +1650,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1738,6 +1666,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1746,10 +1682,36 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -1760,6 +1722,26 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1768,6 +1750,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1776,6 +1766,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1784,6 +1782,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1792,6 +1798,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1800,6 +1814,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1809,36 +1831,42 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -1854,6 +1882,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1862,6 +1898,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1870,6 +1914,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1878,6 +1930,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1886,6 +1946,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1894,6 +1962,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1903,19 +1979,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
@@ -1924,6 +1990,14 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1932,6 +2006,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1940,6 +2022,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1948,6 +2038,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1956,6 +2054,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1964,6 +2070,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1972,6 +2086,14 @@
       </extLst>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -1984,76 +2106,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
@@ -2106,31 +2158,31 @@
   <autoFilter ref="B2:M29" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{9D61239E-9B4A-4932-AB0D-EB9D9921B03D}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="114" totalsRowDxfId="78"/>
+    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="115" totalsRowDxfId="114"/>
     <tableColumn id="5" xr3:uid="{8B6AF1D4-2216-4B85-BA7D-212BA502015B}" name="Duration"/>
     <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description"/>
-    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="113" totalsRowDxfId="77">
+    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="113" totalsRowDxfId="112">
       <calculatedColumnFormula>F2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="112" totalsRowDxfId="76">
+    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="111" totalsRowDxfId="110">
       <totalsRowFormula>COUNTIF(monday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="84" totalsRowDxfId="75">
+    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="109" totalsRowDxfId="108">
       <totalsRowFormula>COUNTIF(monday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="83" totalsRowDxfId="74">
+    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="107" totalsRowDxfId="106">
       <totalsRowFormula>COUNTIF(monday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="82" totalsRowDxfId="73">
+    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="105" totalsRowDxfId="104">
       <totalsRowFormula>COUNTIF(monday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="81" totalsRowDxfId="72">
+    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="103" totalsRowDxfId="102">
       <totalsRowFormula>COUNTIF(monday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="80" totalsRowDxfId="71">
+    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="101" totalsRowDxfId="100">
       <totalsRowFormula>COUNTIF(monday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="79" totalsRowDxfId="70">
+    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="99" totalsRowDxfId="98">
       <totalsRowFormula>COUNTIF(monday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2143,31 +2195,31 @@
   <autoFilter ref="B2:M26" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{A79E8443-E3FC-4A2C-83B2-0E581E8FF9B8}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="69" totalsRowDxfId="60"/>
+    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="97" totalsRowDxfId="96"/>
     <tableColumn id="5" xr3:uid="{C37F49DC-8E37-4F56-B136-B64A492DADC4}" name="Duration"/>
     <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description"/>
-    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="68" totalsRowDxfId="59">
+    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="95" totalsRowDxfId="94">
       <calculatedColumnFormula>F2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="58">
+    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="93" totalsRowDxfId="92">
       <totalsRowFormula>COUNTIF(tuesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="66" totalsRowDxfId="57">
+    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="91" totalsRowDxfId="90">
       <totalsRowFormula>COUNTIF(tuesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="56">
+    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="89" totalsRowDxfId="88">
       <totalsRowFormula>COUNTIF(tuesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="64" totalsRowDxfId="55">
+    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="86">
       <totalsRowFormula>COUNTIF(tuesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="63" totalsRowDxfId="54">
+    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="84">
       <totalsRowFormula>COUNTIF(tuesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="62" totalsRowDxfId="53">
+    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="83" totalsRowDxfId="82">
       <totalsRowFormula>COUNTIF(tuesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="61" totalsRowDxfId="52">
+    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="81" totalsRowDxfId="80">
       <totalsRowFormula>COUNTIF(tuesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2180,31 +2232,31 @@
   <autoFilter ref="B2:M10" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{9E7625E1-2B56-4752-B6F8-BF1B9CB4F92C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="111" totalsRowDxfId="46"/>
+    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="79" totalsRowDxfId="78"/>
     <tableColumn id="5" xr3:uid="{78218F89-BD58-4DD6-9B0D-DCE1B0CA5E74}" name="Duration"/>
     <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description"/>
-    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="110" totalsRowDxfId="45">
+    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="77" totalsRowDxfId="76">
       <calculatedColumnFormula>F2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="109" totalsRowDxfId="44">
+    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="75" totalsRowDxfId="74">
       <totalsRowFormula>COUNTIF(wednesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="108" totalsRowDxfId="43">
+    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="73" totalsRowDxfId="72">
       <totalsRowFormula>COUNTIF(wednesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="107" totalsRowDxfId="42">
+    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="71" totalsRowDxfId="70">
       <totalsRowFormula>COUNTIF(wednesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="106" totalsRowDxfId="41">
+    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="69" totalsRowDxfId="68">
       <totalsRowFormula>COUNTIF(wednesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="105" totalsRowDxfId="40">
+    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
       <totalsRowFormula>COUNTIF(wednesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="104" totalsRowDxfId="39">
+    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="64">
       <totalsRowFormula>COUNTIF(wednesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="103" totalsRowDxfId="38">
+    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="63" totalsRowDxfId="62">
       <totalsRowFormula>COUNTIF(wednesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2217,31 +2269,31 @@
   <autoFilter ref="B2:M14" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{D80C761D-4E7E-4D1A-862A-6769A723C40C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="102" totalsRowDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="61" totalsRowDxfId="60"/>
     <tableColumn id="5" xr3:uid="{F640E5CE-B0CE-4586-AB64-2F877DC1D9FB}" name="Duration"/>
     <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description"/>
-    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="101" totalsRowDxfId="36">
+    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="59" totalsRowDxfId="58">
       <calculatedColumnFormula>F2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="100" totalsRowDxfId="35">
+    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="56">
       <totalsRowFormula>COUNTIF(thursday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="99" totalsRowDxfId="34">
+    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54">
       <totalsRowFormula>COUNTIF(thursday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="98" totalsRowDxfId="33">
+    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="53" totalsRowDxfId="52">
       <totalsRowFormula>COUNTIF(thursday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="32">
+    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="51" totalsRowDxfId="50">
       <totalsRowFormula>COUNTIF(thursday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="96" totalsRowDxfId="31">
+    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="49" totalsRowDxfId="48">
       <totalsRowFormula>COUNTIF(thursday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="30">
+    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="47" totalsRowDxfId="46">
       <totalsRowFormula>COUNTIF(thursday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="94" totalsRowDxfId="29">
+    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="45" totalsRowDxfId="44">
       <totalsRowFormula>COUNTIF(thursday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2254,31 +2306,31 @@
   <autoFilter ref="B2:M23" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{26906033-DBB1-4850-8A65-B0AABB8EB5B7}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="93" totalsRowDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="43" totalsRowDxfId="42"/>
     <tableColumn id="5" xr3:uid="{B474477F-00C6-4EE7-A8CC-63E5347553DE}" name="Duration"/>
     <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description"/>
-    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="92" totalsRowDxfId="27">
+    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="41" totalsRowDxfId="40">
       <calculatedColumnFormula>F2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="91" totalsRowDxfId="26">
+    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="39" totalsRowDxfId="38">
       <totalsRowFormula>COUNTIF(friday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="90" totalsRowDxfId="25">
+    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="37" totalsRowDxfId="36">
       <totalsRowFormula>COUNTIF(friday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="89" totalsRowDxfId="24">
+    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="34">
       <totalsRowFormula>COUNTIF(friday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="88" totalsRowDxfId="23">
+    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="33" totalsRowDxfId="32">
       <totalsRowFormula>COUNTIF(friday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="22">
+    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
       <totalsRowFormula>COUNTIF(friday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="86" totalsRowDxfId="21">
+    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
       <totalsRowFormula>COUNTIF(friday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="20">
+    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
       <totalsRowFormula>COUNTIF(friday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2287,35 +2339,35 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="48" dataDxfId="47" headerRowBorderDxfId="50" tableBorderDxfId="51" totalsRowBorderDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
   <autoFilter ref="B3:I8" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}"/>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="11" totalsRowDxfId="19"/>
-    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="18">
+    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="20" totalsRowDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="18" totalsRowDxfId="17">
       <calculatedColumnFormula>COUNTIF(monday[Copilot],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Copilot])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="9" totalsRowDxfId="17">
+    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="16" totalsRowDxfId="15">
       <calculatedColumnFormula>COUNTIF(monday[Claude],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Claude])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="16">
+    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="13">
       <calculatedColumnFormula>COUNTIF(monday[Visual Studio],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Visual Studio])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="7" totalsRowDxfId="15">
+    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="11">
       <calculatedColumnFormula>COUNTIF(monday[VS Code],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[VS Code])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="6" totalsRowDxfId="14">
+    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
       <calculatedColumnFormula>COUNTIF(monday[GitHub],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[GitHub])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="5" totalsRowDxfId="13">
+    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
       <calculatedColumnFormula>COUNTIF(monday[AzDO],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[AzDO])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="4" totalsRowDxfId="12">
+    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="6" totalsRowDxfId="5">
       <calculatedColumnFormula>COUNTIF(monday[Agnostic],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Agnostic])</totalsRowFormula>
     </tableColumn>
@@ -2325,12 +2377,37 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="C16:E23" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{57A5629B-B8CE-4BC6-BAD3-F09212A4A15E}" name="Table8" displayName="Table8" ref="G28:H33" totalsRowShown="0">
+  <autoFilter ref="G28:H33" xr:uid="{57A5629B-B8CE-4BC6-BAD3-F09212A4A15E}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{97340A0D-C519-465F-8671-FEEA6666F503}" name="Column1"/>
+    <tableColumn id="3" xr3:uid="{B9786568-43CB-4AB0-8E09-6868576B0452}" name="Column3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{EF1BA374-5AD9-4719-9FF3-682D1B38151C}" name="Table9" displayName="Table9" ref="C4:E12" totalsRowCount="1">
+  <autoFilter ref="C4:E11" xr:uid="{EF1BA374-5AD9-4719-9FF3-682D1B38151C}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{7AD14052-080E-4E37-8C5E-B2CB6B097298}" name="Section"/>
+    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{3E1642EC-6329-4B91-8040-267B6F5F8CED}" name="Hours" totalsRowFunction="custom">
+      <totalsRowFormula>SUM(Table9[Hours])</totalsRowFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6471,14 +6548,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDF57F64-64AA-48D6-B233-5D19F1E2205C}">
-  <dimension ref="B2:I25"/>
+  <dimension ref="B2:I33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.453125" customWidth="1"/>
+    <col min="3" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.81640625" customWidth="1"/>
     <col min="8" max="8" width="7.54296875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.26953125" bestFit="1" customWidth="1"/>
   </cols>
@@ -6750,7 +6827,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C17" s="22" t="s">
         <v>52</v>
       </c>
@@ -6761,7 +6838,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C18" s="22" t="s">
         <v>52</v>
       </c>
@@ -6772,7 +6849,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C19" s="22" t="s">
         <v>52</v>
       </c>
@@ -6783,7 +6860,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C20" s="22" t="s">
         <v>188</v>
       </c>
@@ -6794,7 +6871,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C21" s="22" t="s">
         <v>188</v>
       </c>
@@ -6805,7 +6882,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C22" s="22" t="s">
         <v>188</v>
       </c>
@@ -6816,7 +6893,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C23" s="22" t="s">
         <v>188</v>
       </c>
@@ -6827,9 +6904,57 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="G28" t="s">
+        <v>199</v>
+      </c>
+      <c r="H28" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="G29" t="s">
+        <v>194</v>
+      </c>
+      <c r="H29">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="G30" t="s">
+        <v>195</v>
+      </c>
+      <c r="H30">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="G31" t="s">
+        <v>196</v>
+      </c>
+      <c r="H31">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.35">
+      <c r="G32" t="s">
+        <v>197</v>
+      </c>
+      <c r="H32">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="7:8" x14ac:dyDescent="0.35">
+      <c r="G33" t="s">
+        <v>198</v>
+      </c>
+      <c r="H33">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -6839,9 +6964,132 @@
     <mergeCell ref="G2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="2">
+  <tableParts count="3">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1E0D4B9-8091-457D-8F80-D7E20EC6E158}">
+  <dimension ref="C2:E12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="C2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="4" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="C4" t="s">
+        <v>201</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="C5" t="str">
+        <f>monday!B6</f>
+        <v>GitHub Copilot UI Tour</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="C6" t="str">
+        <f>monday!B28</f>
+        <v>Creating Instruction Files with Sessions</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="C7" t="str">
+        <f>tuesday!B17</f>
+        <v>Code Explanation and Analysis</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="C8" t="str">
+        <f>wednesday!B9</f>
+        <v>MCP (Model Context Protocol) Servers</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="C9" t="str">
+        <f>wednesday!B10</f>
+        <v>Exercise: MCP Servers</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="C10" t="s">
+        <v>194</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E10">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+      <c r="C11" t="s">
+        <v>195</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="3:5" x14ac:dyDescent="0.35">
+      <c r="E12">
+        <f>SUM(Table9[Hours])</f>
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(course-modules): update AIASD-311 CourseModules spreadsheet
</commit_message>
<xml_diff>
--- a/AIASD-311-CourseModules.xlsx
+++ b/AIASD-311-CourseModules.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\AIASD\AI-Assisted-Software-Development-Course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19B3AD11-C6BB-437F-AE47-7FA82F086634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941C8383-6279-4D4F-B65F-5DB9CDA5BD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="2" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
   </bookViews>
@@ -225,9 +225,6 @@
     <t>Test Automation &amp; Code Quality</t>
   </si>
   <si>
-    <t>Prompt Guidance Discussion</t>
-  </si>
-  <si>
     <t>Testing Frameworks</t>
   </si>
   <si>
@@ -396,9 +393,6 @@
     <t>AI-assisted test generation (unit, integration, e2e, performance); Intelligent linting beyond static analysis; Coverage analysis and adequacy assessment; Automated quality gates; Continuous deployment strategies</t>
   </si>
   <si>
-    <t>Structured prompting for AI-assisted development; Effective prompt examples; Avoiding literal copying of activity descriptions; Phrase prompts for architectural analysis</t>
-  </si>
-  <si>
     <t>Key Practices: Prune obsolete tests, update with code changes, TDD with AI; Test Review: Detect missing assertions, redundant tests, edge cases; Critical Principle: Validate intent, not implementation; AI-Generated Tests: Create instruction files with test expectations; Trust Building: Use different models for analysis; Key Practices: Prune obsolete tests, update with code changes, TDD with AI; Test Review: Detect missing assertions, redundant tests, edge cases; Critical Principle: Validate intent, not implementation; AI-Generated Tests: Create instruction files with test expectations; Trust Building: Use different models for analysis</t>
   </si>
   <si>
@@ -663,9 +657,6 @@
     <t>_Hands-On with GitHub Copilot (VS Code).pptx</t>
   </si>
   <si>
-    <t>Test Automation &amp; Code Quality.pptx</t>
-  </si>
-  <si>
     <t>github-copilot-chat-mode-personas.pptx</t>
   </si>
   <si>
@@ -1132,6 +1123,15 @@
   </si>
   <si>
     <t>large-language-models.md</t>
+  </si>
+  <si>
+    <t>code-explanation-and-analysis.md</t>
+  </si>
+  <si>
+    <t>test-automation-and-code-quality.md; exercise-test-automation-quality.md</t>
+  </si>
+  <si>
+    <t>feature-flags-and-test-suites.md</t>
   </si>
 </sst>
 </file>
@@ -1431,6 +1431,71 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2543,71 +2608,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2660,7 +2660,7 @@
     <tableColumn id="2" xr3:uid="{B07EACE5-F752-4991-BE23-9BE11BB23286}" name="Column1">
       <calculatedColumnFormula>LOWER(Table11[[#This Row],[Name]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B8942215-B69E-4093-A1A0-3CA4C76B06EE}" name="Column2" dataDxfId="113"/>
+    <tableColumn id="3" xr3:uid="{B8942215-B69E-4093-A1A0-3CA4C76B06EE}" name="Column2" dataDxfId="123"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2671,7 +2671,7 @@
   <autoFilter ref="C4:E11" xr:uid="{EF1BA374-5AD9-4719-9FF3-682D1B38151C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7AD14052-080E-4E37-8C5E-B2CB6B097298}" name="Section"/>
-    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="19"/>
     <tableColumn id="2" xr3:uid="{3E1642EC-6329-4B91-8040-267B6F5F8CED}" name="Hours" totalsRowFunction="custom">
       <totalsRowFormula>SUM(Table9[Hours])</totalsRowFormula>
     </tableColumn>
@@ -2685,33 +2685,33 @@
   <autoFilter ref="C2:P30" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9D61239E-9B4A-4932-AB0D-EB9D9921B03D}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="112" totalsRowDxfId="111"/>
+    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="122" totalsRowDxfId="121"/>
     <tableColumn id="5" xr3:uid="{8B6AF1D4-2216-4B85-BA7D-212BA502015B}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description" dataDxfId="110"/>
+    <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description" dataDxfId="120"/>
     <tableColumn id="19" xr3:uid="{6CD3E0DC-278C-498A-A888-BE6341994574}" name="Deck"/>
     <tableColumn id="18" xr3:uid="{7E153D0B-3D6F-4A51-B6D2-9A0BE0E451DA}" name="Slide(s)"/>
-    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="109" totalsRowDxfId="108">
+    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="119" totalsRowDxfId="118">
       <calculatedColumnFormula>I2 + (E2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="107" totalsRowDxfId="106">
+    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="117" totalsRowDxfId="116">
       <totalsRowFormula>COUNTIF(monday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="105" totalsRowDxfId="104">
+    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="115" totalsRowDxfId="114">
       <totalsRowFormula>COUNTIF(monday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="103" totalsRowDxfId="102">
+    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="113" totalsRowDxfId="112">
       <totalsRowFormula>COUNTIF(monday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="101" totalsRowDxfId="100">
+    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="111" totalsRowDxfId="110">
       <totalsRowFormula>COUNTIF(monday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="99" totalsRowDxfId="98">
+    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="109" totalsRowDxfId="108">
       <totalsRowFormula>COUNTIF(monday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="96">
+    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="107" totalsRowDxfId="106">
       <totalsRowFormula>COUNTIF(monday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="94">
+    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="105" totalsRowDxfId="104">
       <totalsRowFormula>COUNTIF(monday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2720,37 +2720,37 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{790B1945-1A22-4D91-B3FB-F5CFCB0BC598}" name="tuesday" displayName="tuesday" ref="B2:O26" totalsRowCount="1">
-  <autoFilter ref="B2:O25" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{790B1945-1A22-4D91-B3FB-F5CFCB0BC598}" name="tuesday" displayName="tuesday" ref="B2:O25" totalsRowCount="1">
+  <autoFilter ref="B2:O24" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{A79E8443-E3FC-4A2C-83B2-0E581E8FF9B8}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="123" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="18" totalsRowDxfId="8"/>
     <tableColumn id="5" xr3:uid="{C37F49DC-8E37-4F56-B136-B64A492DADC4}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="122"/>
+    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="17"/>
     <tableColumn id="14" xr3:uid="{BD249784-C12F-4B3B-8752-038CF2024DD9}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{E7140FF5-BE1A-4956-A3E4-A572C8619336}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="121" totalsRowDxfId="7">
+    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="16" totalsRowDxfId="7">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="120" totalsRowDxfId="6">
+    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="15" totalsRowDxfId="6">
       <totalsRowFormula>COUNTIF(tuesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="119" totalsRowDxfId="5">
+    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="5">
       <totalsRowFormula>COUNTIF(tuesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="118" totalsRowDxfId="4">
+    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="4">
       <totalsRowFormula>COUNTIF(tuesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="117" totalsRowDxfId="3">
+    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="3">
       <totalsRowFormula>COUNTIF(tuesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="116" totalsRowDxfId="2">
+    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="2">
       <totalsRowFormula>COUNTIF(tuesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="115" totalsRowDxfId="1">
+    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="1">
       <totalsRowFormula>COUNTIF(tuesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="114" totalsRowDxfId="0">
+    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="9" totalsRowDxfId="0">
       <totalsRowFormula>COUNTIF(tuesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2763,33 +2763,33 @@
   <autoFilter ref="B2:O12" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9E7625E1-2B56-4752-B6F8-BF1B9CB4F92C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="93" totalsRowDxfId="92"/>
+    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="103" totalsRowDxfId="102"/>
     <tableColumn id="5" xr3:uid="{78218F89-BD58-4DD6-9B0D-DCE1B0CA5E74}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="91"/>
-    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="90"/>
+    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="101"/>
+    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="100"/>
     <tableColumn id="2" xr3:uid="{06859EAF-BB57-49A2-83C0-AA6CD01CE733}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="89" totalsRowDxfId="88">
+    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="99" totalsRowDxfId="98">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="86">
+    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="96">
       <totalsRowFormula>COUNTIF(wednesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="84">
+    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="94">
       <totalsRowFormula>COUNTIF(wednesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="83" totalsRowDxfId="82">
+    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="93" totalsRowDxfId="92">
       <totalsRowFormula>COUNTIF(wednesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="81" totalsRowDxfId="80">
+    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="91" totalsRowDxfId="90">
       <totalsRowFormula>COUNTIF(wednesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="79" totalsRowDxfId="78">
+    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="89" totalsRowDxfId="88">
       <totalsRowFormula>COUNTIF(wednesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="77" totalsRowDxfId="76">
+    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="86">
       <totalsRowFormula>COUNTIF(wednesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="75" totalsRowDxfId="74">
+    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="84">
       <totalsRowFormula>COUNTIF(wednesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2802,33 +2802,33 @@
   <autoFilter ref="B2:O15" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{D80C761D-4E7E-4D1A-862A-6769A723C40C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="73" totalsRowDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="83" totalsRowDxfId="82"/>
     <tableColumn id="5" xr3:uid="{F640E5CE-B0CE-4586-AB64-2F877DC1D9FB}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="71"/>
-    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="81"/>
+    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="80"/>
     <tableColumn id="2" xr3:uid="{76D09C9B-F732-4E1C-945B-A497FD16EFDB}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="69" totalsRowDxfId="68">
+    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="79" totalsRowDxfId="78">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
+    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="77" totalsRowDxfId="76">
       <totalsRowFormula>COUNTIF(thursday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="64">
+    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="75" totalsRowDxfId="74">
       <totalsRowFormula>COUNTIF(thursday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="63" totalsRowDxfId="62">
+    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="73" totalsRowDxfId="72">
       <totalsRowFormula>COUNTIF(thursday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="61" totalsRowDxfId="60">
+    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="71" totalsRowDxfId="70">
       <totalsRowFormula>COUNTIF(thursday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="58">
+    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="69" totalsRowDxfId="68">
       <totalsRowFormula>COUNTIF(thursday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="56">
+    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
       <totalsRowFormula>COUNTIF(thursday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54">
+    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="64">
       <totalsRowFormula>COUNTIF(thursday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2841,33 +2841,33 @@
   <autoFilter ref="B2:O25" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{26906033-DBB1-4850-8A65-B0AABB8EB5B7}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="53" totalsRowDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="63" totalsRowDxfId="62"/>
     <tableColumn id="5" xr3:uid="{B474477F-00C6-4EE7-A8CC-63E5347553DE}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="61"/>
     <tableColumn id="14" xr3:uid="{DF3B0E26-BDAD-42AF-AA94-ECF071ABBC93}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{FDADF079-31AD-4240-B382-130BDA5B792F}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="50" totalsRowDxfId="49">
+    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="60" totalsRowDxfId="59">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="47">
+    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="58" totalsRowDxfId="57">
       <totalsRowFormula>COUNTIF(friday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="45">
+    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="56" totalsRowDxfId="55">
       <totalsRowFormula>COUNTIF(friday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="44" totalsRowDxfId="43">
+    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="54" totalsRowDxfId="53">
       <totalsRowFormula>COUNTIF(friday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="42" totalsRowDxfId="41">
+    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="52" totalsRowDxfId="51">
       <totalsRowFormula>COUNTIF(friday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="40" totalsRowDxfId="39">
+    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="50" totalsRowDxfId="49">
       <totalsRowFormula>COUNTIF(friday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="38" totalsRowDxfId="37">
+    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="47">
       <totalsRowFormula>COUNTIF(friday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="35">
+    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="45">
       <totalsRowFormula>COUNTIF(friday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2876,35 +2876,35 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31" totalsRowBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="44" dataDxfId="42" headerRowBorderDxfId="43" tableBorderDxfId="41" totalsRowBorderDxfId="40">
   <autoFilter ref="B3:I8" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}"/>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
+    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="37" totalsRowDxfId="36">
       <calculatedColumnFormula>COUNTIF(monday[Copilot],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Copilot])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="25" totalsRowDxfId="24">
+    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="34">
       <calculatedColumnFormula>COUNTIF(monday[Claude],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Claude])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="23" totalsRowDxfId="22">
+    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="33" totalsRowDxfId="32">
       <calculatedColumnFormula>COUNTIF(monday[Visual Studio],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Visual Studio])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="21" totalsRowDxfId="20">
+    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
       <calculatedColumnFormula>COUNTIF(monday[VS Code],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[VS Code])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="19" totalsRowDxfId="18">
+    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
       <calculatedColumnFormula>COUNTIF(monday[GitHub],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[GitHub])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="17" totalsRowDxfId="16">
+    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
       <calculatedColumnFormula>COUNTIF(monday[AzDO],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[AzDO])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="15" totalsRowDxfId="14">
+    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="25" totalsRowDxfId="24">
       <calculatedColumnFormula>COUNTIF(monday[Agnostic],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Agnostic])</totalsRowFormula>
     </tableColumn>
@@ -2914,12 +2914,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="23">
   <autoFilter ref="C16:E23" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3263,42 +3263,42 @@
   <sheetData>
     <row r="3" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="4" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D4" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^chat-mode.pptx</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="5" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C5" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D5" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^creating robust testing frameworks.pptx</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C6" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D6" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3308,7 +3308,7 @@
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C7" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D7" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3318,7 +3318,7 @@
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C8" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D8" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3328,7 +3328,7 @@
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C9" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D9" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3338,7 +3338,7 @@
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D10" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3348,7 +3348,7 @@
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D11" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3358,7 +3358,7 @@
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C12" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D12" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3368,7 +3368,7 @@
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C13" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D13" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3378,7 +3378,7 @@
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C14" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D14" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3388,7 +3388,7 @@
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C15" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D15" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3398,247 +3398,247 @@
     </row>
     <row r="16" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C16" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D16" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^overview of llms.pptx</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="17" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C17" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="D17" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_advanced context techniques.pptx</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="18" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C18" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="D18" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai practitioner resources.pptx</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="19" spans="3:5" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C19" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="D19" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai-development-approaches-comparison.pptx</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
     </row>
     <row r="20" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C20" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="D20" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai-first-vs-prompt-first.pptx</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="21" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C21" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D21" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_building a backlog.pptx</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="22" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C22" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D22" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_building safety nets.pptx</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="23" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C23" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D23" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_conformance &amp; gap analysis.pptx</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="24" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C24" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D24" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot instruction stack.pptx</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="25" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C25" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="D25" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot-instruction-control.pptx</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="26" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C26" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="D26" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot-instruction-files-vs-prompt-files-vs-chatmodes.pptx</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="27" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C27" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D27" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_core instruction files.pptx</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="28" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C28" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D28" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_cqrs-architecture.pptx</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
     </row>
     <row r="29" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C29" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D29" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_custom agents.pptx</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="30" spans="3:5" ht="114" x14ac:dyDescent="0.45">
       <c r="C30" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D30" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_documentation generation &amp; code analysis.pptx</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="31" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C31" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D31" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_essential safety measures.pptx</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="32" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C32" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D32" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_generating implementation prompts &amp; verification.pptx</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="33" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C33" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D33" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_getting started checklist.pptx</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
     </row>
     <row r="34" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C34" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D34" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_github copilot for teams.pptx</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="35" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C35" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D35" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_github-copilot-chat-mode-personas.pptx</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="36" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C36" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D36" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3648,127 +3648,127 @@
     </row>
     <row r="37" spans="3:5" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C37" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D37" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_implementing-vertical-slices.pptx</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="38" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C38" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D38" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instruction files.pptx</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="39" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C39" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D39" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instruction-file-applyto-patterns.pptx</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="40" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C40" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D40" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instructions vs prompts vs custom chat modes.pptx</v>
       </c>
       <c r="E40" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="41" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C41" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D41" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_managing github copilot effectively.pptx</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
     </row>
     <row r="42" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C42" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D42" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_mcp servers.pptx</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="43" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C43" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D43" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_mcp-servers-vscode-copilot.pptx</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="44" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C44" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D44" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_model selection &amp; comparison.pptx</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="45" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C45" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D45" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_multi‑model implementation comparison.pptx</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="46" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C46" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D46" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_prompt files.pptx</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="47" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C47" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D47" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3778,31 +3778,31 @@
     </row>
     <row r="48" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C48" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D48" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_safe brownfield coding.pptx</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="49" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C49" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D49" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_starting with project requirements.pptx</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="50" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C50" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D50" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3812,7 +3812,7 @@
     </row>
     <row r="51" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C51" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="D51" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3822,7 +3822,7 @@
     </row>
     <row r="52" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C52" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D52" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3832,7 +3832,7 @@
     </row>
     <row r="53" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C53" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D53" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3842,7 +3842,7 @@
     </row>
     <row r="54" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C54" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D54" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3852,7 +3852,7 @@
     </row>
     <row r="55" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C55" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D55" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3862,7 +3862,7 @@
     </row>
     <row r="56" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C56" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="D56" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3872,7 +3872,7 @@
     </row>
     <row r="57" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C57" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D57" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3882,7 +3882,7 @@
     </row>
     <row r="58" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C58" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="D58" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3892,26 +3892,26 @@
     </row>
     <row r="59" spans="3:5" ht="156.75" x14ac:dyDescent="0.45">
       <c r="C59" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D59" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>adding ai guardrails.pptx</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="60" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C60" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="D60" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_addressing technical debt.pptx</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
   </sheetData>
@@ -3951,10 +3951,10 @@
         <v>4</v>
       </c>
       <c r="G2" t="s">
+        <v>187</v>
+      </c>
+      <c r="H2" t="s">
         <v>189</v>
-      </c>
-      <c r="H2" t="s">
-        <v>191</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>28</v>
@@ -3995,10 +3995,10 @@
         <v>6</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="I3" s="6" t="str">
         <f>I2</f>
@@ -4028,19 +4028,19 @@
     </row>
     <row r="4" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E4">
         <v>5</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I4" s="1">
         <f>I3 + (E3/ 1440)</f>
@@ -4079,13 +4079,13 @@
         <v>10</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" ref="I5:I30" si="0">I4 + (E4/ 1440)</f>
@@ -4121,7 +4121,7 @@
         <v>10</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>33</v>
@@ -4164,10 +4164,10 @@
         <v>15</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="1">
@@ -4198,16 +4198,16 @@
     </row>
     <row r="8" spans="3:16" ht="57" x14ac:dyDescent="0.45">
       <c r="C8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E8">
         <v>70</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H8" s="2">
         <v>2</v>
@@ -4240,7 +4240,7 @@
     </row>
     <row r="9" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C9" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -4249,7 +4249,7 @@
         <v>11</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H9" s="2">
         <v>11</v>
@@ -4282,7 +4282,7 @@
     </row>
     <row r="10" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -4291,7 +4291,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H10" s="2">
         <v>12</v>
@@ -4324,16 +4324,16 @@
     </row>
     <row r="11" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H11" s="2">
         <v>13</v>
@@ -4366,16 +4366,16 @@
     </row>
     <row r="12" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C12" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="H12" s="2">
         <v>14</v>
@@ -4408,16 +4408,16 @@
     </row>
     <row r="13" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C13" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H13" s="2">
         <v>15</v>
@@ -4462,7 +4462,7 @@
         <v>13</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="1">
@@ -4505,7 +4505,7 @@
         <v>15</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="1">
@@ -4748,7 +4748,7 @@
         <v>27</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="1">
@@ -4791,7 +4791,7 @@
         <v>25</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="1">
@@ -4822,13 +4822,13 @@
     </row>
     <row r="23" spans="3:16" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C23" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="1">
@@ -4859,13 +4859,13 @@
     </row>
     <row r="24" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C24" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="G24" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="1">
@@ -4896,13 +4896,13 @@
     </row>
     <row r="25" spans="3:16" ht="99.75" x14ac:dyDescent="0.45">
       <c r="C25" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="1">
@@ -4939,10 +4939,10 @@
         <v>40</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="1">
@@ -4979,10 +4979,10 @@
         <v>5</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="H27" s="2"/>
       <c r="I27" s="1">
@@ -5019,10 +5019,10 @@
         <v>15</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="1">
@@ -5053,16 +5053,16 @@
     </row>
     <row r="29" spans="3:16" ht="57" x14ac:dyDescent="0.45">
       <c r="C29" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E29">
         <v>20</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G29" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="I29" s="1">
         <f t="shared" si="0"/>
@@ -5098,10 +5098,10 @@
         <v>5</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G30" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="I30" s="1">
         <f t="shared" si="0"/>
@@ -5172,7 +5172,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6092BCC8-4678-4A74-B9FA-42E487B327B3}">
-  <dimension ref="B2:O26"/>
+  <dimension ref="B2:O25"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="40.06640625" customWidth="1"/>
@@ -5197,10 +5197,10 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>28</v>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="E3" s="2"/>
       <c r="F3" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="H3" s="6" t="str">
         <f>H2</f>
@@ -5276,13 +5276,13 @@
         <v>5</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F4" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="H4" s="1">
-        <f t="shared" ref="H4:H25" si="0">H3 + (D3/ 1440)</f>
+        <f t="shared" ref="H4:H24" si="0">H3 + (D3/ 1440)</f>
         <v>0.4236111111111111</v>
       </c>
       <c r="I4" s="5" t="b">
@@ -5316,10 +5316,10 @@
         <v>5</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F5" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" si="0"/>
@@ -5349,7 +5349,7 @@
     </row>
     <row r="6" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B6" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C6" s="7">
         <v>6.2500000000000003E-3</v>
@@ -5361,7 +5361,7 @@
         <v>7</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="1">
@@ -5404,7 +5404,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="1">
@@ -5444,10 +5444,10 @@
         <v>20</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F8" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="H8" s="1">
         <f>H9 + (D9/ 1440)</f>
@@ -5489,7 +5489,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="1">
@@ -5529,10 +5529,10 @@
         <v>10</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F10" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="H10" s="1">
         <f>H8 + (D8/ 1440)</f>
@@ -5562,19 +5562,19 @@
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D11">
         <v>15</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F11" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="H11" s="1">
-        <f t="shared" si="0"/>
+        <f>H10 + (D10/ 1440)</f>
         <v>0.46527777777777768</v>
       </c>
       <c r="I11" s="5" t="b">
@@ -5601,7 +5601,7 @@
     </row>
     <row r="12" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="C12" s="1">
         <v>2.013888888888889E-2</v>
@@ -5610,13 +5610,13 @@
         <v>20</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F12" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="H12" s="1">
-        <f t="shared" si="0"/>
+        <f>H11 + (D11/ 1440)</f>
         <v>0.47569444444444436</v>
       </c>
       <c r="I12" s="5" t="b">
@@ -5652,13 +5652,13 @@
         <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F13" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="H13" s="1">
-        <f t="shared" si="0"/>
+        <f>H12 + (D12/ 1440)</f>
         <v>0.48958333333333326</v>
       </c>
       <c r="I13" s="5" t="b">
@@ -5727,10 +5727,10 @@
         <v>20</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F15" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="H15" s="1">
         <f t="shared" si="0"/>
@@ -5769,10 +5769,10 @@
         <v>10</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F16" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="H16" s="1">
         <f t="shared" si="0"/>
@@ -5808,9 +5808,11 @@
         <v>10</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F17"/>
+        <v>108</v>
+      </c>
+      <c r="F17" t="s">
+        <v>360</v>
+      </c>
       <c r="H17" s="1">
         <f t="shared" si="0"/>
         <v>0.56597222222222199</v>
@@ -5845,10 +5847,10 @@
         <v>10</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F18" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="H18" s="1">
         <f t="shared" si="0"/>
@@ -5884,10 +5886,10 @@
         <v>5</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F19" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H19" s="1">
         <f t="shared" si="0"/>
@@ -5917,16 +5919,16 @@
     </row>
     <row r="20" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D20">
         <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F20" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H20" s="1">
         <f t="shared" si="0"/>
@@ -5962,10 +5964,10 @@
         <v>5</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F21" t="s">
-        <v>206</v>
+        <v>361</v>
       </c>
       <c r="H21" s="1">
         <f t="shared" si="0"/>
@@ -5993,17 +5995,22 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:15" ht="156.75" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
         <v>60</v>
       </c>
+      <c r="C22" s="1">
+        <v>1.2500000000000001E-2</v>
+      </c>
       <c r="D22">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="F22"/>
+        <v>116</v>
+      </c>
+      <c r="F22" t="s">
+        <v>350</v>
+      </c>
       <c r="H22" s="1" t="e">
         <f>#REF! + (#REF!/ 1440)</f>
         <v>#REF!</v>
@@ -6030,21 +6037,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:15" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
         <v>61</v>
       </c>
       <c r="C23" s="1">
-        <v>1.2500000000000001E-2</v>
+        <v>2.361111111111111E-2</v>
       </c>
       <c r="D23">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F23" t="s">
-        <v>353</v>
+        <v>362</v>
       </c>
       <c r="H23" s="1" t="e">
         <f t="shared" si="0"/>
@@ -6072,20 +6079,22 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
         <v>62</v>
       </c>
       <c r="C24" s="1">
-        <v>2.361111111111111E-2</v>
+        <v>2.5694444444444443E-2</v>
       </c>
       <c r="D24">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="F24"/>
+        <v>118</v>
+      </c>
+      <c r="F24" t="s">
+        <v>349</v>
+      </c>
       <c r="H24" s="1" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
@@ -6112,78 +6121,36 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="B25" t="s">
-        <v>63</v>
-      </c>
-      <c r="C25" s="1">
-        <v>2.5694444444444443E-2</v>
-      </c>
-      <c r="D25">
-        <v>5</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="F25" t="s">
-        <v>352</v>
-      </c>
-      <c r="H25" s="1" t="e">
-        <f t="shared" si="0"/>
-        <v>#REF!</v>
-      </c>
-      <c r="I25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O25" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="F26"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="16">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="F25"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="16">
         <f>COUNTIF(tuesday[Copilot],TRUE)</f>
         <v>8</v>
       </c>
-      <c r="J26" s="16">
+      <c r="J25" s="16">
         <f>COUNTIF(tuesday[Claude],TRUE)</f>
         <v>8</v>
       </c>
-      <c r="K26" s="16">
+      <c r="K25" s="16">
         <f>COUNTIF(tuesday[Visual Studio],TRUE)</f>
         <v>2</v>
       </c>
-      <c r="L26" s="16">
+      <c r="L25" s="16">
         <f>COUNTIF(tuesday[VS Code],TRUE)</f>
         <v>1</v>
       </c>
-      <c r="M26" s="16">
+      <c r="M25" s="16">
         <f>COUNTIF(tuesday[GitHub],TRUE)</f>
         <v>1</v>
       </c>
-      <c r="N26" s="16">
+      <c r="N25" s="16">
         <f>COUNTIF(tuesday[AzDO],TRUE)</f>
         <v>2</v>
       </c>
-      <c r="O26" s="16">
+      <c r="O25" s="16">
         <f>COUNTIF(tuesday[Agnostic],TRUE)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -6222,10 +6189,10 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>28</v>
@@ -6292,13 +6259,13 @@
     </row>
     <row r="4" spans="2:15" ht="199.5" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="H4" s="6">
         <f>H3 + (D3/ 1440)</f>
@@ -6328,16 +6295,16 @@
     </row>
     <row r="5" spans="2:15" ht="171" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D5">
         <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="H5" s="1">
         <f>H3 + (D3/ 1440)</f>
@@ -6367,13 +6334,13 @@
     </row>
     <row r="6" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="H6" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6403,14 +6370,14 @@
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B7" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="4">
         <v>15</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F7" s="2"/>
       <c r="H7" s="1">
@@ -6441,16 +6408,16 @@
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D8">
         <v>40</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="H8" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -6480,13 +6447,13 @@
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D9">
         <v>40</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F9" s="2"/>
       <c r="H9" s="1">
@@ -6517,13 +6484,13 @@
     </row>
     <row r="10" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D10">
         <v>5</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F10" s="2"/>
       <c r="H10" s="1">
@@ -6554,17 +6521,17 @@
     </row>
     <row r="11" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B11" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="4">
         <v>15</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="H11" s="1">
         <f>H10 + (D10/ 1440)</f>
@@ -6594,14 +6561,14 @@
     </row>
     <row r="12" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B12" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13">
         <v>40</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F12" s="2"/>
       <c r="H12" s="1">
@@ -6697,10 +6664,10 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>28</v>
@@ -6767,16 +6734,16 @@
     </row>
     <row r="4" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D4">
         <v>20</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="H4" s="1">
         <f>H3 + (D3/ 1440)</f>
@@ -6806,13 +6773,13 @@
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D5">
         <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F5" s="2"/>
       <c r="H5" s="1">
@@ -6843,16 +6810,16 @@
     </row>
     <row r="6" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D6">
         <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H6" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6888,10 +6855,10 @@
         <v>10</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="H7" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6921,13 +6888,13 @@
     </row>
     <row r="8" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D8">
         <v>15</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F8" s="2"/>
       <c r="H8" s="1">
@@ -6958,13 +6925,13 @@
     </row>
     <row r="9" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D9">
         <v>20</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F9" s="2"/>
       <c r="H9" s="1">
@@ -7001,10 +6968,10 @@
         <v>45</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="H10" s="1">
         <f t="shared" si="0"/>
@@ -7075,7 +7042,7 @@
         <v>15</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F12" s="2"/>
       <c r="H12" s="1">
@@ -7106,16 +7073,16 @@
     </row>
     <row r="13" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D13">
         <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="H13" s="1">
         <f t="shared" si="0"/>
@@ -7145,13 +7112,13 @@
     </row>
     <row r="14" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D14">
         <v>45</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F14" s="2"/>
       <c r="H14" s="1">
@@ -7182,13 +7149,13 @@
     </row>
     <row r="15" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D15">
         <v>30</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F15" s="2"/>
       <c r="H15" s="1">
@@ -7284,10 +7251,10 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>28</v>
@@ -7354,13 +7321,13 @@
     </row>
     <row r="4" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D4">
         <v>5</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F4"/>
       <c r="H4" s="1">
@@ -7391,7 +7358,7 @@
     </row>
     <row r="5" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C5" s="1">
         <v>4.8611111111111112E-3</v>
@@ -7400,7 +7367,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F5"/>
       <c r="H5" s="1">
@@ -7431,13 +7398,13 @@
     </row>
     <row r="6" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D6">
         <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F6"/>
       <c r="H6" s="1">
@@ -7468,16 +7435,16 @@
     </row>
     <row r="7" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7">
         <v>5</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F7" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="H7" s="1">
         <f>H6 + (D6/ 1440)</f>
@@ -7507,13 +7474,13 @@
     </row>
     <row r="8" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="F8" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="H8" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -7543,16 +7510,16 @@
     </row>
     <row r="9" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D9">
         <v>15</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F9" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="H9" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -7582,13 +7549,13 @@
     </row>
     <row r="10" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F10" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="H10" s="1">
         <f>H9 + (D9/ 1440)</f>
@@ -7618,13 +7585,13 @@
     </row>
     <row r="11" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D11">
         <v>15</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F11"/>
       <c r="H11" s="1">
@@ -7655,16 +7622,16 @@
     </row>
     <row r="12" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D12">
         <v>20</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F12" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="H12" s="1">
         <f t="shared" ref="H12:H25" si="0">H11 + (D11/ 1440)</f>
@@ -7694,13 +7661,13 @@
     </row>
     <row r="13" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D13">
         <v>15</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H13" s="1">
         <f t="shared" si="0"/>
@@ -7730,13 +7697,13 @@
     </row>
     <row r="14" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D14">
         <v>5</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F14"/>
       <c r="H14" s="1">
@@ -7767,13 +7734,13 @@
     </row>
     <row r="15" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D15">
         <v>5</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F15"/>
       <c r="H15" s="1">
@@ -7804,13 +7771,13 @@
     </row>
     <row r="16" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D16">
         <v>10</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F16"/>
       <c r="H16" s="1">
@@ -7876,16 +7843,16 @@
     </row>
     <row r="18" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D18">
         <v>20</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F18" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="H18" s="1">
         <f t="shared" si="0"/>
@@ -7915,16 +7882,16 @@
     </row>
     <row r="19" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D19">
         <v>40</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F19" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="H19" s="1">
         <f t="shared" si="0"/>
@@ -7954,13 +7921,13 @@
     </row>
     <row r="20" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D20">
         <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F20"/>
       <c r="H20" s="1">
@@ -7991,13 +7958,13 @@
     </row>
     <row r="21" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D21">
         <v>5</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F21"/>
       <c r="H21" s="1">
@@ -8028,13 +7995,13 @@
     </row>
     <row r="22" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D22">
         <v>20</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F22"/>
       <c r="H22" s="1">
@@ -8065,13 +8032,13 @@
     </row>
     <row r="23" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D23">
         <v>15</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F23"/>
       <c r="H23" s="1">
@@ -8102,13 +8069,13 @@
     </row>
     <row r="24" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D24">
         <v>10</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F24"/>
       <c r="H24" s="1">
@@ -8139,13 +8106,13 @@
     </row>
     <row r="25" spans="2:15" ht="99.75" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D25">
         <v>10</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F25"/>
       <c r="H25" s="1">
@@ -8230,21 +8197,21 @@
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.45">
       <c r="C2" s="25" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D2" s="25"/>
       <c r="E2" s="25" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F2" s="25"/>
       <c r="G2" s="25" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H2" s="25"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B3" s="17" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C3" s="17" t="s">
         <v>39</v>
@@ -8270,7 +8237,7 @@
     </row>
     <row r="4" spans="2:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="18" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C4" s="20">
         <f>COUNTIF(monday[Copilot],TRUE)</f>
@@ -8303,7 +8270,7 @@
     </row>
     <row r="5" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B5" s="19" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C5" s="20">
         <f>COUNTIF(tuesday[Copilot],TRUE)</f>
@@ -8331,12 +8298,12 @@
       </c>
       <c r="I5" s="20">
         <f>COUNTIF(tuesday[Agnostic],TRUE)</f>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B6" s="19" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C6" s="20">
         <f>COUNTIF(wednesday[Copilot],TRUE)</f>
@@ -8369,7 +8336,7 @@
     </row>
     <row r="7" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="19" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C7" s="20">
         <f>COUNTIF(thursday[Copilot],TRUE)</f>
@@ -8402,7 +8369,7 @@
     </row>
     <row r="8" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="19" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C8" s="20">
         <f>COUNTIF(friday[Copilot],TRUE)</f>
@@ -8461,38 +8428,38 @@
       </c>
       <c r="I9" s="21">
         <f>SUM(Totals[Agnostic])</f>
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.45">
       <c r="C16" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="E16" s="22" t="s">
         <v>168</v>
-      </c>
-      <c r="D16" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="E16" s="22" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.45">
@@ -8530,7 +8497,7 @@
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C20" s="22" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D20" s="22" t="s">
         <v>41</v>
@@ -8541,7 +8508,7 @@
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C21" s="22" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D21" s="22" t="s">
         <v>41</v>
@@ -8552,7 +8519,7 @@
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C22" s="22" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D22" s="22" t="s">
         <v>42</v>
@@ -8563,7 +8530,7 @@
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C23" s="22" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D23" s="22" t="s">
         <v>42</v>
@@ -8574,20 +8541,20 @@
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G28" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H28" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G29" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H29">
         <v>8</v>
@@ -8595,7 +8562,7 @@
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G30" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H30">
         <v>8</v>
@@ -8603,7 +8570,7 @@
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G31" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="H31">
         <v>2</v>
@@ -8611,7 +8578,7 @@
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G32" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H32">
         <v>4</v>
@@ -8619,7 +8586,7 @@
     </row>
     <row r="33" spans="7:8" x14ac:dyDescent="0.45">
       <c r="G33" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H33">
         <v>2</v>
@@ -8652,18 +8619,18 @@
   <sheetData>
     <row r="2" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
@@ -8672,7 +8639,7 @@
         <v>GitHub Copilot UI Tour</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -8684,7 +8651,7 @@
         <v>#REF!</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -8696,7 +8663,7 @@
         <v>Code Explanation and Analysis</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -8708,7 +8675,7 @@
         <v>MCP (Model Context Protocol) Servers</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E8">
         <v>2</v>
@@ -8720,7 +8687,7 @@
         <v>Exercise: MCP Servers</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -8728,10 +8695,10 @@
     </row>
     <row r="10" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E10">
         <v>8</v>
@@ -8739,10 +8706,10 @@
     </row>
     <row r="11" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E11">
         <v>8</v>

</xml_diff>

<commit_message>
Add AIASD Class 311 Tuesday draft presentation and course modules spreadsheet
</commit_message>
<xml_diff>
--- a/AIASD-311-CourseModules.xlsx
+++ b/AIASD-311-CourseModules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\AIASD\AI-Assisted-Software-Development-Course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941C8383-6279-4D4F-B65F-5DB9CDA5BD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D69D90E-DBDD-4524-8EB1-2FF0DE49DD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="2" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
+    <workbookView xWindow="4583" yWindow="16103" windowWidth="21795" windowHeight="13875" activeTab="3" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
   </bookViews>
   <sheets>
     <sheet name="decks" sheetId="10" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="364">
   <si>
     <t>CI/CD Pipeline Creation</t>
   </si>
@@ -1132,6 +1132,9 @@
   </si>
   <si>
     <t>feature-flags-and-test-suites.md</t>
+  </si>
+  <si>
+    <t>skills.md</t>
   </si>
 </sst>
 </file>
@@ -1431,6 +1434,68 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
@@ -2350,7 +2415,7 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2366,7 +2431,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2382,7 +2447,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2398,7 +2463,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2407,74 +2472,12 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
@@ -2671,7 +2674,7 @@
   <autoFilter ref="C4:E11" xr:uid="{EF1BA374-5AD9-4719-9FF3-682D1B38151C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7AD14052-080E-4E37-8C5E-B2CB6B097298}" name="Section"/>
-    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="28"/>
     <tableColumn id="2" xr3:uid="{3E1642EC-6329-4B91-8040-267B6F5F8CED}" name="Hours" totalsRowFunction="custom">
       <totalsRowFormula>SUM(Table9[Hours])</totalsRowFormula>
     </tableColumn>
@@ -2724,33 +2727,33 @@
   <autoFilter ref="B2:O24" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{A79E8443-E3FC-4A2C-83B2-0E581E8FF9B8}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="18" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="27" totalsRowDxfId="17"/>
     <tableColumn id="5" xr3:uid="{C37F49DC-8E37-4F56-B136-B64A492DADC4}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="26"/>
     <tableColumn id="14" xr3:uid="{BD249784-C12F-4B3B-8752-038CF2024DD9}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{E7140FF5-BE1A-4956-A3E4-A572C8619336}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="16" totalsRowDxfId="7">
+    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="25" totalsRowDxfId="16">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="15" totalsRowDxfId="6">
+    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="24" totalsRowDxfId="15">
       <totalsRowFormula>COUNTIF(tuesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="5">
+    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="23" totalsRowDxfId="14">
       <totalsRowFormula>COUNTIF(tuesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="4">
+    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="22" totalsRowDxfId="13">
       <totalsRowFormula>COUNTIF(tuesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="3">
+    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="21" totalsRowDxfId="12">
       <totalsRowFormula>COUNTIF(tuesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="2">
+    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="20" totalsRowDxfId="11">
       <totalsRowFormula>COUNTIF(tuesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="1">
+    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="19" totalsRowDxfId="10">
       <totalsRowFormula>COUNTIF(tuesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="9" totalsRowDxfId="0">
+    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="18" totalsRowDxfId="9">
       <totalsRowFormula>COUNTIF(tuesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2763,33 +2766,33 @@
   <autoFilter ref="B2:O12" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9E7625E1-2B56-4752-B6F8-BF1B9CB4F92C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="103" totalsRowDxfId="102"/>
+    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="103" totalsRowDxfId="8"/>
     <tableColumn id="5" xr3:uid="{78218F89-BD58-4DD6-9B0D-DCE1B0CA5E74}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="101"/>
-    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="100"/>
+    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="102"/>
+    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="101"/>
     <tableColumn id="2" xr3:uid="{06859EAF-BB57-49A2-83C0-AA6CD01CE733}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="99" totalsRowDxfId="98">
+    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="100" totalsRowDxfId="7">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="96">
+    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="99" totalsRowDxfId="6">
       <totalsRowFormula>COUNTIF(wednesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="94">
+    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="98" totalsRowDxfId="5">
       <totalsRowFormula>COUNTIF(wednesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="93" totalsRowDxfId="92">
+    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="4">
       <totalsRowFormula>COUNTIF(wednesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="91" totalsRowDxfId="90">
+    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="96" totalsRowDxfId="3">
       <totalsRowFormula>COUNTIF(wednesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="89" totalsRowDxfId="88">
+    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="2">
       <totalsRowFormula>COUNTIF(wednesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="86">
+    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="94" totalsRowDxfId="1">
       <totalsRowFormula>COUNTIF(wednesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="84">
+    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="93" totalsRowDxfId="0">
       <totalsRowFormula>COUNTIF(wednesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2802,33 +2805,33 @@
   <autoFilter ref="B2:O15" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{D80C761D-4E7E-4D1A-862A-6769A723C40C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="83" totalsRowDxfId="82"/>
+    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="92" totalsRowDxfId="91"/>
     <tableColumn id="5" xr3:uid="{F640E5CE-B0CE-4586-AB64-2F877DC1D9FB}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="81"/>
-    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="80"/>
+    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="90"/>
+    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="89"/>
     <tableColumn id="2" xr3:uid="{76D09C9B-F732-4E1C-945B-A497FD16EFDB}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="79" totalsRowDxfId="78">
+    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="88" totalsRowDxfId="87">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="77" totalsRowDxfId="76">
+    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="86" totalsRowDxfId="85">
       <totalsRowFormula>COUNTIF(thursday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="75" totalsRowDxfId="74">
+    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="84" totalsRowDxfId="83">
       <totalsRowFormula>COUNTIF(thursday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="73" totalsRowDxfId="72">
+    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="82" totalsRowDxfId="81">
       <totalsRowFormula>COUNTIF(thursday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="71" totalsRowDxfId="70">
+    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="80" totalsRowDxfId="79">
       <totalsRowFormula>COUNTIF(thursday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="69" totalsRowDxfId="68">
+    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="78" totalsRowDxfId="77">
       <totalsRowFormula>COUNTIF(thursday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
+    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="76" totalsRowDxfId="75">
       <totalsRowFormula>COUNTIF(thursday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="64">
+    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="74" totalsRowDxfId="73">
       <totalsRowFormula>COUNTIF(thursday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2841,33 +2844,33 @@
   <autoFilter ref="B2:O25" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{26906033-DBB1-4850-8A65-B0AABB8EB5B7}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="63" totalsRowDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="72" totalsRowDxfId="71"/>
     <tableColumn id="5" xr3:uid="{B474477F-00C6-4EE7-A8CC-63E5347553DE}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="61"/>
+    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="70"/>
     <tableColumn id="14" xr3:uid="{DF3B0E26-BDAD-42AF-AA94-ECF071ABBC93}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{FDADF079-31AD-4240-B382-130BDA5B792F}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="60" totalsRowDxfId="59">
+    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="69" totalsRowDxfId="68">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="58" totalsRowDxfId="57">
+    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
       <totalsRowFormula>COUNTIF(friday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="56" totalsRowDxfId="55">
+    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="64">
       <totalsRowFormula>COUNTIF(friday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="54" totalsRowDxfId="53">
+    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="63" totalsRowDxfId="62">
       <totalsRowFormula>COUNTIF(friday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="52" totalsRowDxfId="51">
+    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="61" totalsRowDxfId="60">
       <totalsRowFormula>COUNTIF(friday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="50" totalsRowDxfId="49">
+    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="58">
       <totalsRowFormula>COUNTIF(friday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="47">
+    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="56">
       <totalsRowFormula>COUNTIF(friday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="45">
+    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54">
       <totalsRowFormula>COUNTIF(friday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2876,35 +2879,35 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="44" dataDxfId="42" headerRowBorderDxfId="43" tableBorderDxfId="41" totalsRowBorderDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50" totalsRowBorderDxfId="49">
   <autoFilter ref="B3:I8" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}"/>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="39" totalsRowDxfId="38"/>
-    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="37" totalsRowDxfId="36">
+    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="45">
       <calculatedColumnFormula>COUNTIF(monday[Copilot],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Copilot])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="34">
+    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="44" totalsRowDxfId="43">
       <calculatedColumnFormula>COUNTIF(monday[Claude],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Claude])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="33" totalsRowDxfId="32">
+    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="42" totalsRowDxfId="41">
       <calculatedColumnFormula>COUNTIF(monday[Visual Studio],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Visual Studio])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
+    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="40" totalsRowDxfId="39">
       <calculatedColumnFormula>COUNTIF(monday[VS Code],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[VS Code])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
+    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="38" totalsRowDxfId="37">
       <calculatedColumnFormula>COUNTIF(monday[GitHub],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[GitHub])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
+    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="35">
       <calculatedColumnFormula>COUNTIF(monday[AzDO],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[AzDO])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="25" totalsRowDxfId="24">
+    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="34" totalsRowDxfId="33">
       <calculatedColumnFormula>COUNTIF(monday[Agnostic],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Agnostic])</totalsRowFormula>
     </tableColumn>
@@ -2914,12 +2917,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="32">
   <autoFilter ref="C16:E23" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6379,7 +6382,9 @@
       <c r="E7" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="F7" s="2"/>
+      <c r="F7" s="2" t="s">
+        <v>363</v>
+      </c>
       <c r="H7" s="1">
         <f>H5 + (D5/ 1440)</f>
         <v>0.43750000000000006</v>
@@ -6631,8 +6636,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
slides: update 311 course manifests and schedule map
</commit_message>
<xml_diff>
--- a/AIASD-311-CourseModules.xlsx
+++ b/AIASD-311-CourseModules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\AIASD\AI-Assisted-Software-Development-Course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D69D90E-DBDD-4524-8EB1-2FF0DE49DD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE79AE39-0B25-4CE5-8EA8-3468A9B72A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4583" yWindow="16103" windowWidth="21795" windowHeight="13875" activeTab="3" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="2" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
   </bookViews>
   <sheets>
     <sheet name="decks" sheetId="10" r:id="rId1"/>
@@ -1434,133 +1434,6 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2477,9 +2350,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
@@ -2611,6 +2481,136 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2663,7 +2663,7 @@
     <tableColumn id="2" xr3:uid="{B07EACE5-F752-4991-BE23-9BE11BB23286}" name="Column1">
       <calculatedColumnFormula>LOWER(Table11[[#This Row],[Name]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B8942215-B69E-4093-A1A0-3CA4C76B06EE}" name="Column2" dataDxfId="123"/>
+    <tableColumn id="3" xr3:uid="{B8942215-B69E-4093-A1A0-3CA4C76B06EE}" name="Column2" dataDxfId="103"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2674,7 +2674,7 @@
   <autoFilter ref="C4:E11" xr:uid="{EF1BA374-5AD9-4719-9FF3-682D1B38151C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7AD14052-080E-4E37-8C5E-B2CB6B097298}" name="Section"/>
-    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{3E1642EC-6329-4B91-8040-267B6F5F8CED}" name="Hours" totalsRowFunction="custom">
       <totalsRowFormula>SUM(Table9[Hours])</totalsRowFormula>
     </tableColumn>
@@ -2688,33 +2688,33 @@
   <autoFilter ref="C2:P30" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9D61239E-9B4A-4932-AB0D-EB9D9921B03D}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="122" totalsRowDxfId="121"/>
+    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="102" totalsRowDxfId="101"/>
     <tableColumn id="5" xr3:uid="{8B6AF1D4-2216-4B85-BA7D-212BA502015B}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description" dataDxfId="120"/>
+    <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description" dataDxfId="100"/>
     <tableColumn id="19" xr3:uid="{6CD3E0DC-278C-498A-A888-BE6341994574}" name="Deck"/>
     <tableColumn id="18" xr3:uid="{7E153D0B-3D6F-4A51-B6D2-9A0BE0E451DA}" name="Slide(s)"/>
-    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="119" totalsRowDxfId="118">
+    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="99" totalsRowDxfId="98">
       <calculatedColumnFormula>I2 + (E2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="117" totalsRowDxfId="116">
+    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="96">
       <totalsRowFormula>COUNTIF(monday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="115" totalsRowDxfId="114">
+    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="94">
       <totalsRowFormula>COUNTIF(monday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="113" totalsRowDxfId="112">
+    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="93" totalsRowDxfId="92">
       <totalsRowFormula>COUNTIF(monday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="111" totalsRowDxfId="110">
+    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="91" totalsRowDxfId="90">
       <totalsRowFormula>COUNTIF(monday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="109" totalsRowDxfId="108">
+    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="89" totalsRowDxfId="88">
       <totalsRowFormula>COUNTIF(monday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="107" totalsRowDxfId="106">
+    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="86">
       <totalsRowFormula>COUNTIF(monday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="105" totalsRowDxfId="104">
+    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="84">
       <totalsRowFormula>COUNTIF(monday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2727,33 +2727,33 @@
   <autoFilter ref="B2:O24" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{A79E8443-E3FC-4A2C-83B2-0E581E8FF9B8}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="27" totalsRowDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="83" totalsRowDxfId="8"/>
     <tableColumn id="5" xr3:uid="{C37F49DC-8E37-4F56-B136-B64A492DADC4}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="26"/>
+    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="82"/>
     <tableColumn id="14" xr3:uid="{BD249784-C12F-4B3B-8752-038CF2024DD9}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{E7140FF5-BE1A-4956-A3E4-A572C8619336}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="25" totalsRowDxfId="16">
+    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="81" totalsRowDxfId="7">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="24" totalsRowDxfId="15">
+    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="80" totalsRowDxfId="6">
       <totalsRowFormula>COUNTIF(tuesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="23" totalsRowDxfId="14">
+    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="79" totalsRowDxfId="5">
       <totalsRowFormula>COUNTIF(tuesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="22" totalsRowDxfId="13">
+    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="78" totalsRowDxfId="4">
       <totalsRowFormula>COUNTIF(tuesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="21" totalsRowDxfId="12">
+    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="77" totalsRowDxfId="3">
       <totalsRowFormula>COUNTIF(tuesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="20" totalsRowDxfId="11">
+    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="76" totalsRowDxfId="2">
       <totalsRowFormula>COUNTIF(tuesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="19" totalsRowDxfId="10">
+    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="75" totalsRowDxfId="1">
       <totalsRowFormula>COUNTIF(tuesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="18" totalsRowDxfId="9">
+    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="74" totalsRowDxfId="0">
       <totalsRowFormula>COUNTIF(tuesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2766,33 +2766,33 @@
   <autoFilter ref="B2:O12" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9E7625E1-2B56-4752-B6F8-BF1B9CB4F92C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="103" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="123" totalsRowDxfId="122"/>
     <tableColumn id="5" xr3:uid="{78218F89-BD58-4DD6-9B0D-DCE1B0CA5E74}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="102"/>
-    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="101"/>
+    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="121"/>
+    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="120"/>
     <tableColumn id="2" xr3:uid="{06859EAF-BB57-49A2-83C0-AA6CD01CE733}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="100" totalsRowDxfId="7">
+    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="119" totalsRowDxfId="118">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="99" totalsRowDxfId="6">
+    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="117" totalsRowDxfId="116">
       <totalsRowFormula>COUNTIF(wednesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="98" totalsRowDxfId="5">
+    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="115" totalsRowDxfId="114">
       <totalsRowFormula>COUNTIF(wednesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="4">
+    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="113" totalsRowDxfId="112">
       <totalsRowFormula>COUNTIF(wednesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="96" totalsRowDxfId="3">
+    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="111" totalsRowDxfId="110">
       <totalsRowFormula>COUNTIF(wednesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="2">
+    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="109" totalsRowDxfId="108">
       <totalsRowFormula>COUNTIF(wednesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="94" totalsRowDxfId="1">
+    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="107" totalsRowDxfId="106">
       <totalsRowFormula>COUNTIF(wednesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="93" totalsRowDxfId="0">
+    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="105" totalsRowDxfId="104">
       <totalsRowFormula>COUNTIF(wednesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2805,33 +2805,33 @@
   <autoFilter ref="B2:O15" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{D80C761D-4E7E-4D1A-862A-6769A723C40C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="92" totalsRowDxfId="91"/>
+    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="73" totalsRowDxfId="72"/>
     <tableColumn id="5" xr3:uid="{F640E5CE-B0CE-4586-AB64-2F877DC1D9FB}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="90"/>
-    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="89"/>
+    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="71"/>
+    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="70"/>
     <tableColumn id="2" xr3:uid="{76D09C9B-F732-4E1C-945B-A497FD16EFDB}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="88" totalsRowDxfId="87">
+    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="69" totalsRowDxfId="68">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="86" totalsRowDxfId="85">
+    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
       <totalsRowFormula>COUNTIF(thursday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="84" totalsRowDxfId="83">
+    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="64">
       <totalsRowFormula>COUNTIF(thursday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="82" totalsRowDxfId="81">
+    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="63" totalsRowDxfId="62">
       <totalsRowFormula>COUNTIF(thursday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="80" totalsRowDxfId="79">
+    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="61" totalsRowDxfId="60">
       <totalsRowFormula>COUNTIF(thursday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="78" totalsRowDxfId="77">
+    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="58">
       <totalsRowFormula>COUNTIF(thursday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="76" totalsRowDxfId="75">
+    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="56">
       <totalsRowFormula>COUNTIF(thursday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="74" totalsRowDxfId="73">
+    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54">
       <totalsRowFormula>COUNTIF(thursday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2844,33 +2844,33 @@
   <autoFilter ref="B2:O25" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{26906033-DBB1-4850-8A65-B0AABB8EB5B7}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="72" totalsRowDxfId="71"/>
+    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="53" totalsRowDxfId="52"/>
     <tableColumn id="5" xr3:uid="{B474477F-00C6-4EE7-A8CC-63E5347553DE}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="51"/>
     <tableColumn id="14" xr3:uid="{DF3B0E26-BDAD-42AF-AA94-ECF071ABBC93}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{FDADF079-31AD-4240-B382-130BDA5B792F}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="69" totalsRowDxfId="68">
+    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="50" totalsRowDxfId="49">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
+    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="47">
       <totalsRowFormula>COUNTIF(friday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="64">
+    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="45">
       <totalsRowFormula>COUNTIF(friday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="63" totalsRowDxfId="62">
+    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="44" totalsRowDxfId="43">
       <totalsRowFormula>COUNTIF(friday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="61" totalsRowDxfId="60">
+    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="42" totalsRowDxfId="41">
       <totalsRowFormula>COUNTIF(friday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="58">
+    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="40" totalsRowDxfId="39">
       <totalsRowFormula>COUNTIF(friday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="56">
+    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="38" totalsRowDxfId="37">
       <totalsRowFormula>COUNTIF(friday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54">
+    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="35">
       <totalsRowFormula>COUNTIF(friday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2879,35 +2879,35 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="53" dataDxfId="51" headerRowBorderDxfId="52" tableBorderDxfId="50" totalsRowBorderDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31" totalsRowBorderDxfId="30">
   <autoFilter ref="B3:I8" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}"/>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="48" totalsRowDxfId="47"/>
-    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="45">
+    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
       <calculatedColumnFormula>COUNTIF(monday[Copilot],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Copilot])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="44" totalsRowDxfId="43">
+    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="25" totalsRowDxfId="24">
       <calculatedColumnFormula>COUNTIF(monday[Claude],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Claude])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="42" totalsRowDxfId="41">
+    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="23" totalsRowDxfId="22">
       <calculatedColumnFormula>COUNTIF(monday[Visual Studio],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Visual Studio])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="40" totalsRowDxfId="39">
+    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="21" totalsRowDxfId="20">
       <calculatedColumnFormula>COUNTIF(monday[VS Code],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[VS Code])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="38" totalsRowDxfId="37">
+    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="19" totalsRowDxfId="18">
       <calculatedColumnFormula>COUNTIF(monday[GitHub],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[GitHub])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="35">
+    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="17" totalsRowDxfId="16">
       <calculatedColumnFormula>COUNTIF(monday[AzDO],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[AzDO])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="34" totalsRowDxfId="33">
+    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="15" totalsRowDxfId="14">
       <calculatedColumnFormula>COUNTIF(monday[Agnostic],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Agnostic])</totalsRowFormula>
     </tableColumn>
@@ -2917,12 +2917,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="13">
   <autoFilter ref="C16:E23" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3257,14 +3257,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BDF954-FF19-4C47-AD82-6E7FB7023B19}">
   <dimension ref="C3:E60"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="64.53125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="44.796875" customWidth="1"/>
+    <col min="3" max="3" width="64.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>202</v>
       </c>
@@ -3275,7 +3275,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="4" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>306</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="5" spans="3:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="5" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>289</v>
       </c>
@@ -3299,7 +3299,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>280</v>
       </c>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>270</v>
       </c>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>269</v>
       </c>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
         <v>268</v>
       </c>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>267</v>
       </c>
@@ -3349,7 +3349,7 @@
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>266</v>
       </c>
@@ -3359,7 +3359,7 @@
       </c>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>265</v>
       </c>
@@ -3369,7 +3369,7 @@
       </c>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>264</v>
       </c>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
         <v>263</v>
       </c>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
         <v>243</v>
       </c>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="16" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C16" t="s">
         <v>237</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="17" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="3:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
         <v>324</v>
       </c>
@@ -3423,7 +3423,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C18" t="s">
         <v>322</v>
       </c>
@@ -3435,7 +3435,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="19" spans="3:5" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="19" spans="3:5" ht="145" x14ac:dyDescent="0.35">
       <c r="C19" t="s">
         <v>320</v>
       </c>
@@ -3447,7 +3447,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="20" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="20" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C20" t="s">
         <v>316</v>
       </c>
@@ -3459,7 +3459,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="21" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C21" t="s">
         <v>313</v>
       </c>
@@ -3471,7 +3471,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="22" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C22" t="s">
         <v>309</v>
       </c>
@@ -3483,7 +3483,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="23" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="3:5" ht="87" x14ac:dyDescent="0.35">
       <c r="C23" t="s">
         <v>304</v>
       </c>
@@ -3495,7 +3495,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="24" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="24" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C24" t="s">
         <v>301</v>
       </c>
@@ -3507,7 +3507,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="25" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="25" spans="3:5" ht="87" x14ac:dyDescent="0.35">
       <c r="C25" t="s">
         <v>302</v>
       </c>
@@ -3519,7 +3519,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="26" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="26" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C26" t="s">
         <v>294</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="27" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C27" t="s">
         <v>300</v>
       </c>
@@ -3543,7 +3543,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="28" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="28" spans="3:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="C28" t="s">
         <v>292</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="29" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="29" spans="3:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="C29" t="s">
         <v>287</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="30" spans="3:5" ht="114" x14ac:dyDescent="0.45">
+    <row r="30" spans="3:5" ht="130.5" x14ac:dyDescent="0.35">
       <c r="C30" t="s">
         <v>284</v>
       </c>
@@ -3579,7 +3579,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="31" spans="3:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="31" spans="3:5" ht="58" x14ac:dyDescent="0.35">
       <c r="C31" t="s">
         <v>282</v>
       </c>
@@ -3591,7 +3591,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="32" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C32" t="s">
         <v>279</v>
       </c>
@@ -3603,7 +3603,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="33" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C33" t="s">
         <v>277</v>
       </c>
@@ -3615,7 +3615,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="34" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="34" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="C34" t="s">
         <v>275</v>
       </c>
@@ -3627,7 +3627,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="35" spans="3:5" ht="57" x14ac:dyDescent="0.45">
+    <row r="35" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="C35" t="s">
         <v>273</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="36" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="36" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C36" t="s">
         <v>203</v>
       </c>
@@ -3649,7 +3649,7 @@
       </c>
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="3:5" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="37" spans="3:5" ht="130.5" x14ac:dyDescent="0.35">
       <c r="C37" t="s">
         <v>262</v>
       </c>
@@ -3661,7 +3661,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="38" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="38" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C38" t="s">
         <v>260</v>
       </c>
@@ -3673,7 +3673,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="39" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="39" spans="3:5" ht="87" x14ac:dyDescent="0.35">
       <c r="C39" t="s">
         <v>258</v>
       </c>
@@ -3685,7 +3685,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="40" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="40" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C40" t="s">
         <v>252</v>
       </c>
@@ -3697,7 +3697,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="41" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="41" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C41" t="s">
         <v>251</v>
       </c>
@@ -3709,7 +3709,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="42" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="42" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="C42" t="s">
         <v>248</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="43" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="43" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="C43" t="s">
         <v>245</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="44" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="44" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C44" t="s">
         <v>242</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="45" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="45" spans="3:5" ht="101.5" x14ac:dyDescent="0.35">
       <c r="C45" t="s">
         <v>240</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="46" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="46" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C46" t="s">
         <v>235</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="47" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="47" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C47" t="s">
         <v>205</v>
       </c>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="E47" s="2"/>
     </row>
-    <row r="48" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="48" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C48" t="s">
         <v>233</v>
       </c>
@@ -3791,7 +3791,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="49" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="49" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="C49" t="s">
         <v>231</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="50" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="50" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C50" t="s">
         <v>228</v>
       </c>
@@ -3813,7 +3813,7 @@
       </c>
       <c r="E50" s="2"/>
     </row>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="51" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C51" t="s">
         <v>206</v>
       </c>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="E51" s="2"/>
     </row>
-    <row r="52" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="52" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C52" t="s">
         <v>207</v>
       </c>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="E52" s="2"/>
     </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="53" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C53" t="s">
         <v>227</v>
       </c>
@@ -3843,7 +3843,7 @@
       </c>
       <c r="E53" s="2"/>
     </row>
-    <row r="54" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="54" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C54" t="s">
         <v>208</v>
       </c>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="E54" s="2"/>
     </row>
-    <row r="55" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="55" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C55" t="s">
         <v>209</v>
       </c>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="E55" s="2"/>
     </row>
-    <row r="56" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="56" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C56" t="s">
         <v>225</v>
       </c>
@@ -3873,7 +3873,7 @@
       </c>
       <c r="E56" s="2"/>
     </row>
-    <row r="57" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="57" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C57" t="s">
         <v>223</v>
       </c>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="E57" s="2"/>
     </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="58" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C58" t="s">
         <v>220</v>
       </c>
@@ -3893,7 +3893,7 @@
       </c>
       <c r="E58" s="2"/>
     </row>
-    <row r="59" spans="3:5" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="59" spans="3:5" ht="159.5" x14ac:dyDescent="0.35">
       <c r="C59" t="s">
         <v>210</v>
       </c>
@@ -3905,7 +3905,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="60" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="60" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
       <c r="C60" t="s">
         <v>327</v>
       </c>
@@ -3929,18 +3929,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B10EB54-2E02-4CB7-9831-8B22CDCFE359}">
   <dimension ref="C2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="40.06640625" customWidth="1"/>
-    <col min="4" max="4" width="11.06640625" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="9.796875" customWidth="1"/>
-    <col min="6" max="6" width="52.06640625" customWidth="1"/>
-    <col min="7" max="7" width="29.796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.08984375" customWidth="1"/>
+    <col min="4" max="4" width="11.08984375" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" customWidth="1"/>
+    <col min="6" max="6" width="52.08984375" customWidth="1"/>
+    <col min="7" max="7" width="29.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="2" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
         <v>1</v>
       </c>
@@ -3984,7 +3984,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="3:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>5</v>
       </c>
@@ -4029,7 +4029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="4" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>217</v>
       </c>
@@ -4071,7 +4071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="3:16" ht="57" x14ac:dyDescent="0.45">
+    <row r="5" spans="3:16" ht="58" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>30</v>
       </c>
@@ -4116,7 +4116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="6" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>33</v>
       </c>
@@ -4156,7 +4156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="3:16" ht="57" x14ac:dyDescent="0.45">
+    <row r="7" spans="3:16" ht="58" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>9</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="3:16" ht="57" x14ac:dyDescent="0.45">
+    <row r="8" spans="3:16" ht="58" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>192</v>
       </c>
@@ -4241,7 +4241,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="9" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
         <v>193</v>
       </c>
@@ -4283,7 +4283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="10" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>194</v>
       </c>
@@ -4325,7 +4325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="3:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>195</v>
       </c>
@@ -4367,7 +4367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="3:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>196</v>
       </c>
@@ -4409,7 +4409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="3:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>197</v>
       </c>
@@ -4451,7 +4451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="3:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
         <v>0</v>
       </c>
@@ -4494,7 +4494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="15" spans="3:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
         <v>14</v>
       </c>
@@ -4537,7 +4537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="16" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C16" t="s">
         <v>16</v>
       </c>
@@ -4578,7 +4578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="17" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
         <v>18</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="18" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C18" t="s">
         <v>20</v>
       </c>
@@ -4660,7 +4660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="19" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C19" t="s">
         <v>22</v>
       </c>
@@ -4701,7 +4701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="20" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C20" t="s">
         <v>29</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="21" spans="3:16" x14ac:dyDescent="0.35">
       <c r="C21" t="s">
         <v>26</v>
       </c>
@@ -4780,7 +4780,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="3:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C22" t="s">
         <v>24</v>
       </c>
@@ -4823,7 +4823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="3:16" ht="128.25" x14ac:dyDescent="0.45">
+    <row r="23" spans="3:16" ht="145" x14ac:dyDescent="0.35">
       <c r="C23" t="s">
         <v>329</v>
       </c>
@@ -4860,7 +4860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="24" spans="3:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C24" t="s">
         <v>255</v>
       </c>
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="3:16" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="3:16" ht="101.5" x14ac:dyDescent="0.35">
       <c r="C25" t="s">
         <v>257</v>
       </c>
@@ -4934,7 +4934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="3:16" ht="57" x14ac:dyDescent="0.45">
+    <row r="26" spans="3:16" ht="58" x14ac:dyDescent="0.35">
       <c r="C26" t="s">
         <v>38</v>
       </c>
@@ -4974,7 +4974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="27" spans="3:16" ht="29" x14ac:dyDescent="0.35">
       <c r="C27" t="s">
         <v>35</v>
       </c>
@@ -5014,7 +5014,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="3:16" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="28" spans="3:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C28" t="s">
         <v>37</v>
       </c>
@@ -5054,7 +5054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="3:16" ht="57" x14ac:dyDescent="0.45">
+    <row r="29" spans="3:16" ht="72.5" x14ac:dyDescent="0.35">
       <c r="C29" t="s">
         <v>68</v>
       </c>
@@ -5093,7 +5093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="3:16" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="30" spans="3:16" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C30" t="s">
         <v>56</v>
       </c>
@@ -5132,7 +5132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="3:16" x14ac:dyDescent="0.45">
+    <row r="31" spans="3:16" x14ac:dyDescent="0.35">
       <c r="G31"/>
       <c r="I31" s="1"/>
       <c r="J31" s="16">
@@ -5176,17 +5176,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6092BCC8-4678-4A74-B9FA-42E487B327B3}">
   <dimension ref="B2:O25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="40.06640625" customWidth="1"/>
-    <col min="3" max="3" width="11.06640625" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="9.796875" customWidth="1"/>
-    <col min="5" max="5" width="52.06640625" customWidth="1"/>
-    <col min="6" max="6" width="30.73046875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.08984375" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" customWidth="1"/>
+    <col min="5" max="5" width="52.08984375" customWidth="1"/>
+    <col min="6" max="6" width="30.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -5230,7 +5230,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>46</v>
       </c>
@@ -5270,7 +5270,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>54</v>
       </c>
@@ -5310,7 +5310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B5" s="3" t="s">
         <v>48</v>
       </c>
@@ -5350,7 +5350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B6" s="3" t="s">
         <v>147</v>
       </c>
@@ -5393,7 +5393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>32</v>
       </c>
@@ -5436,7 +5436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>34</v>
       </c>
@@ -5478,7 +5478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B9" s="3" t="s">
         <v>31</v>
       </c>
@@ -5521,7 +5521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>47</v>
       </c>
@@ -5563,7 +5563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>149</v>
       </c>
@@ -5602,7 +5602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>354</v>
       </c>
@@ -5644,7 +5644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>36</v>
       </c>
@@ -5686,7 +5686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B14" s="3" t="s">
         <v>29</v>
       </c>
@@ -5722,7 +5722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>49</v>
       </c>
@@ -5761,7 +5761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>50</v>
       </c>
@@ -5803,7 +5803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>51</v>
       </c>
@@ -5842,7 +5842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>52</v>
       </c>
@@ -5881,7 +5881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>53</v>
       </c>
@@ -5920,7 +5920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>111</v>
       </c>
@@ -5959,7 +5959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>59</v>
       </c>
@@ -5998,7 +5998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:15" ht="156.75" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:15" ht="159.5" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>60</v>
       </c>
@@ -6040,7 +6040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>61</v>
       </c>
@@ -6082,7 +6082,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>62</v>
       </c>
@@ -6124,7 +6124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
       <c r="F25"/>
       <c r="H25" s="1"/>
       <c r="I25" s="16">
@@ -6168,17 +6168,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB629B16-57A4-4E69-AF5C-15C19AF94F46}">
   <dimension ref="B2:O13"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="40.06640625" customWidth="1"/>
-    <col min="3" max="3" width="11.06640625" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="9.796875" customWidth="1"/>
-    <col min="5" max="5" width="52.06640625" customWidth="1"/>
-    <col min="6" max="6" width="44.265625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.08984375" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" customWidth="1"/>
+    <col min="5" max="5" width="52.08984375" customWidth="1"/>
+    <col min="6" max="6" width="44.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -6222,7 +6222,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>46</v>
       </c>
@@ -6260,7 +6260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="199.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:15" ht="203" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>250</v>
       </c>
@@ -6296,7 +6296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:15" ht="171" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="174" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>70</v>
       </c>
@@ -6335,7 +6335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>272</v>
       </c>
@@ -6371,7 +6371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="3" t="s">
         <v>119</v>
       </c>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>150</v>
       </c>
@@ -6450,7 +6450,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>152</v>
       </c>
@@ -6487,7 +6487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>71</v>
       </c>
@@ -6524,7 +6524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:15" ht="87" x14ac:dyDescent="0.35">
       <c r="B11" s="3" t="s">
         <v>69</v>
       </c>
@@ -6564,7 +6564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:15" ht="87" x14ac:dyDescent="0.35">
       <c r="B12" s="11" t="s">
         <v>154</v>
       </c>
@@ -6602,7 +6602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
       <c r="F13"/>
       <c r="H13" s="1"/>
       <c r="I13" s="16">
@@ -6646,17 +6646,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0484BF16-0A49-4DE6-BE0D-A8B6D297E051}">
   <dimension ref="B2:O16"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="40.06640625" customWidth="1"/>
-    <col min="3" max="3" width="11.06640625" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="9.796875" customWidth="1"/>
-    <col min="5" max="5" width="52.06640625" customWidth="1"/>
-    <col min="6" max="6" width="25.46484375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.08984375" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" customWidth="1"/>
+    <col min="5" max="5" width="52.08984375" customWidth="1"/>
+    <col min="6" max="6" width="25.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -6700,7 +6700,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>46</v>
       </c>
@@ -6738,7 +6738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>80</v>
       </c>
@@ -6777,7 +6777,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>112</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>221</v>
       </c>
@@ -6853,7 +6853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:15" ht="87" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>58</v>
       </c>
@@ -6892,7 +6892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>64</v>
       </c>
@@ -6929,7 +6929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>65</v>
       </c>
@@ -6966,7 +6966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:15" ht="171" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:15" ht="174" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>55</v>
       </c>
@@ -7005,7 +7005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>29</v>
       </c>
@@ -7040,7 +7040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>57</v>
       </c>
@@ -7077,7 +7077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>63</v>
       </c>
@@ -7116,7 +7116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>66</v>
       </c>
@@ -7153,7 +7153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>67</v>
       </c>
@@ -7190,7 +7190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
       <c r="F16"/>
       <c r="H16" s="1"/>
       <c r="I16" s="16">
@@ -7233,17 +7233,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD15E000-1B92-41C3-BF19-4CD4B65C581F}">
   <dimension ref="B2:O26"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="40.06640625" customWidth="1"/>
-    <col min="3" max="3" width="11.06640625" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="9.796875" customWidth="1"/>
-    <col min="5" max="5" width="52.06640625" customWidth="1"/>
-    <col min="6" max="6" width="33.06640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.08984375" customWidth="1"/>
+    <col min="3" max="3" width="11.08984375" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" customWidth="1"/>
+    <col min="5" max="5" width="52.08984375" customWidth="1"/>
+    <col min="6" max="6" width="33.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -7287,7 +7287,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>46</v>
       </c>
@@ -7325,7 +7325,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>81</v>
       </c>
@@ -7362,7 +7362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>72</v>
       </c>
@@ -7402,7 +7402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:15" ht="87" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>74</v>
       </c>
@@ -7439,7 +7439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>75</v>
       </c>
@@ -7478,7 +7478,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>230</v>
       </c>
@@ -7514,7 +7514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>73</v>
       </c>
@@ -7553,7 +7553,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:15" ht="87" x14ac:dyDescent="0.35">
       <c r="B10" t="s">
         <v>291</v>
       </c>
@@ -7589,7 +7589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>76</v>
       </c>
@@ -7626,7 +7626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>77</v>
       </c>
@@ -7665,7 +7665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:15" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>78</v>
       </c>
@@ -7701,7 +7701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>82</v>
       </c>
@@ -7738,7 +7738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B15" t="s">
         <v>85</v>
       </c>
@@ -7775,7 +7775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B16" t="s">
         <v>86</v>
       </c>
@@ -7812,7 +7812,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B17" t="s">
         <v>29</v>
       </c>
@@ -7847,7 +7847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
       <c r="B18" t="s">
         <v>79</v>
       </c>
@@ -7886,7 +7886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:15" ht="87" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>83</v>
       </c>
@@ -7925,7 +7925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>84</v>
       </c>
@@ -7962,7 +7962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>87</v>
       </c>
@@ -7999,7 +7999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>88</v>
       </c>
@@ -8036,7 +8036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:15" ht="29" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>89</v>
       </c>
@@ -8073,7 +8073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:15" ht="58" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>90</v>
       </c>
@@ -8110,7 +8110,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:15" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:15" ht="101.5" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>91</v>
       </c>
@@ -8147,7 +8147,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
       <c r="F26"/>
       <c r="H26" s="1"/>
       <c r="I26" s="16">
@@ -8190,18 +8190,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDF57F64-64AA-48D6-B233-5D19F1E2205C}">
   <dimension ref="B2:I33"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.19921875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.08984375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.796875" customWidth="1"/>
-    <col min="8" max="8" width="7.53125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.81640625" customWidth="1"/>
+    <col min="8" max="8" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C2" s="25" t="s">
         <v>169</v>
       </c>
@@ -8215,7 +8215,7 @@
       </c>
       <c r="H2" s="25"/>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B3" s="17" t="s">
         <v>156</v>
       </c>
@@ -8241,7 +8241,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="4" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="18" t="s">
         <v>155</v>
       </c>
@@ -8274,7 +8274,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:9" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="19" t="s">
         <v>157</v>
       </c>
@@ -8307,7 +8307,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:9" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B6" s="19" t="s">
         <v>158</v>
       </c>
@@ -8340,7 +8340,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:9" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="19" t="s">
         <v>159</v>
       </c>
@@ -8373,7 +8373,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:9" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B8" s="19" t="s">
         <v>160</v>
       </c>
@@ -8406,7 +8406,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:9" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B9" s="19"/>
       <c r="C9" s="21">
         <f>SUM(Totals[Copilot])</f>
@@ -8437,27 +8437,27 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B11" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B12" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B13" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
       <c r="B14" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
       <c r="C16" s="22" t="s">
         <v>166</v>
       </c>
@@ -8468,7 +8468,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C17" s="22" t="s">
         <v>39</v>
       </c>
@@ -8479,7 +8479,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C18" s="22" t="s">
         <v>39</v>
       </c>
@@ -8490,7 +8490,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C19" s="22" t="s">
         <v>39</v>
       </c>
@@ -8501,7 +8501,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C20" s="22" t="s">
         <v>165</v>
       </c>
@@ -8512,7 +8512,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C21" s="22" t="s">
         <v>165</v>
       </c>
@@ -8523,7 +8523,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C22" s="22" t="s">
         <v>165</v>
       </c>
@@ -8534,7 +8534,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C23" s="22" t="s">
         <v>165</v>
       </c>
@@ -8545,12 +8545,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G28" t="s">
         <v>176</v>
       </c>
@@ -8558,7 +8558,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G29" t="s">
         <v>171</v>
       </c>
@@ -8566,7 +8566,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G30" t="s">
         <v>172</v>
       </c>
@@ -8574,7 +8574,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G31" t="s">
         <v>173</v>
       </c>
@@ -8582,7 +8582,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.35">
       <c r="G32" t="s">
         <v>174</v>
       </c>
@@ -8590,7 +8590,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="7:8" x14ac:dyDescent="0.45">
+    <row r="33" spans="7:8" x14ac:dyDescent="0.35">
       <c r="G33" t="s">
         <v>175</v>
       </c>
@@ -8616,19 +8616,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1E0D4B9-8091-457D-8F80-D7E20EC6E158}">
   <dimension ref="C2:E12"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="35.46484375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.46484375" customWidth="1"/>
-    <col min="5" max="5" width="10.265625" customWidth="1"/>
+    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C2" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="4" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="3:5" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>178</v>
       </c>
@@ -8639,7 +8639,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="5" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C5" t="str">
         <f>monday!C7</f>
         <v>GitHub Copilot UI Tour</v>
@@ -8651,7 +8651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="6" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="C6" t="e">
         <f>monday!#REF!</f>
         <v>#REF!</v>
@@ -8663,7 +8663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="7" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C7" t="str">
         <f>tuesday!B17</f>
         <v>Code Explanation and Analysis</v>
@@ -8675,7 +8675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="8" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C8" t="str">
         <f>wednesday!B11</f>
         <v>MCP (Model Context Protocol) Servers</v>
@@ -8687,7 +8687,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="9" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C9" t="str">
         <f>wednesday!B12</f>
         <v>Exercise: MCP Servers</v>
@@ -8699,7 +8699,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="10" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>171</v>
       </c>
@@ -8710,7 +8710,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="11" spans="3:5" ht="29" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>172</v>
       </c>
@@ -8721,7 +8721,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="3:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="3:5" x14ac:dyDescent="0.35">
       <c r="E12">
         <f>SUM(Table9[Hours])</f>
         <v>24</v>

</xml_diff>

<commit_message>
slides: add friday requirements and technology artifacts
</commit_message>
<xml_diff>
--- a/AIASD-311-CourseModules.xlsx
+++ b/AIASD-311-CourseModules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\AIASD\AI-Assisted-Software-Development-Course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE79AE39-0B25-4CE5-8EA8-3468A9B72A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB3CD87F-F8A9-422B-9D0A-B08B535B13DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="2" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="5" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
   </bookViews>
   <sheets>
     <sheet name="decks" sheetId="10" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="375">
   <si>
     <t>CI/CD Pipeline Creation</t>
   </si>
@@ -678,21 +678,9 @@
     <t>Adding AI Guardrails.pptx</t>
   </si>
   <si>
-    <t>Addressing Technical Debt.pptx</t>
-  </si>
-  <si>
-    <t>AI Practitioner Resources.pptx</t>
-  </si>
-  <si>
-    <t>cqrs-architecture.pptx</t>
-  </si>
-  <si>
     <t>Custom Agents.pptx</t>
   </si>
   <si>
-    <t>Getting Started Checklist.pptx</t>
-  </si>
-  <si>
     <t>whats-the-big-deal.pptx</t>
   </si>
   <si>
@@ -978,9 +966,6 @@
     <t>Identifying Technical Debt; Automating the Creation of GitHub Issues; Exercise: Building the Backlog</t>
   </si>
   <si>
-    <t>Conformance &amp; Gap Analysis.pptx; Building a Backlog.pptx</t>
-  </si>
-  <si>
     <t>What AI Can Identify: Outdated coding patterns; High complexity areas; Duplicate logic; Missing tests; Security vulnerabilities; Architectural drift; Exercise: Comprehensive backlog creation in ~1 hour; Prioritization: Impact vs. effort evaluation; Issue Creation: GitHub issues vs. Azure DevOps work items; Comparing Implementations Against Instruction Files; Automated Issue Generation From Conformance Gaps; Prioritizing Technical Debt Remediation; Creating Actionable Remediation Plans; Exercise: Generate Issues to Make the Codebase Evergreen; Exercise: Create an Implementation Plan; Identifying Technical Debt; Automating the Creation of GitHub Issues; Exercise: Building the Backlog</t>
   </si>
   <si>
@@ -1135,6 +1120,54 @@
   </si>
   <si>
     <t>skills.md</t>
+  </si>
+  <si>
+    <t>ai-practitioner-resources.md</t>
+  </si>
+  <si>
+    <t>what-is-brownfield-software.md</t>
+  </si>
+  <si>
+    <t>ai-implementation-workflow.md</t>
+  </si>
+  <si>
+    <t>effective-prompts-for-technical-debt.md</t>
+  </si>
+  <si>
+    <t>conformance-and-gap-analysis.md; building-a-backlog.md</t>
+  </si>
+  <si>
+    <t>issue-prioritization-management.md</t>
+  </si>
+  <si>
+    <t>multi‑model-implementation-comparison.md</t>
+  </si>
+  <si>
+    <t>addressing-technical-debt.md</t>
+  </si>
+  <si>
+    <t>exercise-addressing-technical-debt.md</t>
+  </si>
+  <si>
+    <t>ai-first-development.md</t>
+  </si>
+  <si>
+    <t>greenfield-development-workflow.md</t>
+  </si>
+  <si>
+    <t>getting-started.md</t>
+  </si>
+  <si>
+    <t>starting-with-requirements.md</t>
+  </si>
+  <si>
+    <t>exercise-business-requirements-generation.md</t>
+  </si>
+  <si>
+    <t>cqrs-architecture.md</t>
+  </si>
+  <si>
+    <t>technology-stack-instruction-files.md</t>
   </si>
 </sst>
 </file>
@@ -1434,6 +1467,68 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2031,7 +2126,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2047,7 +2142,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2063,7 +2158,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2079,7 +2174,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2088,6 +2183,15 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2095,7 +2199,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2111,7 +2215,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2127,7 +2231,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2146,13 +2250,10 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
@@ -2288,7 +2389,7 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2304,7 +2405,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2320,7 +2421,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2336,7 +2437,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2345,15 +2446,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2361,7 +2453,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2369,7 +2461,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2377,7 +2469,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2385,7 +2477,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2393,7 +2485,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2401,7 +2493,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2410,6 +2502,24 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2417,7 +2527,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2425,7 +2535,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2433,7 +2543,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2441,7 +2551,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2449,7 +2559,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2457,7 +2567,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2466,24 +2576,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2491,7 +2583,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2499,7 +2591,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2507,7 +2599,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2515,7 +2607,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2523,7 +2615,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2531,7 +2623,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2540,68 +2632,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2663,7 +2696,7 @@
     <tableColumn id="2" xr3:uid="{B07EACE5-F752-4991-BE23-9BE11BB23286}" name="Column1">
       <calculatedColumnFormula>LOWER(Table11[[#This Row],[Name]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B8942215-B69E-4093-A1A0-3CA4C76B06EE}" name="Column2" dataDxfId="103"/>
+    <tableColumn id="3" xr3:uid="{B8942215-B69E-4093-A1A0-3CA4C76B06EE}" name="Column2" dataDxfId="104"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2674,7 +2707,7 @@
   <autoFilter ref="C4:E11" xr:uid="{EF1BA374-5AD9-4719-9FF3-682D1B38151C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7AD14052-080E-4E37-8C5E-B2CB6B097298}" name="Section"/>
-    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="18"/>
     <tableColumn id="2" xr3:uid="{3E1642EC-6329-4B91-8040-267B6F5F8CED}" name="Hours" totalsRowFunction="custom">
       <totalsRowFormula>SUM(Table9[Hours])</totalsRowFormula>
     </tableColumn>
@@ -2688,33 +2721,33 @@
   <autoFilter ref="C2:P30" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9D61239E-9B4A-4932-AB0D-EB9D9921B03D}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="102" totalsRowDxfId="101"/>
+    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="103" totalsRowDxfId="102"/>
     <tableColumn id="5" xr3:uid="{8B6AF1D4-2216-4B85-BA7D-212BA502015B}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description" dataDxfId="100"/>
+    <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description" dataDxfId="101"/>
     <tableColumn id="19" xr3:uid="{6CD3E0DC-278C-498A-A888-BE6341994574}" name="Deck"/>
     <tableColumn id="18" xr3:uid="{7E153D0B-3D6F-4A51-B6D2-9A0BE0E451DA}" name="Slide(s)"/>
-    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="99" totalsRowDxfId="98">
+    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="100" totalsRowDxfId="99">
       <calculatedColumnFormula>I2 + (E2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="97" totalsRowDxfId="96">
+    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="98" totalsRowDxfId="97">
       <totalsRowFormula>COUNTIF(monday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="95" totalsRowDxfId="94">
+    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="96" totalsRowDxfId="95">
       <totalsRowFormula>COUNTIF(monday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="93" totalsRowDxfId="92">
+    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="94" totalsRowDxfId="93">
       <totalsRowFormula>COUNTIF(monday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="91" totalsRowDxfId="90">
+    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="92" totalsRowDxfId="91">
       <totalsRowFormula>COUNTIF(monday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="89" totalsRowDxfId="88">
+    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="90" totalsRowDxfId="89">
       <totalsRowFormula>COUNTIF(monday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="87" totalsRowDxfId="86">
+    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="88" totalsRowDxfId="87">
       <totalsRowFormula>COUNTIF(monday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="85" totalsRowDxfId="84">
+    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="86" totalsRowDxfId="85">
       <totalsRowFormula>COUNTIF(monday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2727,33 +2760,33 @@
   <autoFilter ref="B2:O24" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{A79E8443-E3FC-4A2C-83B2-0E581E8FF9B8}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="83" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="123" totalsRowDxfId="122"/>
     <tableColumn id="5" xr3:uid="{C37F49DC-8E37-4F56-B136-B64A492DADC4}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="82"/>
+    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="121"/>
     <tableColumn id="14" xr3:uid="{BD249784-C12F-4B3B-8752-038CF2024DD9}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{E7140FF5-BE1A-4956-A3E4-A572C8619336}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="81" totalsRowDxfId="7">
+    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="120" totalsRowDxfId="119">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="80" totalsRowDxfId="6">
+    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="118" totalsRowDxfId="117">
       <totalsRowFormula>COUNTIF(tuesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="79" totalsRowDxfId="5">
+    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="116" totalsRowDxfId="115">
       <totalsRowFormula>COUNTIF(tuesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="78" totalsRowDxfId="4">
+    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="114" totalsRowDxfId="113">
       <totalsRowFormula>COUNTIF(tuesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="77" totalsRowDxfId="3">
+    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="112" totalsRowDxfId="111">
       <totalsRowFormula>COUNTIF(tuesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="76" totalsRowDxfId="2">
+    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="110" totalsRowDxfId="109">
       <totalsRowFormula>COUNTIF(tuesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="75" totalsRowDxfId="1">
+    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="108" totalsRowDxfId="107">
       <totalsRowFormula>COUNTIF(tuesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="74" totalsRowDxfId="0">
+    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="106" totalsRowDxfId="105">
       <totalsRowFormula>COUNTIF(tuesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2766,33 +2799,33 @@
   <autoFilter ref="B2:O12" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9E7625E1-2B56-4752-B6F8-BF1B9CB4F92C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="123" totalsRowDxfId="122"/>
+    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="84" totalsRowDxfId="83"/>
     <tableColumn id="5" xr3:uid="{78218F89-BD58-4DD6-9B0D-DCE1B0CA5E74}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="121"/>
-    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="120"/>
+    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="82"/>
+    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="81"/>
     <tableColumn id="2" xr3:uid="{06859EAF-BB57-49A2-83C0-AA6CD01CE733}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="119" totalsRowDxfId="118">
+    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="80" totalsRowDxfId="79">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="117" totalsRowDxfId="116">
+    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="78" totalsRowDxfId="77">
       <totalsRowFormula>COUNTIF(wednesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="115" totalsRowDxfId="114">
+    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="76" totalsRowDxfId="75">
       <totalsRowFormula>COUNTIF(wednesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="113" totalsRowDxfId="112">
+    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="74" totalsRowDxfId="73">
       <totalsRowFormula>COUNTIF(wednesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="111" totalsRowDxfId="110">
+    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="72" totalsRowDxfId="71">
       <totalsRowFormula>COUNTIF(wednesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="109" totalsRowDxfId="108">
+    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="70" totalsRowDxfId="69">
       <totalsRowFormula>COUNTIF(wednesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="107" totalsRowDxfId="106">
+    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="68" totalsRowDxfId="67">
       <totalsRowFormula>COUNTIF(wednesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="105" totalsRowDxfId="104">
+    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="66" totalsRowDxfId="65">
       <totalsRowFormula>COUNTIF(wednesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2805,33 +2838,33 @@
   <autoFilter ref="B2:O15" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{D80C761D-4E7E-4D1A-862A-6769A723C40C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="73" totalsRowDxfId="72"/>
+    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="64" totalsRowDxfId="17"/>
     <tableColumn id="5" xr3:uid="{F640E5CE-B0CE-4586-AB64-2F877DC1D9FB}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="71"/>
-    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="70"/>
+    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="63"/>
+    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="62"/>
     <tableColumn id="2" xr3:uid="{76D09C9B-F732-4E1C-945B-A497FD16EFDB}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="69" totalsRowDxfId="68">
+    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="61" totalsRowDxfId="16">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
+    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="60" totalsRowDxfId="15">
       <totalsRowFormula>COUNTIF(thursday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="65" totalsRowDxfId="64">
+    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="14">
       <totalsRowFormula>COUNTIF(thursday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="63" totalsRowDxfId="62">
+    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="58" totalsRowDxfId="13">
       <totalsRowFormula>COUNTIF(thursday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="61" totalsRowDxfId="60">
+    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="12">
       <totalsRowFormula>COUNTIF(thursday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="58">
+    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="56" totalsRowDxfId="11">
       <totalsRowFormula>COUNTIF(thursday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="56">
+    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="10">
       <totalsRowFormula>COUNTIF(thursday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54">
+    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="54" totalsRowDxfId="9">
       <totalsRowFormula>COUNTIF(thursday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2844,33 +2877,33 @@
   <autoFilter ref="B2:O25" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{26906033-DBB1-4850-8A65-B0AABB8EB5B7}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="53" totalsRowDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="53" totalsRowDxfId="8"/>
     <tableColumn id="5" xr3:uid="{B474477F-00C6-4EE7-A8CC-63E5347553DE}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="52"/>
     <tableColumn id="14" xr3:uid="{DF3B0E26-BDAD-42AF-AA94-ECF071ABBC93}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{FDADF079-31AD-4240-B382-130BDA5B792F}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="50" totalsRowDxfId="49">
+    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="51" totalsRowDxfId="7">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="47">
+    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="50" totalsRowDxfId="6">
       <totalsRowFormula>COUNTIF(friday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="45">
+    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="49" totalsRowDxfId="5">
       <totalsRowFormula>COUNTIF(friday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="44" totalsRowDxfId="43">
+    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="4">
       <totalsRowFormula>COUNTIF(friday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="42" totalsRowDxfId="41">
+    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="47" totalsRowDxfId="3">
       <totalsRowFormula>COUNTIF(friday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="40" totalsRowDxfId="39">
+    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="2">
       <totalsRowFormula>COUNTIF(friday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="38" totalsRowDxfId="37">
+    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="45" totalsRowDxfId="1">
       <totalsRowFormula>COUNTIF(friday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="35">
+    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="44" totalsRowDxfId="0">
       <totalsRowFormula>COUNTIF(friday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2879,35 +2912,35 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33" tableBorderDxfId="31" totalsRowBorderDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="43" dataDxfId="41" headerRowBorderDxfId="42" tableBorderDxfId="40" totalsRowBorderDxfId="39">
   <autoFilter ref="B3:I8" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}"/>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="29" totalsRowDxfId="28"/>
-    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
+    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="38" totalsRowDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="35">
       <calculatedColumnFormula>COUNTIF(monday[Copilot],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Copilot])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="25" totalsRowDxfId="24">
+    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="34" totalsRowDxfId="33">
       <calculatedColumnFormula>COUNTIF(monday[Claude],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Claude])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="23" totalsRowDxfId="22">
+    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="32" totalsRowDxfId="31">
       <calculatedColumnFormula>COUNTIF(monday[Visual Studio],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Visual Studio])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="21" totalsRowDxfId="20">
+    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="30" totalsRowDxfId="29">
       <calculatedColumnFormula>COUNTIF(monday[VS Code],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[VS Code])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="19" totalsRowDxfId="18">
+    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="28" totalsRowDxfId="27">
       <calculatedColumnFormula>COUNTIF(monday[GitHub],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[GitHub])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="17" totalsRowDxfId="16">
+    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="26" totalsRowDxfId="25">
       <calculatedColumnFormula>COUNTIF(monday[AzDO],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[AzDO])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="15" totalsRowDxfId="14">
+    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="24" totalsRowDxfId="23">
       <calculatedColumnFormula>COUNTIF(monday[Agnostic],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Agnostic])</totalsRowFormula>
     </tableColumn>
@@ -2917,12 +2950,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="22">
   <autoFilter ref="C16:E23" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3257,14 +3290,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BDF954-FF19-4C47-AD82-6E7FB7023B19}">
   <dimension ref="C3:E60"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="64.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="61.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="44.81640625" customWidth="1"/>
+    <col min="3" max="3" width="64.53125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="61.265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C3" t="s">
         <v>202</v>
       </c>
@@ -3275,33 +3308,33 @@
         <v>188</v>
       </c>
     </row>
-    <row r="4" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D4" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^chat-mode.pptx</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="5" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C5" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="D5" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^creating robust testing frameworks.pptx</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="6" spans="3:5" x14ac:dyDescent="0.35">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C6" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="D6" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3309,9 +3342,9 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C7" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="D7" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3319,9 +3352,9 @@
       </c>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C8" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="D8" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3329,9 +3362,9 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C9" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="D9" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3339,9 +3372,9 @@
       </c>
       <c r="E9" s="2"/>
     </row>
-    <row r="10" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="D10" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3349,9 +3382,9 @@
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D11" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3359,9 +3392,9 @@
       </c>
       <c r="E11" s="2"/>
     </row>
-    <row r="12" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C12" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="D12" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3369,9 +3402,9 @@
       </c>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C13" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="D13" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3379,9 +3412,9 @@
       </c>
       <c r="E13" s="2"/>
     </row>
-    <row r="14" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C14" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="D14" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3389,9 +3422,9 @@
       </c>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C15" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D15" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3399,247 +3432,247 @@
       </c>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C16" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="D16" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^overview of llms.pptx</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="17" spans="3:5" ht="101.5" x14ac:dyDescent="0.35">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="17" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C17" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="D17" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_advanced context techniques.pptx</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.35">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="18" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C18" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D18" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai practitioner resources.pptx</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="19" spans="3:5" ht="145" x14ac:dyDescent="0.35">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="19" spans="3:5" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C19" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="D19" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai-development-approaches-comparison.pptx</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="20" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="20" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C20" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="D20" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai-first-vs-prompt-first.pptx</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="21" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="21" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C21" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="D21" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_building a backlog.pptx</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="22" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="22" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C22" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="D22" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_building safety nets.pptx</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="23" spans="3:5" ht="87" x14ac:dyDescent="0.35">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="23" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C23" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D23" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_conformance &amp; gap analysis.pptx</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="24" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="24" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C24" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D24" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot instruction stack.pptx</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="25" spans="3:5" ht="87" x14ac:dyDescent="0.35">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="25" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C25" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="D25" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot-instruction-control.pptx</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="26" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="26" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C26" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="D26" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot-instruction-files-vs-prompt-files-vs-chatmodes.pptx</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="27" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="27" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C27" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D27" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_core instruction files.pptx</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="28" spans="3:5" ht="101.5" x14ac:dyDescent="0.35">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="28" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C28" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="D28" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_cqrs-architecture.pptx</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="29" spans="3:5" ht="101.5" x14ac:dyDescent="0.35">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="29" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C29" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="D29" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_custom agents.pptx</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="30" spans="3:5" ht="130.5" x14ac:dyDescent="0.35">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="30" spans="3:5" ht="114" x14ac:dyDescent="0.45">
       <c r="C30" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="D30" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_documentation generation &amp; code analysis.pptx</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="31" spans="3:5" ht="58" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="31" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C31" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="D31" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_essential safety measures.pptx</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="32" spans="3:5" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="32" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C32" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="D32" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_generating implementation prompts &amp; verification.pptx</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="33" spans="3:5" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="33" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C33" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="D33" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_getting started checklist.pptx</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="34" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="34" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C34" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D34" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_github copilot for teams.pptx</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="35" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="35" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C35" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="D35" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_github-copilot-chat-mode-personas.pptx</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="36" spans="3:5" x14ac:dyDescent="0.35">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="36" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C36" t="s">
         <v>203</v>
       </c>
@@ -3649,127 +3682,127 @@
       </c>
       <c r="E36" s="2"/>
     </row>
-    <row r="37" spans="3:5" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="3:5" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C37" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D37" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_implementing-vertical-slices.pptx</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="38" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="38" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C38" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D38" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instruction files.pptx</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="39" spans="3:5" ht="87" x14ac:dyDescent="0.35">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="39" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C39" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="D39" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instruction-file-applyto-patterns.pptx</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="40" spans="3:5" x14ac:dyDescent="0.35">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="40" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C40" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D40" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instructions vs prompts vs custom chat modes.pptx</v>
       </c>
       <c r="E40" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="41" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="41" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C41" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D41" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_managing github copilot effectively.pptx</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="42" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="42" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C42" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="D42" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_mcp servers.pptx</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="43" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="43" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C43" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="D43" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_mcp-servers-vscode-copilot.pptx</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="44" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="44" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C44" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="D44" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_model selection &amp; comparison.pptx</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="45" spans="3:5" ht="101.5" x14ac:dyDescent="0.35">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="45" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C45" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="D45" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_multi‑model implementation comparison.pptx</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="46" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="46" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C46" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="D46" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_prompt files.pptx</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="47" spans="3:5" x14ac:dyDescent="0.35">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="47" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C47" t="s">
         <v>205</v>
       </c>
@@ -3779,33 +3812,33 @@
       </c>
       <c r="E47" s="2"/>
     </row>
-    <row r="48" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C48" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="D48" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_safe brownfield coding.pptx</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="49" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="49" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C49" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D49" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_starting with project requirements.pptx</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="50" spans="3:5" x14ac:dyDescent="0.35">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="50" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C50" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="D50" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3813,7 +3846,7 @@
       </c>
       <c r="E50" s="2"/>
     </row>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="51" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C51" t="s">
         <v>206</v>
       </c>
@@ -3823,7 +3856,7 @@
       </c>
       <c r="E51" s="2"/>
     </row>
-    <row r="52" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="52" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C52" t="s">
         <v>207</v>
       </c>
@@ -3833,9 +3866,9 @@
       </c>
       <c r="E52" s="2"/>
     </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="53" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C53" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="D53" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3843,7 +3876,7 @@
       </c>
       <c r="E53" s="2"/>
     </row>
-    <row r="54" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="54" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C54" t="s">
         <v>208</v>
       </c>
@@ -3853,7 +3886,7 @@
       </c>
       <c r="E54" s="2"/>
     </row>
-    <row r="55" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="55" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C55" t="s">
         <v>209</v>
       </c>
@@ -3863,9 +3896,9 @@
       </c>
       <c r="E55" s="2"/>
     </row>
-    <row r="56" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="56" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C56" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="D56" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3873,9 +3906,9 @@
       </c>
       <c r="E56" s="2"/>
     </row>
-    <row r="57" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="57" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C57" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D57" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3883,9 +3916,9 @@
       </c>
       <c r="E57" s="2"/>
     </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="58" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C58" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D58" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3893,7 +3926,7 @@
       </c>
       <c r="E58" s="2"/>
     </row>
-    <row r="59" spans="3:5" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="3:5" ht="156.75" x14ac:dyDescent="0.45">
       <c r="C59" t="s">
         <v>210</v>
       </c>
@@ -3902,19 +3935,19 @@
         <v>adding ai guardrails.pptx</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="60" spans="3:5" ht="72.5" x14ac:dyDescent="0.35">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="60" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C60" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="D60" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_addressing technical debt.pptx</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -3929,18 +3962,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B10EB54-2E02-4CB7-9831-8B22CDCFE359}">
   <dimension ref="C2:P31"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="40.08984375" customWidth="1"/>
-    <col min="4" max="4" width="11.08984375" style="1" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" customWidth="1"/>
-    <col min="6" max="6" width="52.08984375" customWidth="1"/>
-    <col min="7" max="7" width="29.81640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.06640625" customWidth="1"/>
+    <col min="4" max="4" width="11.06640625" style="1" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="9.796875" customWidth="1"/>
+    <col min="6" max="6" width="52.06640625" customWidth="1"/>
+    <col min="7" max="7" width="29.796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C2" t="s">
         <v>1</v>
       </c>
@@ -3984,7 +4017,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="3:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C3" t="s">
         <v>5</v>
       </c>
@@ -3998,7 +4031,7 @@
         <v>6</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="H3" s="23" t="s">
         <v>190</v>
@@ -4029,21 +4062,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="E4">
         <v>5</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="G4" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="I4" s="1">
         <f>I3 + (E3/ 1440)</f>
@@ -4071,7 +4104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="3:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="3:16" ht="57" x14ac:dyDescent="0.45">
       <c r="C5" t="s">
         <v>30</v>
       </c>
@@ -4082,10 +4115,10 @@
         <v>10</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>191</v>
@@ -4116,7 +4149,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C6" t="s">
         <v>33</v>
       </c>
@@ -4156,7 +4189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="3:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="7" spans="3:16" ht="57" x14ac:dyDescent="0.45">
       <c r="C7" t="s">
         <v>9</v>
       </c>
@@ -4167,7 +4200,7 @@
         <v>15</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>198</v>
@@ -4199,7 +4232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="3:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="3:16" ht="57" x14ac:dyDescent="0.45">
       <c r="C8" t="s">
         <v>192</v>
       </c>
@@ -4241,7 +4274,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C9" t="s">
         <v>193</v>
       </c>
@@ -4283,7 +4316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
         <v>194</v>
       </c>
@@ -4325,7 +4358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="3:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
         <v>195</v>
       </c>
@@ -4367,7 +4400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="3:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C12" t="s">
         <v>196</v>
       </c>
@@ -4409,7 +4442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="3:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C13" t="s">
         <v>197</v>
       </c>
@@ -4420,7 +4453,7 @@
         <v>100</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="H13" s="2">
         <v>15</v>
@@ -4451,7 +4484,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="3:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C14" t="s">
         <v>0</v>
       </c>
@@ -4465,7 +4498,7 @@
         <v>13</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="1">
@@ -4494,7 +4527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="3:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C15" t="s">
         <v>14</v>
       </c>
@@ -4508,7 +4541,7 @@
         <v>15</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="1">
@@ -4537,7 +4570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C16" t="s">
         <v>16</v>
       </c>
@@ -4578,7 +4611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C17" t="s">
         <v>18</v>
       </c>
@@ -4619,7 +4652,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C18" t="s">
         <v>20</v>
       </c>
@@ -4660,7 +4693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C19" t="s">
         <v>22</v>
       </c>
@@ -4701,7 +4734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C20" t="s">
         <v>29</v>
       </c>
@@ -4737,7 +4770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C21" t="s">
         <v>26</v>
       </c>
@@ -4751,7 +4784,7 @@
         <v>27</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="1">
@@ -4780,7 +4813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="3:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C22" t="s">
         <v>24</v>
       </c>
@@ -4794,7 +4827,7 @@
         <v>25</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="1">
@@ -4823,12 +4856,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="3:16" ht="145" x14ac:dyDescent="0.35">
+    <row r="23" spans="3:16" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C23" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>210</v>
@@ -4860,15 +4893,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="3:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="24" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C24" t="s">
+        <v>251</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>259</v>
-      </c>
       <c r="G24" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="1">
@@ -4897,15 +4930,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="3:16" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="3:16" ht="99.75" x14ac:dyDescent="0.45">
       <c r="C25" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="1">
@@ -4934,7 +4967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="3:16" ht="58" x14ac:dyDescent="0.35">
+    <row r="26" spans="3:16" ht="57" x14ac:dyDescent="0.45">
       <c r="C26" t="s">
         <v>38</v>
       </c>
@@ -4945,7 +4978,7 @@
         <v>97</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="1">
@@ -4974,7 +5007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="3:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C27" t="s">
         <v>35</v>
       </c>
@@ -4985,7 +5018,7 @@
         <v>96</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="H27" s="2"/>
       <c r="I27" s="1">
@@ -5014,7 +5047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="3:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="3:16" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C28" t="s">
         <v>37</v>
       </c>
@@ -5025,7 +5058,7 @@
         <v>95</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="1">
@@ -5054,7 +5087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="3:16" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="3:16" ht="57" x14ac:dyDescent="0.45">
       <c r="C29" t="s">
         <v>68</v>
       </c>
@@ -5065,7 +5098,7 @@
         <v>126</v>
       </c>
       <c r="G29" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="I29" s="1">
         <f t="shared" si="0"/>
@@ -5093,7 +5126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="3:16" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="3:16" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C30" t="s">
         <v>56</v>
       </c>
@@ -5104,7 +5137,7 @@
         <v>92</v>
       </c>
       <c r="G30" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="I30" s="1">
         <f t="shared" si="0"/>
@@ -5132,7 +5165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="3:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="3:16" x14ac:dyDescent="0.45">
       <c r="G31"/>
       <c r="I31" s="1"/>
       <c r="J31" s="16">
@@ -5176,17 +5209,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6092BCC8-4678-4A74-B9FA-42E487B327B3}">
   <dimension ref="B2:O25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="40.08984375" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" customWidth="1"/>
-    <col min="5" max="5" width="52.08984375" customWidth="1"/>
-    <col min="6" max="6" width="30.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.06640625" customWidth="1"/>
+    <col min="3" max="3" width="11.06640625" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.796875" customWidth="1"/>
+    <col min="5" max="5" width="52.06640625" customWidth="1"/>
+    <col min="6" max="6" width="30.73046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -5230,7 +5263,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>46</v>
       </c>
@@ -5242,7 +5275,7 @@
       </c>
       <c r="E3" s="2"/>
       <c r="F3" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="H3" s="6" t="str">
         <f>H2</f>
@@ -5270,7 +5303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B4" s="3" t="s">
         <v>54</v>
       </c>
@@ -5282,7 +5315,7 @@
         <v>93</v>
       </c>
       <c r="F4" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="H4" s="1">
         <f t="shared" ref="H4:H24" si="0">H3 + (D3/ 1440)</f>
@@ -5310,7 +5343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B5" s="3" t="s">
         <v>48</v>
       </c>
@@ -5322,7 +5355,7 @@
         <v>94</v>
       </c>
       <c r="F5" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" si="0"/>
@@ -5350,7 +5383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B6" s="3" t="s">
         <v>147</v>
       </c>
@@ -5364,7 +5397,7 @@
         <v>7</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="1">
@@ -5393,7 +5426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B7" s="3" t="s">
         <v>32</v>
       </c>
@@ -5407,7 +5440,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="1">
@@ -5436,7 +5469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>34</v>
       </c>
@@ -5450,7 +5483,7 @@
         <v>99</v>
       </c>
       <c r="F8" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="H8" s="1">
         <f>H9 + (D9/ 1440)</f>
@@ -5478,7 +5511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B9" s="3" t="s">
         <v>31</v>
       </c>
@@ -5492,7 +5525,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="1">
@@ -5521,7 +5554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>47</v>
       </c>
@@ -5535,7 +5568,7 @@
         <v>98</v>
       </c>
       <c r="F10" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="H10" s="1">
         <f>H8 + (D8/ 1440)</f>
@@ -5563,7 +5596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>149</v>
       </c>
@@ -5574,7 +5607,7 @@
         <v>148</v>
       </c>
       <c r="F11" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="H11" s="1">
         <f>H10 + (D10/ 1440)</f>
@@ -5602,9 +5635,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="C12" s="1">
         <v>2.013888888888889E-2</v>
@@ -5616,7 +5649,7 @@
         <v>104</v>
       </c>
       <c r="F12" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="H12" s="1">
         <f>H11 + (D11/ 1440)</f>
@@ -5644,7 +5677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>36</v>
       </c>
@@ -5658,7 +5691,7 @@
         <v>105</v>
       </c>
       <c r="F13" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="H13" s="1">
         <f>H12 + (D12/ 1440)</f>
@@ -5686,7 +5719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B14" s="3" t="s">
         <v>29</v>
       </c>
@@ -5722,7 +5755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
         <v>49</v>
       </c>
@@ -5733,7 +5766,7 @@
         <v>106</v>
       </c>
       <c r="F15" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="H15" s="1">
         <f t="shared" si="0"/>
@@ -5761,7 +5794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
         <v>50</v>
       </c>
@@ -5775,7 +5808,7 @@
         <v>107</v>
       </c>
       <c r="F16" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="H16" s="1">
         <f t="shared" si="0"/>
@@ -5803,7 +5836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
         <v>51</v>
       </c>
@@ -5814,7 +5847,7 @@
         <v>108</v>
       </c>
       <c r="F17" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="H17" s="1">
         <f t="shared" si="0"/>
@@ -5842,7 +5875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
         <v>52</v>
       </c>
@@ -5853,7 +5886,7 @@
         <v>109</v>
       </c>
       <c r="F18" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="H18" s="1">
         <f t="shared" si="0"/>
@@ -5881,7 +5914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
         <v>53</v>
       </c>
@@ -5920,7 +5953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
         <v>111</v>
       </c>
@@ -5959,7 +5992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
         <v>59</v>
       </c>
@@ -5970,7 +6003,7 @@
         <v>115</v>
       </c>
       <c r="F21" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="H21" s="1">
         <f t="shared" si="0"/>
@@ -5998,7 +6031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:15" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:15" ht="156.75" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
         <v>60</v>
       </c>
@@ -6012,7 +6045,7 @@
         <v>116</v>
       </c>
       <c r="F22" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="H22" s="1" t="e">
         <f>#REF! + (#REF!/ 1440)</f>
@@ -6040,7 +6073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
         <v>61</v>
       </c>
@@ -6054,7 +6087,7 @@
         <v>117</v>
       </c>
       <c r="F23" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="H23" s="1" t="e">
         <f t="shared" si="0"/>
@@ -6082,7 +6115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
         <v>62</v>
       </c>
@@ -6096,7 +6129,7 @@
         <v>118</v>
       </c>
       <c r="F24" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="H24" s="1" t="e">
         <f t="shared" si="0"/>
@@ -6124,7 +6157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:15" x14ac:dyDescent="0.45">
       <c r="F25"/>
       <c r="H25" s="1"/>
       <c r="I25" s="16">
@@ -6168,17 +6201,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB629B16-57A4-4E69-AF5C-15C19AF94F46}">
   <dimension ref="B2:O13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="40.08984375" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" customWidth="1"/>
-    <col min="5" max="5" width="52.08984375" customWidth="1"/>
-    <col min="6" max="6" width="44.26953125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.06640625" customWidth="1"/>
+    <col min="3" max="3" width="11.06640625" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.796875" customWidth="1"/>
+    <col min="5" max="5" width="52.06640625" customWidth="1"/>
+    <col min="6" max="6" width="44.265625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="13.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -6222,7 +6255,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>46</v>
       </c>
@@ -6260,15 +6293,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="203" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:15" ht="199.5" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="H4" s="6">
         <f>H3 + (D3/ 1440)</f>
@@ -6296,7 +6329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:15" ht="174" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:15" ht="171" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>70</v>
       </c>
@@ -6304,10 +6337,10 @@
         <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="H5" s="1">
         <f>H3 + (D3/ 1440)</f>
@@ -6335,12 +6368,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>204</v>
@@ -6371,7 +6404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B7" s="3" t="s">
         <v>119</v>
       </c>
@@ -6383,7 +6416,7 @@
         <v>119</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="H7" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6411,7 +6444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>150</v>
       </c>
@@ -6422,7 +6455,7 @@
         <v>151</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="H8" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -6450,7 +6483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
         <v>152</v>
       </c>
@@ -6487,7 +6520,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>71</v>
       </c>
@@ -6524,7 +6557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="2:15" ht="87" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B11" s="3" t="s">
         <v>69</v>
       </c>
@@ -6536,7 +6569,7 @@
         <v>120</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="H11" s="1">
         <f>H10 + (D10/ 1440)</f>
@@ -6564,7 +6597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:15" ht="87" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B12" s="11" t="s">
         <v>154</v>
       </c>
@@ -6602,7 +6635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" x14ac:dyDescent="0.45">
       <c r="F13"/>
       <c r="H13" s="1"/>
       <c r="I13" s="16">
@@ -6646,17 +6679,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0484BF16-0A49-4DE6-BE0D-A8B6D297E051}">
   <dimension ref="B2:O16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="40.08984375" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" customWidth="1"/>
-    <col min="5" max="5" width="52.08984375" customWidth="1"/>
-    <col min="6" max="6" width="25.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.06640625" customWidth="1"/>
+    <col min="3" max="3" width="11.06640625" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.796875" customWidth="1"/>
+    <col min="5" max="5" width="52.06640625" customWidth="1"/>
+    <col min="6" max="6" width="25.46484375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -6700,7 +6733,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>46</v>
       </c>
@@ -6738,7 +6771,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
         <v>80</v>
       </c>
@@ -6749,7 +6782,7 @@
         <v>127</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>212</v>
+        <v>359</v>
       </c>
       <c r="H4" s="1">
         <f>H3 + (D3/ 1440)</f>
@@ -6777,7 +6810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>112</v>
       </c>
@@ -6814,18 +6847,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="D6">
         <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>221</v>
+        <v>360</v>
       </c>
       <c r="H6" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6853,7 +6886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="87" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>58</v>
       </c>
@@ -6861,10 +6894,10 @@
         <v>10</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="H7" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6892,7 +6925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>64</v>
       </c>
@@ -6902,7 +6935,9 @@
       <c r="E8" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F8" s="2"/>
+      <c r="F8" s="2" t="s">
+        <v>361</v>
+      </c>
       <c r="H8" s="1">
         <f t="shared" ref="H8:H15" si="0">H7 + (D7/ 1440)</f>
         <v>0.4548611111111111</v>
@@ -6929,7 +6964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
         <v>65</v>
       </c>
@@ -6939,7 +6974,9 @@
       <c r="E9" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F9" s="2"/>
+      <c r="F9" s="2" t="s">
+        <v>362</v>
+      </c>
       <c r="H9" s="1">
         <f t="shared" si="0"/>
         <v>0.46527777777777779</v>
@@ -6966,7 +7003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:15" ht="174" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" ht="171" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
         <v>55</v>
       </c>
@@ -6974,10 +7011,10 @@
         <v>45</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>311</v>
+        <v>363</v>
       </c>
       <c r="H10" s="1">
         <f t="shared" si="0"/>
@@ -7005,7 +7042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>29</v>
       </c>
@@ -7040,7 +7077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>57</v>
       </c>
@@ -7050,7 +7087,9 @@
       <c r="E12" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="F12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>364</v>
+      </c>
       <c r="H12" s="1">
         <f t="shared" si="0"/>
         <v>0.55208333333333337</v>
@@ -7077,7 +7116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>63</v>
       </c>
@@ -7085,10 +7124,10 @@
         <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>211</v>
+        <v>366</v>
       </c>
       <c r="H13" s="1">
         <f t="shared" si="0"/>
@@ -7116,7 +7155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
         <v>66</v>
       </c>
@@ -7126,7 +7165,9 @@
       <c r="E14" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="F14" s="2"/>
+      <c r="F14" s="2" t="s">
+        <v>367</v>
+      </c>
       <c r="H14" s="1">
         <f t="shared" si="0"/>
         <v>0.57638888888888884</v>
@@ -7153,7 +7194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
         <v>67</v>
       </c>
@@ -7163,7 +7204,9 @@
       <c r="E15" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="F15" s="2"/>
+      <c r="F15" s="2" t="s">
+        <v>365</v>
+      </c>
       <c r="H15" s="1">
         <f t="shared" si="0"/>
         <v>0.60763888888888884</v>
@@ -7190,7 +7233,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" x14ac:dyDescent="0.45">
       <c r="F16"/>
       <c r="H16" s="1"/>
       <c r="I16" s="16">
@@ -7224,8 +7267,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -7233,17 +7277,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD15E000-1B92-41C3-BF19-4CD4B65C581F}">
   <dimension ref="B2:O26"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="40.08984375" customWidth="1"/>
-    <col min="3" max="3" width="11.08984375" style="1" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" customWidth="1"/>
-    <col min="5" max="5" width="52.08984375" customWidth="1"/>
-    <col min="6" max="6" width="33.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="40.06640625" customWidth="1"/>
+    <col min="3" max="3" width="11.06640625" style="1" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="9.796875" customWidth="1"/>
+    <col min="5" max="5" width="52.06640625" customWidth="1"/>
+    <col min="6" max="6" width="33.06640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B2" t="s">
         <v>1</v>
       </c>
@@ -7287,7 +7331,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>46</v>
       </c>
@@ -7325,7 +7369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
         <v>81</v>
       </c>
@@ -7335,7 +7379,9 @@
       <c r="E4" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F4"/>
+      <c r="F4" t="s">
+        <v>368</v>
+      </c>
       <c r="H4" s="1">
         <f>H3 + (D3/ 1440)</f>
         <v>0.42708333333333337</v>
@@ -7362,7 +7408,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
         <v>72</v>
       </c>
@@ -7402,7 +7448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="87" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
         <v>74</v>
       </c>
@@ -7412,7 +7458,9 @@
       <c r="E6" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F6"/>
+      <c r="F6" t="s">
+        <v>369</v>
+      </c>
       <c r="H6" s="1">
         <f>H5 + (D5/ 1440)</f>
         <v>0.43402777777777779</v>
@@ -7439,7 +7487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>75</v>
       </c>
@@ -7450,7 +7498,7 @@
         <v>131</v>
       </c>
       <c r="F7" t="s">
-        <v>215</v>
+        <v>370</v>
       </c>
       <c r="H7" s="1">
         <f>H6 + (D6/ 1440)</f>
@@ -7478,15 +7526,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="F8" t="s">
-        <v>230</v>
+        <v>371</v>
       </c>
       <c r="H8" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -7514,7 +7562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
         <v>73</v>
       </c>
@@ -7525,7 +7573,7 @@
         <v>129</v>
       </c>
       <c r="F9" t="s">
-        <v>230</v>
+        <v>372</v>
       </c>
       <c r="H9" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -7553,15 +7601,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:15" ht="87" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="F10" t="s">
-        <v>213</v>
+        <v>373</v>
       </c>
       <c r="H10" s="1">
         <f>H9 + (D9/ 1440)</f>
@@ -7589,7 +7637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>76</v>
       </c>
@@ -7599,7 +7647,9 @@
       <c r="E11" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="F11"/>
+      <c r="F11" t="s">
+        <v>374</v>
+      </c>
       <c r="H11" s="1">
         <f>H9 + (D9/ 1440)</f>
         <v>0.4548611111111111</v>
@@ -7626,7 +7676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>77</v>
       </c>
@@ -7637,7 +7687,7 @@
         <v>133</v>
       </c>
       <c r="F12" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="H12" s="1">
         <f t="shared" ref="H12:H25" si="0">H11 + (D11/ 1440)</f>
@@ -7665,7 +7715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:15" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>78</v>
       </c>
@@ -7701,7 +7751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
         <v>82</v>
       </c>
@@ -7738,7 +7788,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
         <v>85</v>
       </c>
@@ -7775,7 +7825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
         <v>86</v>
       </c>
@@ -7812,7 +7862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
         <v>29</v>
       </c>
@@ -7847,7 +7897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="2:15" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
         <v>79</v>
       </c>
@@ -7858,7 +7908,7 @@
         <v>135</v>
       </c>
       <c r="F18" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="H18" s="1">
         <f t="shared" si="0"/>
@@ -7886,7 +7936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="2:15" ht="87" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
         <v>83</v>
       </c>
@@ -7897,7 +7947,7 @@
         <v>138</v>
       </c>
       <c r="F19" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="H19" s="1">
         <f t="shared" si="0"/>
@@ -7925,7 +7975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
         <v>84</v>
       </c>
@@ -7962,7 +8012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
         <v>87</v>
       </c>
@@ -7999,7 +8049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:15" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
         <v>88</v>
       </c>
@@ -8036,7 +8086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="2:15" ht="29" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
         <v>89</v>
       </c>
@@ -8073,7 +8123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:15" ht="58" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
         <v>90</v>
       </c>
@@ -8110,7 +8160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="2:15" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:15" ht="99.75" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
         <v>91</v>
       </c>
@@ -8147,7 +8197,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:15" x14ac:dyDescent="0.45">
       <c r="F26"/>
       <c r="H26" s="1"/>
       <c r="I26" s="16">
@@ -8181,8 +8231,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -8190,18 +8241,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDF57F64-64AA-48D6-B233-5D19F1E2205C}">
   <dimension ref="B2:I33"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.06640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.81640625" customWidth="1"/>
-    <col min="8" max="8" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.796875" customWidth="1"/>
+    <col min="8" max="8" width="7.53125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:9" x14ac:dyDescent="0.45">
       <c r="C2" s="25" t="s">
         <v>169</v>
       </c>
@@ -8215,7 +8266,7 @@
       </c>
       <c r="H2" s="25"/>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B3" s="17" t="s">
         <v>156</v>
       </c>
@@ -8241,7 +8292,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="18" t="s">
         <v>155</v>
       </c>
@@ -8274,7 +8325,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="2:9" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B5" s="19" t="s">
         <v>157</v>
       </c>
@@ -8307,7 +8358,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="2:9" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B6" s="19" t="s">
         <v>158</v>
       </c>
@@ -8340,7 +8391,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="2:9" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="19" t="s">
         <v>159</v>
       </c>
@@ -8373,7 +8424,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="19" t="s">
         <v>160</v>
       </c>
@@ -8406,7 +8457,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="2:9" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
       <c r="B9" s="19"/>
       <c r="C9" s="21">
         <f>SUM(Totals[Copilot])</f>
@@ -8437,27 +8488,27 @@
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.45">
       <c r="C16" s="22" t="s">
         <v>166</v>
       </c>
@@ -8468,7 +8519,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C17" s="22" t="s">
         <v>39</v>
       </c>
@@ -8479,7 +8530,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C18" s="22" t="s">
         <v>39</v>
       </c>
@@ -8490,7 +8541,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C19" s="22" t="s">
         <v>39</v>
       </c>
@@ -8501,7 +8552,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C20" s="22" t="s">
         <v>165</v>
       </c>
@@ -8512,7 +8563,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C21" s="22" t="s">
         <v>165</v>
       </c>
@@ -8523,7 +8574,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C22" s="22" t="s">
         <v>165</v>
       </c>
@@ -8534,7 +8585,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C23" s="22" t="s">
         <v>165</v>
       </c>
@@ -8545,12 +8596,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G28" t="s">
         <v>176</v>
       </c>
@@ -8558,7 +8609,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G29" t="s">
         <v>171</v>
       </c>
@@ -8566,7 +8617,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="30" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G30" t="s">
         <v>172</v>
       </c>
@@ -8574,7 +8625,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G31" t="s">
         <v>173</v>
       </c>
@@ -8582,7 +8633,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G32" t="s">
         <v>174</v>
       </c>
@@ -8590,7 +8641,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="7:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="7:8" x14ac:dyDescent="0.45">
       <c r="G33" t="s">
         <v>175</v>
       </c>
@@ -8616,19 +8667,19 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1E0D4B9-8091-457D-8F80-D7E20EC6E158}">
   <dimension ref="C2:E12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="35.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="3" max="3" width="35.46484375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.46484375" customWidth="1"/>
+    <col min="5" max="5" width="10.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C2" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="4" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
         <v>178</v>
       </c>
@@ -8639,7 +8690,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C5" t="str">
         <f>monday!C7</f>
         <v>GitHub Copilot UI Tour</v>
@@ -8651,7 +8702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C6" t="e">
         <f>monday!#REF!</f>
         <v>#REF!</v>
@@ -8663,7 +8714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="7" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C7" t="str">
         <f>tuesday!B17</f>
         <v>Code Explanation and Analysis</v>
@@ -8675,7 +8726,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="8" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C8" t="str">
         <f>wednesday!B11</f>
         <v>MCP (Model Context Protocol) Servers</v>
@@ -8687,7 +8738,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C9" t="str">
         <f>wednesday!B12</f>
         <v>Exercise: MCP Servers</v>
@@ -8699,7 +8750,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
         <v>171</v>
       </c>
@@ -8710,7 +8761,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="3:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
         <v>172</v>
       </c>
@@ -8721,7 +8772,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="3:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="3:5" x14ac:dyDescent="0.45">
       <c r="E12">
         <f>SUM(Table9[Hours])</f>
         <v>24</v>

</xml_diff>

<commit_message>
slides: integrate Copilot labs into Monday deck outputs
</commit_message>
<xml_diff>
--- a/AIASD-311-CourseModules.xlsx
+++ b/AIASD-311-CourseModules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\AIASD\AI-Assisted-Software-Development-Course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB3CD87F-F8A9-422B-9D0A-B08B535B13DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6310788A-54C4-43FA-BE82-F4FF2AC935DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" activeTab="5" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
+    <workbookView xWindow="4583" yWindow="16103" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
   </bookViews>
   <sheets>
     <sheet name="decks" sheetId="10" r:id="rId1"/>
@@ -23,6 +23,7 @@
     <sheet name="GE Mods" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="373">
   <si>
     <t>CI/CD Pipeline Creation</t>
   </si>
@@ -300,21 +301,9 @@
     <t>Pull Request and Code Review</t>
   </si>
   <si>
-    <t>Vertical Slice Review</t>
-  </si>
-  <si>
-    <t>Issue Identification &amp; Diagram Corrections</t>
-  </si>
-  <si>
-    <t>Slice 4 Showcase - Order of Operations</t>
-  </si>
-  <si>
     <t>GitHub Code Review with Copilot</t>
   </si>
   <si>
-    <t>Slice 3 Showcase - Clear Button</t>
-  </si>
-  <si>
     <t>GitHub CLI &amp; PR Management</t>
   </si>
   <si>
@@ -465,21 +454,9 @@
     <t>Creating PR with "slice-1" branch; Associating PRs with issues; Assigning human reviewers; Initiating GitHub Copilot code review; Addressing review comments</t>
   </si>
   <si>
-    <t>Review of dependency diagram; Parallel implementation capabilities; Critical path identification (VSO 2 → VSO 3); Task assignments</t>
-  </si>
-  <si>
-    <t>Slice numbering inconsistencies found; AI-assisted validation and correction; Iterative debugging of Mermaid diagrams</t>
-  </si>
-  <si>
-    <t>Attendee demonstrates implementation; Test scenarios: Basic operations, order of operations, edge cases</t>
-  </si>
-  <si>
     <t>PR Review: 8 comments identified; Findings: Unicode characters, state management, missing metadata, dead code, test gaps</t>
   </si>
   <si>
-    <t>Attendee demonstrates implementation; Merged VSO 4 work first; Clear button resets calculator</t>
-  </si>
-  <si>
     <t>Default merge strategy discussion (squash vs. merge commit); GitHub settings navigation; Requesting Copilot code reviews via web interface; GitHub CLI commands for comment resolution; Personal access token permissions</t>
   </si>
   <si>
@@ -657,9 +634,6 @@
     <t>_Hands-On with GitHub Copilot (VS Code).pptx</t>
   </si>
   <si>
-    <t>github-copilot-chat-mode-personas.pptx</t>
-  </si>
-  <si>
     <t>_Repository and Tool Setup.pptx</t>
   </si>
   <si>
@@ -678,9 +652,6 @@
     <t>Adding AI Guardrails.pptx</t>
   </si>
   <si>
-    <t>Custom Agents.pptx</t>
-  </si>
-  <si>
     <t>whats-the-big-deal.pptx</t>
   </si>
   <si>
@@ -705,15 +676,9 @@
     <t>_What Defines Brownfield Code.pptx</t>
   </si>
   <si>
-    <t>What Are Vertical Slices</t>
-  </si>
-  <si>
     <t>_What Are Vertical Slices.pptx</t>
   </si>
   <si>
-    <t>vscode-copilot-agents-overview</t>
-  </si>
-  <si>
     <t>_vscode-copilot-agents-overview.pptx</t>
   </si>
   <si>
@@ -774,9 +739,6 @@
     <t>What is MCP?; MCP Architecture Overview; Installing Your First MCP Server; Copilot + MCP Integration; Popular MCP Servers to Use; Finding MCP Servers; Configuring Servers Securely; Exercise: Using MCP Servers</t>
   </si>
   <si>
-    <t>mcp-servers-vscode-copilot; MCP Servers.pptx</t>
-  </si>
-  <si>
     <t>_MCP Servers.pptx</t>
   </si>
   <si>
@@ -792,9 +754,6 @@
     <t>_Instructions vs Prompts vs Custom Chat Modes.pptx</t>
   </si>
   <si>
-    <t>Generating Implementation Prompts &amp; Verification</t>
-  </si>
-  <si>
     <t>implementing-vertical-slices</t>
   </si>
   <si>
@@ -987,9 +946,6 @@
     <t>What Are They?; Purpose; Scope &amp; Control; How They Work Together; Key Takeaways; The Core Concept; The applyTo Field: Pattern Matching; Prompt Files: Reference, Don’t Control; Chat Modes: Persona, Not Pattern Control; The Control Hierarchy; Practical Control Strategies; Real-World Examples; Key Takeaways; Questions &amp; Discussion; Instruction Files vs Prompt Files vs Custom Chat Modes; AI Development Approaches Overview; What Are Custom Chat Modes?; Custom Chat Mode Examples; Custom Chat Modes: Use Cases; Comparison Matrix; Execution Timeline; Decision Framework; Layered Integration Approach; Real-World Integration Example; Getting Started Checklist; Summary: Three Complementary Approaches; The Integration Advantage; Resources &amp; References; Questions &amp; Discussion</t>
   </si>
   <si>
-    <t>Instructions vs Prompts vs Custom Chat Modes; copilot-instruction-files-vs-prompt-files-vs-chatmodes.pptx; copilot-instruction-control.pptx; AI-Development-Approaches-Comparison.pptx</t>
-  </si>
-  <si>
     <t>_AI-Development-Approaches-Comparison.pptx</t>
   </si>
   <si>
@@ -1119,15 +1075,9 @@
     <t>feature-flags-and-test-suites.md</t>
   </si>
   <si>
-    <t>skills.md</t>
-  </si>
-  <si>
     <t>ai-practitioner-resources.md</t>
   </si>
   <si>
-    <t>what-is-brownfield-software.md</t>
-  </si>
-  <si>
     <t>ai-implementation-workflow.md</t>
   </si>
   <si>
@@ -1146,9 +1096,6 @@
     <t>addressing-technical-debt.md</t>
   </si>
   <si>
-    <t>exercise-addressing-technical-debt.md</t>
-  </si>
-  <si>
     <t>ai-first-development.md</t>
   </si>
   <si>
@@ -1168,6 +1115,54 @@
   </si>
   <si>
     <t>technology-stack-instruction-files.md</t>
+  </si>
+  <si>
+    <t>vertical-slicing-architecture-introduction.md</t>
+  </si>
+  <si>
+    <t>vertical-slice-implementation-plans.md</t>
+  </si>
+  <si>
+    <t>dependency-analysis-planning.md</t>
+  </si>
+  <si>
+    <t>implementation-prompts-verification.md</t>
+  </si>
+  <si>
+    <t>github-code-review-with-copilot.md</t>
+  </si>
+  <si>
+    <t>pull-request-code-review.md</t>
+  </si>
+  <si>
+    <t>copilot-instruction-files-vs-prompt-files-vs-chatmodes.md; copilot-instruction-control.md; AI-Development-Approaches-Comparison.pptx</t>
+  </si>
+  <si>
+    <t>custom-agents.md</t>
+  </si>
+  <si>
+    <t>github-copilot-chat-mode-personas.md</t>
+  </si>
+  <si>
+    <t>github-copilot-skills-practical-introduction.md</t>
+  </si>
+  <si>
+    <t>custom-agent-best-practices.md</t>
+  </si>
+  <si>
+    <t>mcp-model-context-protocol-servers.md</t>
+  </si>
+  <si>
+    <t>exercise-create-and-use-custom-skill.md</t>
+  </si>
+  <si>
+    <t>exercise-create-and-use-custom-agent.md</t>
+  </si>
+  <si>
+    <t>understanding-legacy-code.md</t>
+  </si>
+  <si>
+    <t>exercise-addressing-technical-debt-with-copilot.md</t>
   </si>
 </sst>
 </file>
@@ -1177,7 +1172,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1199,8 +1194,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1211,6 +1213,11 @@
       <patternFill patternType="solid">
         <fgColor theme="4"/>
         <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1309,10 +1316,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1396,138 +1404,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="124">
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -2126,7 +2012,7 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2142,7 +2028,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2158,7 +2044,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2174,7 +2060,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2183,15 +2069,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2199,7 +2076,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2215,7 +2092,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2231,7 +2108,7 @@
       </extLst>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
           <xfpb:DXFComplement i="0"/>
@@ -2250,10 +2127,16 @@
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
@@ -2378,6 +2261,133 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2707,7 +2717,7 @@
   <autoFilter ref="C4:E11" xr:uid="{EF1BA374-5AD9-4719-9FF3-682D1B38151C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7AD14052-080E-4E37-8C5E-B2CB6B097298}" name="Section"/>
-    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="0"/>
     <tableColumn id="2" xr3:uid="{3E1642EC-6329-4B91-8040-267B6F5F8CED}" name="Hours" totalsRowFunction="custom">
       <totalsRowFormula>SUM(Table9[Hours])</totalsRowFormula>
     </tableColumn>
@@ -2760,33 +2770,33 @@
   <autoFilter ref="B2:O24" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{A79E8443-E3FC-4A2C-83B2-0E581E8FF9B8}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="123" totalsRowDxfId="122"/>
+    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="84" totalsRowDxfId="83"/>
     <tableColumn id="5" xr3:uid="{C37F49DC-8E37-4F56-B136-B64A492DADC4}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="121"/>
+    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="82"/>
     <tableColumn id="14" xr3:uid="{BD249784-C12F-4B3B-8752-038CF2024DD9}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{E7140FF5-BE1A-4956-A3E4-A572C8619336}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="120" totalsRowDxfId="119">
+    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="81" totalsRowDxfId="80">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="118" totalsRowDxfId="117">
+    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="79" totalsRowDxfId="78">
       <totalsRowFormula>COUNTIF(tuesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="116" totalsRowDxfId="115">
+    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="77" totalsRowDxfId="76">
       <totalsRowFormula>COUNTIF(tuesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="114" totalsRowDxfId="113">
+    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="75" totalsRowDxfId="74">
       <totalsRowFormula>COUNTIF(tuesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="112" totalsRowDxfId="111">
+    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="73" totalsRowDxfId="72">
       <totalsRowFormula>COUNTIF(tuesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="110" totalsRowDxfId="109">
+    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="71" totalsRowDxfId="70">
       <totalsRowFormula>COUNTIF(tuesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="108" totalsRowDxfId="107">
+    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="69" totalsRowDxfId="68">
       <totalsRowFormula>COUNTIF(tuesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="106" totalsRowDxfId="105">
+    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
       <totalsRowFormula>COUNTIF(tuesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2799,33 +2809,33 @@
   <autoFilter ref="B2:O12" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9E7625E1-2B56-4752-B6F8-BF1B9CB4F92C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="84" totalsRowDxfId="83"/>
+    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="65" totalsRowDxfId="64"/>
     <tableColumn id="5" xr3:uid="{78218F89-BD58-4DD6-9B0D-DCE1B0CA5E74}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="82"/>
-    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="81"/>
+    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="63"/>
+    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="62"/>
     <tableColumn id="2" xr3:uid="{06859EAF-BB57-49A2-83C0-AA6CD01CE733}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="80" totalsRowDxfId="79">
+    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="61" totalsRowDxfId="60">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="78" totalsRowDxfId="77">
+    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="58">
       <totalsRowFormula>COUNTIF(wednesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="76" totalsRowDxfId="75">
+    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="56">
       <totalsRowFormula>COUNTIF(wednesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="74" totalsRowDxfId="73">
+    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54">
       <totalsRowFormula>COUNTIF(wednesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="72" totalsRowDxfId="71">
+    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="53" totalsRowDxfId="52">
       <totalsRowFormula>COUNTIF(wednesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="70" totalsRowDxfId="69">
+    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="51" totalsRowDxfId="50">
       <totalsRowFormula>COUNTIF(wednesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="68" totalsRowDxfId="67">
+    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="49" totalsRowDxfId="48">
       <totalsRowFormula>COUNTIF(wednesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="66" totalsRowDxfId="65">
+    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="47" totalsRowDxfId="46">
       <totalsRowFormula>COUNTIF(wednesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2838,33 +2848,33 @@
   <autoFilter ref="B2:O15" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{D80C761D-4E7E-4D1A-862A-6769A723C40C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="64" totalsRowDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="45" totalsRowDxfId="44"/>
     <tableColumn id="5" xr3:uid="{F640E5CE-B0CE-4586-AB64-2F877DC1D9FB}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="63"/>
-    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="43"/>
+    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="42"/>
     <tableColumn id="2" xr3:uid="{76D09C9B-F732-4E1C-945B-A497FD16EFDB}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="61" totalsRowDxfId="16">
+    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="41" totalsRowDxfId="40">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="60" totalsRowDxfId="15">
+    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="39" totalsRowDxfId="38">
       <totalsRowFormula>COUNTIF(thursday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="14">
+    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="37" totalsRowDxfId="36">
       <totalsRowFormula>COUNTIF(thursday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="58" totalsRowDxfId="13">
+    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="34">
       <totalsRowFormula>COUNTIF(thursday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="12">
+    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="33" totalsRowDxfId="32">
       <totalsRowFormula>COUNTIF(thursday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="56" totalsRowDxfId="11">
+    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
       <totalsRowFormula>COUNTIF(thursday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="10">
+    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
       <totalsRowFormula>COUNTIF(thursday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="54" totalsRowDxfId="9">
+    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
       <totalsRowFormula>COUNTIF(thursday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2873,37 +2883,37 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E7AA1501-B84A-474D-B2E1-AAA4E0FD1225}" name="friday" displayName="friday" ref="B2:O26" totalsRowCount="1">
-  <autoFilter ref="B2:O25" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E7AA1501-B84A-474D-B2E1-AAA4E0FD1225}" name="friday" displayName="friday" ref="B2:O22" totalsRowCount="1">
+  <autoFilter ref="B2:O21" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{26906033-DBB1-4850-8A65-B0AABB8EB5B7}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="53" totalsRowDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="123" totalsRowDxfId="122"/>
     <tableColumn id="5" xr3:uid="{B474477F-00C6-4EE7-A8CC-63E5347553DE}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="52"/>
+    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="121"/>
     <tableColumn id="14" xr3:uid="{DF3B0E26-BDAD-42AF-AA94-ECF071ABBC93}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{FDADF079-31AD-4240-B382-130BDA5B792F}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="51" totalsRowDxfId="7">
+    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="120" totalsRowDxfId="119">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="50" totalsRowDxfId="6">
+    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="118" totalsRowDxfId="117">
       <totalsRowFormula>COUNTIF(friday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="49" totalsRowDxfId="5">
+    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="116" totalsRowDxfId="115">
       <totalsRowFormula>COUNTIF(friday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="4">
+    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="114" totalsRowDxfId="113">
       <totalsRowFormula>COUNTIF(friday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="47" totalsRowDxfId="3">
+    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="112" totalsRowDxfId="111">
       <totalsRowFormula>COUNTIF(friday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="2">
+    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="110" totalsRowDxfId="109">
       <totalsRowFormula>COUNTIF(friday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="45" totalsRowDxfId="1">
+    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="108" totalsRowDxfId="107">
       <totalsRowFormula>COUNTIF(friday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="44" totalsRowDxfId="0">
+    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="106" totalsRowDxfId="105">
       <totalsRowFormula>COUNTIF(friday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2912,35 +2922,35 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="43" dataDxfId="41" headerRowBorderDxfId="42" tableBorderDxfId="40" totalsRowBorderDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
   <autoFilter ref="B3:I8" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}"/>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="38" totalsRowDxfId="37"/>
-    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="36" totalsRowDxfId="35">
+    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="20" totalsRowDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="18" totalsRowDxfId="17">
       <calculatedColumnFormula>COUNTIF(monday[Copilot],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Copilot])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="34" totalsRowDxfId="33">
+    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="16" totalsRowDxfId="15">
       <calculatedColumnFormula>COUNTIF(monday[Claude],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Claude])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="32" totalsRowDxfId="31">
+    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="13">
       <calculatedColumnFormula>COUNTIF(monday[Visual Studio],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Visual Studio])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="30" totalsRowDxfId="29">
+    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="11">
       <calculatedColumnFormula>COUNTIF(monday[VS Code],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[VS Code])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="28" totalsRowDxfId="27">
+    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
       <calculatedColumnFormula>COUNTIF(monday[GitHub],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[GitHub])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="26" totalsRowDxfId="25">
+    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
       <calculatedColumnFormula>COUNTIF(monday[AzDO],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[AzDO])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="24" totalsRowDxfId="23">
+    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="6" totalsRowDxfId="5">
       <calculatedColumnFormula>COUNTIF(monday[Agnostic],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Agnostic])</totalsRowFormula>
     </tableColumn>
@@ -2950,12 +2960,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="C16:E23" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3299,42 +3309,42 @@
   <sheetData>
     <row r="3" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C3" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D3" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="E3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>302</v>
+        <v>288</v>
       </c>
       <c r="D4" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^chat-mode.pptx</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>301</v>
+        <v>287</v>
       </c>
     </row>
     <row r="5" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C5" t="s">
-        <v>285</v>
+        <v>271</v>
       </c>
       <c r="D5" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^creating robust testing frameworks.pptx</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>284</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C6" t="s">
-        <v>276</v>
+        <v>262</v>
       </c>
       <c r="D6" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3344,7 +3354,7 @@
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C7" t="s">
-        <v>266</v>
+        <v>252</v>
       </c>
       <c r="D7" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3354,7 +3364,7 @@
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C8" t="s">
-        <v>265</v>
+        <v>251</v>
       </c>
       <c r="D8" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3364,7 +3374,7 @@
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C9" t="s">
-        <v>264</v>
+        <v>250</v>
       </c>
       <c r="D9" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3374,7 +3384,7 @@
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>263</v>
+        <v>249</v>
       </c>
       <c r="D10" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3384,7 +3394,7 @@
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>262</v>
+        <v>248</v>
       </c>
       <c r="D11" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3394,7 +3404,7 @@
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C12" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
       <c r="D12" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3404,7 +3414,7 @@
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C13" t="s">
-        <v>260</v>
+        <v>246</v>
       </c>
       <c r="D13" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3414,7 +3424,7 @@
     </row>
     <row r="14" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C14" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="D14" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3424,7 +3434,7 @@
     </row>
     <row r="15" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C15" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="D15" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3434,247 +3444,247 @@
     </row>
     <row r="16" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C16" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="D16" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>^overview of llms.pptx</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C17" t="s">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="D17" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_advanced context techniques.pptx</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
     </row>
     <row r="18" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C18" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="D18" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai practitioner resources.pptx</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
     </row>
     <row r="19" spans="3:5" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C19" t="s">
-        <v>315</v>
+        <v>300</v>
       </c>
       <c r="D19" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai-development-approaches-comparison.pptx</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>312</v>
+        <v>298</v>
       </c>
     </row>
     <row r="20" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C20" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
       <c r="D20" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_ai-first-vs-prompt-first.pptx</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>309</v>
+        <v>295</v>
       </c>
     </row>
     <row r="21" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C21" t="s">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="D21" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_building a backlog.pptx</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>306</v>
+        <v>292</v>
       </c>
     </row>
     <row r="22" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C22" t="s">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="D22" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_building safety nets.pptx</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C23" t="s">
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="D23" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_conformance &amp; gap analysis.pptx</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>299</v>
+        <v>285</v>
       </c>
     </row>
     <row r="24" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C24" t="s">
-        <v>297</v>
+        <v>283</v>
       </c>
       <c r="D24" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot instruction stack.pptx</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>292</v>
+        <v>278</v>
       </c>
     </row>
     <row r="25" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C25" t="s">
-        <v>298</v>
+        <v>284</v>
       </c>
       <c r="D25" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot-instruction-control.pptx</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
     </row>
     <row r="26" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C26" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
       <c r="D26" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_copilot-instruction-files-vs-prompt-files-vs-chatmodes.pptx</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>289</v>
+        <v>275</v>
       </c>
     </row>
     <row r="27" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C27" t="s">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="D27" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_core instruction files.pptx</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>294</v>
+        <v>280</v>
       </c>
     </row>
     <row r="28" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C28" t="s">
-        <v>288</v>
+        <v>274</v>
       </c>
       <c r="D28" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_cqrs-architecture.pptx</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
     </row>
     <row r="29" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C29" t="s">
-        <v>283</v>
+        <v>269</v>
       </c>
       <c r="D29" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_custom agents.pptx</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>281</v>
+        <v>267</v>
       </c>
     </row>
     <row r="30" spans="3:5" ht="114" x14ac:dyDescent="0.45">
       <c r="C30" t="s">
-        <v>280</v>
+        <v>266</v>
       </c>
       <c r="D30" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_documentation generation &amp; code analysis.pptx</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>279</v>
+        <v>265</v>
       </c>
     </row>
     <row r="31" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C31" t="s">
-        <v>278</v>
+        <v>264</v>
       </c>
       <c r="D31" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_essential safety measures.pptx</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>277</v>
+        <v>263</v>
       </c>
     </row>
     <row r="32" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C32" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
       <c r="D32" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_generating implementation prompts &amp; verification.pptx</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>274</v>
+        <v>260</v>
       </c>
     </row>
     <row r="33" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C33" t="s">
-        <v>273</v>
+        <v>259</v>
       </c>
       <c r="D33" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_getting started checklist.pptx</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>272</v>
+        <v>258</v>
       </c>
     </row>
     <row r="34" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C34" t="s">
-        <v>271</v>
+        <v>257</v>
       </c>
       <c r="D34" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_github copilot for teams.pptx</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
     </row>
     <row r="35" spans="3:5" ht="57" x14ac:dyDescent="0.45">
       <c r="C35" t="s">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="D35" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_github-copilot-chat-mode-personas.pptx</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
     </row>
     <row r="36" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C36" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="D36" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3684,127 +3694,127 @@
     </row>
     <row r="37" spans="3:5" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C37" t="s">
-        <v>258</v>
+        <v>244</v>
       </c>
       <c r="D37" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_implementing-vertical-slices.pptx</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>257</v>
+        <v>243</v>
       </c>
     </row>
     <row r="38" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C38" t="s">
-        <v>256</v>
+        <v>242</v>
       </c>
       <c r="D38" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instruction files.pptx</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
     </row>
     <row r="39" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C39" t="s">
-        <v>254</v>
+        <v>240</v>
       </c>
       <c r="D39" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instruction-file-applyto-patterns.pptx</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
     </row>
     <row r="40" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C40" t="s">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="D40" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_instructions vs prompts vs custom chat modes.pptx</v>
       </c>
       <c r="E40" t="s">
-        <v>246</v>
+        <v>233</v>
       </c>
     </row>
     <row r="41" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C41" t="s">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="D41" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_managing github copilot effectively.pptx</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>245</v>
+        <v>232</v>
       </c>
     </row>
     <row r="42" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C42" t="s">
-        <v>244</v>
+        <v>231</v>
       </c>
       <c r="D42" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_mcp servers.pptx</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
     </row>
     <row r="43" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C43" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="D43" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_mcp-servers-vscode-copilot.pptx</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
     </row>
     <row r="44" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C44" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="D44" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_model selection &amp; comparison.pptx</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
     </row>
     <row r="45" spans="3:5" ht="85.5" x14ac:dyDescent="0.45">
       <c r="C45" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="D45" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_multi‑model implementation comparison.pptx</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
     </row>
     <row r="46" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C46" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="D46" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_prompt files.pptx</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
     </row>
     <row r="47" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C47" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="D47" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3814,31 +3824,31 @@
     </row>
     <row r="48" spans="3:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="C48" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="D48" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_safe brownfield coding.pptx</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
     </row>
     <row r="49" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C49" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="D49" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_starting with project requirements.pptx</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
     </row>
     <row r="50" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C50" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="D50" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3848,7 +3858,7 @@
     </row>
     <row r="51" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C51" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="D51" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3858,7 +3868,7 @@
     </row>
     <row r="52" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C52" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="D52" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3868,7 +3878,7 @@
     </row>
     <row r="53" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C53" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="D53" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3878,7 +3888,7 @@
     </row>
     <row r="54" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C54" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="D54" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3888,7 +3898,7 @@
     </row>
     <row r="55" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C55" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="D55" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3898,7 +3908,7 @@
     </row>
     <row r="56" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C56" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="D56" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3908,7 +3918,7 @@
     </row>
     <row r="57" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C57" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="D57" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3918,7 +3928,7 @@
     </row>
     <row r="58" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C58" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="D58" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
@@ -3928,26 +3938,26 @@
     </row>
     <row r="59" spans="3:5" ht="156.75" x14ac:dyDescent="0.45">
       <c r="C59" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="D59" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>adding ai guardrails.pptx</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
     </row>
     <row r="60" spans="3:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="C60" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="D60" t="str">
         <f>LOWER(Table11[[#This Row],[Name]])</f>
         <v>_addressing technical debt.pptx</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -3987,10 +3997,10 @@
         <v>4</v>
       </c>
       <c r="G2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="H2" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>28</v>
@@ -4031,10 +4041,10 @@
         <v>6</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>325</v>
+        <v>310</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="I3" s="6" t="str">
         <f>I2</f>
@@ -4064,19 +4074,19 @@
     </row>
     <row r="4" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="E4">
         <v>5</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="G4" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="I4" s="1">
         <f>I3 + (E3/ 1440)</f>
@@ -4115,13 +4125,13 @@
         <v>10</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>310</v>
+        <v>296</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" ref="I5:I30" si="0">I4 + (E4/ 1440)</f>
@@ -4157,7 +4167,7 @@
         <v>10</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>33</v>
@@ -4200,10 +4210,10 @@
         <v>15</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>327</v>
+        <v>312</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="1">
@@ -4234,16 +4244,16 @@
     </row>
     <row r="8" spans="3:16" ht="57" x14ac:dyDescent="0.45">
       <c r="C8" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="E8">
         <v>70</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="H8" s="2">
         <v>2</v>
@@ -4276,7 +4286,7 @@
     </row>
     <row r="9" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C9" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -4285,7 +4295,7 @@
         <v>11</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="H9" s="2">
         <v>11</v>
@@ -4318,7 +4328,7 @@
     </row>
     <row r="10" spans="3:16" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -4327,7 +4337,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="H10" s="2">
         <v>12</v>
@@ -4360,16 +4370,16 @@
     </row>
     <row r="11" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="E11">
         <v>0</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="H11" s="2">
         <v>13</v>
@@ -4402,16 +4412,16 @@
     </row>
     <row r="12" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C12" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="H12" s="2">
         <v>14</v>
@@ -4444,16 +4454,16 @@
     </row>
     <row r="13" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C13" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="E13">
         <v>0</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="H13" s="2">
         <v>15</v>
@@ -4498,7 +4508,7 @@
         <v>13</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>336</v>
+        <v>321</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="1">
@@ -4541,7 +4551,7 @@
         <v>15</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>337</v>
+        <v>322</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="1">
@@ -4784,7 +4794,7 @@
         <v>27</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>338</v>
+        <v>323</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="1">
@@ -4827,7 +4837,7 @@
         <v>25</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="1">
@@ -4858,13 +4868,13 @@
     </row>
     <row r="23" spans="3:16" ht="128.25" x14ac:dyDescent="0.45">
       <c r="C23" t="s">
-        <v>324</v>
+        <v>309</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="1">
@@ -4895,13 +4905,13 @@
     </row>
     <row r="24" spans="3:16" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C24" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>255</v>
+        <v>241</v>
       </c>
       <c r="G24" t="s">
-        <v>251</v>
+        <v>237</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="1">
@@ -4932,13 +4942,13 @@
     </row>
     <row r="25" spans="3:16" ht="99.75" x14ac:dyDescent="0.45">
       <c r="C25" t="s">
-        <v>253</v>
+        <v>239</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>328</v>
+        <v>313</v>
       </c>
       <c r="H25" s="2"/>
       <c r="I25" s="1">
@@ -4975,10 +4985,10 @@
         <v>40</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>295</v>
+        <v>281</v>
       </c>
       <c r="H26" s="2"/>
       <c r="I26" s="1">
@@ -5015,10 +5025,10 @@
         <v>5</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
       <c r="H27" s="2"/>
       <c r="I27" s="1">
@@ -5055,10 +5065,10 @@
         <v>15</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>341</v>
+        <v>326</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="1">
@@ -5095,10 +5105,10 @@
         <v>20</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="G29" t="s">
-        <v>342</v>
+        <v>327</v>
       </c>
       <c r="I29" s="1">
         <f t="shared" si="0"/>
@@ -5134,10 +5144,10 @@
         <v>5</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="G30" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="I30" s="1">
         <f t="shared" si="0"/>
@@ -5233,10 +5243,10 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="G2" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>28</v>
@@ -5275,7 +5285,7 @@
       </c>
       <c r="E3" s="2"/>
       <c r="F3" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="H3" s="6" t="str">
         <f>H2</f>
@@ -5312,10 +5322,10 @@
         <v>5</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="F4" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
       <c r="H4" s="1">
         <f t="shared" ref="H4:H24" si="0">H3 + (D3/ 1440)</f>
@@ -5352,10 +5362,10 @@
         <v>5</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="F5" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
       <c r="H5" s="1">
         <f t="shared" si="0"/>
@@ -5385,7 +5395,7 @@
     </row>
     <row r="6" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B6" s="3" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C6" s="7">
         <v>6.2500000000000003E-3</v>
@@ -5397,7 +5407,7 @@
         <v>7</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>354</v>
+        <v>339</v>
       </c>
       <c r="G6" s="2"/>
       <c r="H6" s="1">
@@ -5440,7 +5450,7 @@
         <v>8</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="1">
@@ -5480,10 +5490,10 @@
         <v>20</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="F8" t="s">
-        <v>347</v>
+        <v>332</v>
       </c>
       <c r="H8" s="1">
         <f>H9 + (D9/ 1440)</f>
@@ -5525,7 +5535,7 @@
         <v>10</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="1">
@@ -5565,10 +5575,10 @@
         <v>10</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="F10" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
       <c r="H10" s="1">
         <f>H8 + (D8/ 1440)</f>
@@ -5598,16 +5608,16 @@
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="D11">
         <v>15</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F11" t="s">
-        <v>348</v>
+        <v>333</v>
       </c>
       <c r="H11" s="1">
         <f>H10 + (D10/ 1440)</f>
@@ -5637,7 +5647,7 @@
     </row>
     <row r="12" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>349</v>
+        <v>334</v>
       </c>
       <c r="C12" s="1">
         <v>2.013888888888889E-2</v>
@@ -5646,10 +5656,10 @@
         <v>20</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="F12" t="s">
-        <v>350</v>
+        <v>335</v>
       </c>
       <c r="H12" s="1">
         <f>H11 + (D11/ 1440)</f>
@@ -5688,10 +5698,10 @@
         <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="F13" t="s">
-        <v>351</v>
+        <v>336</v>
       </c>
       <c r="H13" s="1">
         <f>H12 + (D12/ 1440)</f>
@@ -5763,10 +5773,10 @@
         <v>20</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="F15" t="s">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="H15" s="1">
         <f t="shared" si="0"/>
@@ -5805,10 +5815,10 @@
         <v>10</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="F16" t="s">
-        <v>353</v>
+        <v>338</v>
       </c>
       <c r="H16" s="1">
         <f t="shared" si="0"/>
@@ -5844,10 +5854,10 @@
         <v>10</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F17" t="s">
-        <v>355</v>
+        <v>340</v>
       </c>
       <c r="H17" s="1">
         <f t="shared" si="0"/>
@@ -5883,10 +5893,10 @@
         <v>10</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F18" t="s">
-        <v>346</v>
+        <v>331</v>
       </c>
       <c r="H18" s="1">
         <f t="shared" si="0"/>
@@ -5922,10 +5932,10 @@
         <v>5</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F19" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="H19" s="1">
         <f t="shared" si="0"/>
@@ -5955,16 +5965,16 @@
     </row>
     <row r="20" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D20">
         <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F20" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="H20" s="1">
         <f t="shared" si="0"/>
@@ -6000,10 +6010,10 @@
         <v>5</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F21" t="s">
-        <v>356</v>
+        <v>341</v>
       </c>
       <c r="H21" s="1">
         <f t="shared" si="0"/>
@@ -6042,10 +6052,10 @@
         <v>15</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F22" t="s">
-        <v>345</v>
+        <v>330</v>
       </c>
       <c r="H22" s="1" t="e">
         <f>#REF! + (#REF!/ 1440)</f>
@@ -6084,10 +6094,10 @@
         <v>10</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="F23" t="s">
-        <v>357</v>
+        <v>342</v>
       </c>
       <c r="H23" s="1" t="e">
         <f t="shared" si="0"/>
@@ -6126,10 +6136,10 @@
         <v>5</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F24" t="s">
-        <v>344</v>
+        <v>329</v>
       </c>
       <c r="H24" s="1" t="e">
         <f t="shared" si="0"/>
@@ -6225,10 +6235,10 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="G2" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>28</v>
@@ -6295,13 +6305,13 @@
     </row>
     <row r="4" spans="2:15" ht="199.5" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>246</v>
+        <v>233</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>313</v>
+        <v>299</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>314</v>
+        <v>363</v>
       </c>
       <c r="H4" s="6">
         <f>H3 + (D3/ 1440)</f>
@@ -6337,10 +6347,10 @@
         <v>15</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>282</v>
+        <v>268</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>211</v>
+        <v>364</v>
       </c>
       <c r="H5" s="1">
         <f>H3 + (D3/ 1440)</f>
@@ -6370,13 +6380,13 @@
     </row>
     <row r="6" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>268</v>
+        <v>254</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>267</v>
+        <v>253</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>204</v>
+        <v>365</v>
       </c>
       <c r="H6" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6406,17 +6416,17 @@
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B7" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="4">
         <v>15</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="H7" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6446,16 +6456,16 @@
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D8">
         <v>40</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>222</v>
+        <v>370</v>
       </c>
       <c r="H8" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -6485,15 +6495,17 @@
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="D9">
         <v>40</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="F9" s="2"/>
+        <v>145</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>369</v>
+      </c>
       <c r="H9" s="1">
         <f>H8 + (D8/ 1440)</f>
         <v>0.47569444444444453</v>
@@ -6528,9 +6540,11 @@
         <v>5</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="F10" s="2"/>
+        <v>117</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>367</v>
+      </c>
       <c r="H10" s="1">
         <f>H9 + (D9/ 1440)</f>
         <v>0.50347222222222232</v>
@@ -6566,10 +6580,10 @@
         <v>15</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>243</v>
+        <v>368</v>
       </c>
       <c r="H11" s="1">
         <f>H10 + (D10/ 1440)</f>
@@ -6599,14 +6613,14 @@
     </row>
     <row r="12" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
       <c r="B12" s="11" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="13">
         <v>40</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F12" s="2"/>
       <c r="H12" s="1">
@@ -6703,10 +6717,10 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="G2" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>28</v>
@@ -6779,10 +6793,10 @@
         <v>20</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>359</v>
+        <v>343</v>
       </c>
       <c r="H4" s="1">
         <f>H3 + (D3/ 1440)</f>
@@ -6812,13 +6826,13 @@
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D5">
         <v>10</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F5" s="2"/>
       <c r="H5" s="1">
@@ -6847,18 +6861,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="D6">
         <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>360</v>
+        <v>371</v>
       </c>
       <c r="H6" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6894,10 +6908,10 @@
         <v>10</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>304</v>
+        <v>290</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
       <c r="H7" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -6933,10 +6947,10 @@
         <v>15</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>361</v>
+        <v>119</v>
+      </c>
+      <c r="F8" t="s">
+        <v>344</v>
       </c>
       <c r="H8" s="1">
         <f t="shared" ref="H8:H15" si="0">H7 + (D7/ 1440)</f>
@@ -6972,10 +6986,10 @@
         <v>20</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>362</v>
+        <v>120</v>
+      </c>
+      <c r="F9" t="s">
+        <v>345</v>
       </c>
       <c r="H9" s="1">
         <f t="shared" si="0"/>
@@ -7011,10 +7025,10 @@
         <v>45</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>307</v>
+        <v>293</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>363</v>
+        <v>346</v>
       </c>
       <c r="H10" s="1">
         <f t="shared" si="0"/>
@@ -7085,10 +7099,10 @@
         <v>15</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>364</v>
+        <v>347</v>
       </c>
       <c r="H12" s="1">
         <f t="shared" si="0"/>
@@ -7124,10 +7138,10 @@
         <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>366</v>
+        <v>349</v>
       </c>
       <c r="H13" s="1">
         <f t="shared" si="0"/>
@@ -7163,10 +7177,10 @@
         <v>45</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>367</v>
+        <v>121</v>
+      </c>
+      <c r="F14" t="s">
+        <v>372</v>
       </c>
       <c r="H14" s="1">
         <f t="shared" si="0"/>
@@ -7202,10 +7216,10 @@
         <v>30</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>365</v>
+        <v>348</v>
       </c>
       <c r="H15" s="1">
         <f t="shared" si="0"/>
@@ -7276,7 +7290,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD15E000-1B92-41C3-BF19-4CD4B65C581F}">
-  <dimension ref="B2:O26"/>
+  <dimension ref="B2:O22"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="40.06640625" customWidth="1"/>
@@ -7301,10 +7315,10 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="G2" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>28</v>
@@ -7377,10 +7391,10 @@
         <v>5</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F4" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="H4" s="1">
         <f>H3 + (D3/ 1440)</f>
@@ -7419,7 +7433,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F5"/>
       <c r="H5" s="1">
@@ -7456,10 +7470,10 @@
         <v>10</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="F6" t="s">
-        <v>369</v>
+        <v>126</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>351</v>
       </c>
       <c r="H6" s="1">
         <f>H5 + (D5/ 1440)</f>
@@ -7495,10 +7509,10 @@
         <v>5</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="F7" t="s">
-        <v>370</v>
+        <v>127</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>352</v>
       </c>
       <c r="H7" s="1">
         <f>H6 + (D6/ 1440)</f>
@@ -7528,13 +7542,13 @@
     </row>
     <row r="8" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="F8" t="s">
-        <v>371</v>
+        <v>353</v>
       </c>
       <c r="H8" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -7570,10 +7584,10 @@
         <v>15</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F9" t="s">
-        <v>372</v>
+        <v>354</v>
       </c>
       <c r="H9" s="1">
         <f>H7 + (D7/ 1440)</f>
@@ -7603,13 +7617,13 @@
     </row>
     <row r="10" spans="2:15" ht="71.25" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="F10" t="s">
-        <v>373</v>
+        <v>355</v>
       </c>
       <c r="H10" s="1">
         <f>H9 + (D9/ 1440)</f>
@@ -7645,10 +7659,10 @@
         <v>15</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="F11" t="s">
-        <v>374</v>
+        <v>356</v>
       </c>
       <c r="H11" s="1">
         <f>H9 + (D9/ 1440)</f>
@@ -7684,13 +7698,13 @@
         <v>20</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F12" t="s">
-        <v>220</v>
+        <v>357</v>
       </c>
       <c r="H12" s="1">
-        <f t="shared" ref="H12:H25" si="0">H11 + (D11/ 1440)</f>
+        <f t="shared" ref="H12:H21" si="0">H11 + (D11/ 1440)</f>
         <v>0.46527777777777779</v>
       </c>
       <c r="I12" s="5" t="b">
@@ -7723,7 +7737,10 @@
         <v>15</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>134</v>
+        <v>130</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>358</v>
       </c>
       <c r="H13" s="1">
         <f t="shared" si="0"/>
@@ -7759,9 +7776,11 @@
         <v>5</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F14"/>
+        <v>133</v>
+      </c>
+      <c r="F14" t="s">
+        <v>359</v>
+      </c>
       <c r="H14" s="1">
         <f t="shared" si="0"/>
         <v>0.48958333333333337</v>
@@ -7788,131 +7807,135 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>85</v>
+        <v>29</v>
       </c>
       <c r="D15">
-        <v>5</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>140</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="E15" s="2"/>
       <c r="F15"/>
-      <c r="H15" s="1">
+      <c r="H15" s="1" t="e">
+        <f>#REF! + (#REF!/ 1440)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="I15" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J15" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K15" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L15" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O15" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" ht="57" x14ac:dyDescent="0.45">
+      <c r="B16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D16">
+        <v>20</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F16" t="s">
+        <v>360</v>
+      </c>
+      <c r="H16" s="1" t="e">
         <f t="shared" si="0"/>
-        <v>0.49305555555555558</v>
-      </c>
-      <c r="I15" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J15" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K15" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="L15" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="M15" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N15" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O15" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B16" t="s">
-        <v>86</v>
-      </c>
-      <c r="D16">
+        <v>#REF!</v>
+      </c>
+      <c r="I16" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J16" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K16" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L16" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M16" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N16" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
+      <c r="B17" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17">
+        <v>40</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F17" t="s">
+        <v>236</v>
+      </c>
+      <c r="H17" s="1" t="e">
+        <f t="shared" si="0"/>
+        <v>#REF!</v>
+      </c>
+      <c r="I17" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K17" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L17" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M17" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N17" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O17" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="B18" t="s">
+        <v>84</v>
+      </c>
+      <c r="D18">
         <v>10</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="F16"/>
-      <c r="H16" s="1">
-        <f t="shared" si="0"/>
-        <v>0.49652777777777779</v>
-      </c>
-      <c r="I16" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J16" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K16" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="L16" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="M16" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N16" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O16" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="B17" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17">
-        <v>60</v>
-      </c>
-      <c r="E17" s="2"/>
-      <c r="F17"/>
-      <c r="H17" s="1">
-        <f t="shared" si="0"/>
-        <v>0.50347222222222221</v>
-      </c>
-      <c r="I17" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J17" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K17" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L17" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M17" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N17" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O17" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="2:15" ht="57" x14ac:dyDescent="0.45">
-      <c r="B18" t="s">
-        <v>79</v>
-      </c>
-      <c r="D18">
-        <v>20</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>135</v>
       </c>
       <c r="F18" t="s">
-        <v>249</v>
-      </c>
-      <c r="H18" s="1">
+        <v>362</v>
+      </c>
+      <c r="H18" s="1" t="e">
         <f t="shared" si="0"/>
-        <v>0.54513888888888884</v>
+        <v>#REF!</v>
       </c>
       <c r="I18" s="5" t="b">
         <v>0</v>
@@ -7927,31 +7950,31 @@
         <v>0</v>
       </c>
       <c r="M18" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O18" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="2:15" ht="85.5" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D19">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F19" t="s">
-        <v>250</v>
-      </c>
-      <c r="H19" s="1">
-        <f t="shared" si="0"/>
-        <v>0.55902777777777768</v>
+        <v>361</v>
+      </c>
+      <c r="H19" s="1" t="e">
+        <f>#REF! + (#REF!/ 1440)</f>
+        <v>#REF!</v>
       </c>
       <c r="I19" s="5" t="b">
         <v>0</v>
@@ -7966,29 +7989,29 @@
         <v>0</v>
       </c>
       <c r="M19" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19" s="5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" s="5" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D20">
         <v>10</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F20"/>
-      <c r="H20" s="1">
-        <f t="shared" si="0"/>
-        <v>0.58680555555555547</v>
+      <c r="H20" s="1" t="e">
+        <f>#REF! + (#REF!/ 1440)</f>
+        <v>#REF!</v>
       </c>
       <c r="I20" s="5" t="b">
         <v>0</v>
@@ -8012,20 +8035,20 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:15" ht="99.75" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
         <v>87</v>
       </c>
       <c r="D21">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F21"/>
-      <c r="H21" s="1">
+      <c r="H21" s="1" t="e">
         <f t="shared" si="0"/>
-        <v>0.59374999999999989</v>
+        <v>#REF!</v>
       </c>
       <c r="I21" s="5" t="b">
         <v>0</v>
@@ -8049,184 +8072,36 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B22" t="s">
-        <v>88</v>
-      </c>
-      <c r="D22">
-        <v>20</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>143</v>
-      </c>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.45">
       <c r="F22"/>
-      <c r="H22" s="1">
-        <f t="shared" si="0"/>
-        <v>0.5972222222222221</v>
-      </c>
-      <c r="I22" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J22" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K22" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L22" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M22" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="N22" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="O22" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B23" t="s">
-        <v>89</v>
-      </c>
-      <c r="D23">
-        <v>15</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="F23"/>
-      <c r="H23" s="1">
-        <f t="shared" si="0"/>
-        <v>0.61111111111111094</v>
-      </c>
-      <c r="I23" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J23" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K23" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L23" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M23" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N23" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O23" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="2:15" ht="57" x14ac:dyDescent="0.45">
-      <c r="B24" t="s">
-        <v>90</v>
-      </c>
-      <c r="D24">
-        <v>10</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="F24"/>
-      <c r="H24" s="1">
-        <f t="shared" si="0"/>
-        <v>0.62152777777777757</v>
-      </c>
-      <c r="I24" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J24" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K24" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L24" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M24" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="N24" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="O24" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="2:15" ht="99.75" x14ac:dyDescent="0.45">
-      <c r="B25" t="s">
-        <v>91</v>
-      </c>
-      <c r="D25">
-        <v>10</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="F25"/>
-      <c r="H25" s="1">
-        <f t="shared" si="0"/>
-        <v>0.62847222222222199</v>
-      </c>
-      <c r="I25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N25" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O25" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="F26"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="16">
+      <c r="H22" s="1"/>
+      <c r="I22" s="16">
         <f>COUNTIF(friday[Copilot],TRUE)</f>
         <v>0</v>
       </c>
-      <c r="J26" s="16">
+      <c r="J22" s="16">
         <f>COUNTIF(friday[Claude],TRUE)</f>
         <v>0</v>
       </c>
-      <c r="K26" s="16">
+      <c r="K22" s="16">
         <f>COUNTIF(friday[Visual Studio],TRUE)</f>
-        <v>2</v>
-      </c>
-      <c r="L26" s="16">
+        <v>0</v>
+      </c>
+      <c r="L22" s="16">
         <f>COUNTIF(friday[VS Code],TRUE)</f>
-        <v>2</v>
-      </c>
-      <c r="M26" s="16">
+        <v>0</v>
+      </c>
+      <c r="M22" s="16">
         <f>COUNTIF(friday[GitHub],TRUE)</f>
         <v>3</v>
       </c>
-      <c r="N26" s="16">
+      <c r="N22" s="16">
         <f>COUNTIF(friday[AzDO],TRUE)</f>
         <v>3</v>
       </c>
-      <c r="O26" s="16">
+      <c r="O22" s="16">
         <f>COUNTIF(friday[Agnostic],TRUE)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -8253,22 +8128,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.45">
-      <c r="C2" s="25" t="s">
-        <v>169</v>
-      </c>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25" t="s">
-        <v>168</v>
-      </c>
-      <c r="H2" s="25"/>
+      <c r="C2" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B3" s="17" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C3" s="17" t="s">
         <v>39</v>
@@ -8294,7 +8169,7 @@
     </row>
     <row r="4" spans="2:9" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B4" s="18" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C4" s="20">
         <f>COUNTIF(monday[Copilot],TRUE)</f>
@@ -8327,7 +8202,7 @@
     </row>
     <row r="5" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B5" s="19" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="C5" s="20">
         <f>COUNTIF(tuesday[Copilot],TRUE)</f>
@@ -8360,7 +8235,7 @@
     </row>
     <row r="6" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B6" s="19" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="C6" s="20">
         <f>COUNTIF(wednesday[Copilot],TRUE)</f>
@@ -8393,7 +8268,7 @@
     </row>
     <row r="7" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="19" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C7" s="20">
         <f>COUNTIF(thursday[Copilot],TRUE)</f>
@@ -8426,7 +8301,7 @@
     </row>
     <row r="8" spans="2:9" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="19" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C8" s="20">
         <f>COUNTIF(friday[Copilot],TRUE)</f>
@@ -8438,11 +8313,11 @@
       </c>
       <c r="E8" s="20">
         <f>COUNTIF(friday[Visual Studio],TRUE)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F8" s="20">
         <f>COUNTIF(friday[VS Code],TRUE)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G8" s="20">
         <f>COUNTIF(friday[GitHub],TRUE)</f>
@@ -8454,7 +8329,7 @@
       </c>
       <c r="I8" s="20">
         <f>COUNTIF(friday[Agnostic],TRUE)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="2:9" ht="14.65" thickTop="1" x14ac:dyDescent="0.45">
@@ -8469,11 +8344,11 @@
       </c>
       <c r="E9" s="21">
         <f>SUM(Totals[Visual Studio])</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F9" s="21">
         <f>SUM(Totals[VS Code])</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G9" s="21">
         <f>SUM(Totals[GitHub])</f>
@@ -8485,38 +8360,38 @@
       </c>
       <c r="I9" s="21">
         <f>SUM(Totals[Agnostic])</f>
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.45">
       <c r="C16" s="22" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.45">
@@ -8554,7 +8429,7 @@
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C20" s="22" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D20" s="22" t="s">
         <v>41</v>
@@ -8565,7 +8440,7 @@
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C21" s="22" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D21" s="22" t="s">
         <v>41</v>
@@ -8576,7 +8451,7 @@
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C22" s="22" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D22" s="22" t="s">
         <v>42</v>
@@ -8587,7 +8462,7 @@
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.45">
       <c r="C23" s="22" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D23" s="22" t="s">
         <v>42</v>
@@ -8598,20 +8473,20 @@
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G28" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="H28" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G29" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="H29">
         <v>8</v>
@@ -8619,7 +8494,7 @@
     </row>
     <row r="30" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G30" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="H30">
         <v>8</v>
@@ -8627,7 +8502,7 @@
     </row>
     <row r="31" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G31" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="H31">
         <v>2</v>
@@ -8635,7 +8510,7 @@
     </row>
     <row r="32" spans="2:8" x14ac:dyDescent="0.45">
       <c r="G32" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="H32">
         <v>4</v>
@@ -8643,7 +8518,7 @@
     </row>
     <row r="33" spans="7:8" x14ac:dyDescent="0.45">
       <c r="G33" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="H33">
         <v>2</v>
@@ -8676,18 +8551,18 @@
   <sheetData>
     <row r="2" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C2" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="3:5" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="D4" t="s">
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
@@ -8696,7 +8571,7 @@
         <v>GitHub Copilot UI Tour</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -8708,7 +8583,7 @@
         <v>#REF!</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -8720,7 +8595,7 @@
         <v>Code Explanation and Analysis</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="E7">
         <v>2</v>
@@ -8732,7 +8607,7 @@
         <v>MCP (Model Context Protocol) Servers</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="E8">
         <v>2</v>
@@ -8744,7 +8619,7 @@
         <v>Exercise: MCP Servers</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -8752,10 +8627,10 @@
     </row>
     <row r="10" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="E10">
         <v>8</v>
@@ -8763,10 +8638,10 @@
     </row>
     <row r="11" spans="3:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="E11">
         <v>8</v>

</xml_diff>

<commit_message>
feat: add GE course artifacts and Visual Studio decks
</commit_message>
<xml_diff>
--- a/AIASD-311-CourseModules.xlsx
+++ b/AIASD-311-CourseModules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\AIASD\AI-Assisted-Software-Development-Course\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6310788A-54C4-43FA-BE82-F4FF2AC935DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C60AE73D-C509-45D0-985A-0607DD9C36F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4583" yWindow="16103" windowWidth="21795" windowHeight="13875" activeTab="1" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="2" xr2:uid="{88B4C266-A938-4700-99B3-B927BE83C57A}"/>
   </bookViews>
   <sheets>
     <sheet name="decks" sheetId="10" r:id="rId1"/>
@@ -23,7 +23,6 @@
     <sheet name="GE Mods" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -44,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="373">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="374">
   <si>
     <t>CI/CD Pipeline Creation</t>
   </si>
@@ -1163,6 +1162,9 @@
   </si>
   <si>
     <t>exercise-addressing-technical-debt-with-copilot.md</t>
+  </si>
+  <si>
+    <t>implementation-with-vertical-slices.deck.md</t>
   </si>
 </sst>
 </file>
@@ -1415,6 +1417,133 @@
   </cellStyles>
   <dxfs count="124">
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
+          <xfpb:DXFComplement i="0"/>
+        </ext>
+      </extLst>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2261,133 +2390,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{0417FA29-78FA-4A13-93AC-8FF0FAFDF519}">
-          <xfpb:DXFComplement i="0"/>
-        </ext>
-      </extLst>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2696,8 +2698,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{FC954A70-1543-4974-9FF2-C47266E53D4A}" name="Table11" displayName="Table11" ref="C3:E60" totalsRowShown="0">
-  <autoFilter ref="C3:E60" xr:uid="{FC954A70-1543-4974-9FF2-C47266E53D4A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{FC954A70-1543-4974-9FF2-C47266E53D4A}" name="Table11" displayName="Table11" ref="C3:E62" totalsRowShown="0">
+  <autoFilter ref="C3:E62" xr:uid="{FC954A70-1543-4974-9FF2-C47266E53D4A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C4:E60">
     <sortCondition ref="C3:C60"/>
   </sortState>
@@ -2717,7 +2719,7 @@
   <autoFilter ref="C4:E11" xr:uid="{EF1BA374-5AD9-4719-9FF3-682D1B38151C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{7AD14052-080E-4E37-8C5E-B2CB6B097298}" name="Section"/>
-    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{8BA51BD4-A9EE-4BB2-B57E-B34801A8AD27}" name="Description" dataDxfId="19"/>
     <tableColumn id="2" xr3:uid="{3E1642EC-6329-4B91-8040-267B6F5F8CED}" name="Hours" totalsRowFunction="custom">
       <totalsRowFormula>SUM(Table9[Hours])</totalsRowFormula>
     </tableColumn>
@@ -2731,33 +2733,33 @@
   <autoFilter ref="C2:P30" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9D61239E-9B4A-4932-AB0D-EB9D9921B03D}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="103" totalsRowDxfId="102"/>
+    <tableColumn id="4" xr3:uid="{CF6246D8-1B6E-46F2-8EF3-564EEFD687CC}" name="Start Time" dataDxfId="123" totalsRowDxfId="122"/>
     <tableColumn id="5" xr3:uid="{8B6AF1D4-2216-4B85-BA7D-212BA502015B}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description" dataDxfId="101"/>
+    <tableColumn id="6" xr3:uid="{FC719AB4-7DA0-4CF0-A12A-95985F5C6D2E}" name="Description" dataDxfId="121"/>
     <tableColumn id="19" xr3:uid="{6CD3E0DC-278C-498A-A888-BE6341994574}" name="Deck"/>
     <tableColumn id="18" xr3:uid="{7E153D0B-3D6F-4A51-B6D2-9A0BE0E451DA}" name="Slide(s)"/>
-    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="100" totalsRowDxfId="99">
+    <tableColumn id="7" xr3:uid="{3FD97CAC-BAE8-4A66-B92F-17907FB235F2}" name="10:00:00 AM" dataDxfId="120" totalsRowDxfId="119">
       <calculatedColumnFormula>I2 + (E2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="98" totalsRowDxfId="97">
+    <tableColumn id="3" xr3:uid="{8F73E11B-57E7-46FD-9BC8-9F7C420BAC38}" name="Copilot" totalsRowFunction="custom" dataDxfId="118" totalsRowDxfId="117">
       <totalsRowFormula>COUNTIF(monday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="96" totalsRowDxfId="95">
+    <tableColumn id="8" xr3:uid="{00BFAB92-E224-43B6-A531-DC61138A0CA0}" name="Claude" totalsRowFunction="custom" dataDxfId="116" totalsRowDxfId="115">
       <totalsRowFormula>COUNTIF(monday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="94" totalsRowDxfId="93">
+    <tableColumn id="9" xr3:uid="{B5C7E70A-4192-4A1A-BB50-152DBFD69377}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="114" totalsRowDxfId="113">
       <totalsRowFormula>COUNTIF(monday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="92" totalsRowDxfId="91">
+    <tableColumn id="10" xr3:uid="{BA3C10AA-29E4-463F-BAEF-8EB3E8945B13}" name="VS Code" totalsRowFunction="custom" dataDxfId="112" totalsRowDxfId="111">
       <totalsRowFormula>COUNTIF(monday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="90" totalsRowDxfId="89">
+    <tableColumn id="11" xr3:uid="{F8980FA3-83DA-47C4-AFB7-6CF6A869D269}" name="GitHub" totalsRowFunction="custom" dataDxfId="110" totalsRowDxfId="109">
       <totalsRowFormula>COUNTIF(monday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="88" totalsRowDxfId="87">
+    <tableColumn id="12" xr3:uid="{D8820A44-D6A6-42E2-B181-305F5EE9EEC3}" name="AzDO" totalsRowFunction="custom" dataDxfId="108" totalsRowDxfId="107">
       <totalsRowFormula>COUNTIF(monday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="86" totalsRowDxfId="85">
+    <tableColumn id="13" xr3:uid="{14EF33C0-8AAA-4364-B51A-665DB2BE5F06}" name="Agnostic" totalsRowFunction="custom" dataDxfId="106" totalsRowDxfId="105">
       <totalsRowFormula>COUNTIF(monday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2770,33 +2772,33 @@
   <autoFilter ref="B2:O24" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{A79E8443-E3FC-4A2C-83B2-0E581E8FF9B8}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="84" totalsRowDxfId="83"/>
+    <tableColumn id="4" xr3:uid="{74997477-BD6E-4263-B07D-B967AADDCC4B}" name="Start Time" dataDxfId="103" totalsRowDxfId="102"/>
     <tableColumn id="5" xr3:uid="{C37F49DC-8E37-4F56-B136-B64A492DADC4}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="82"/>
+    <tableColumn id="6" xr3:uid="{DF401DF3-0654-4023-93D4-9F6D3305611B}" name="Description" dataDxfId="101"/>
     <tableColumn id="14" xr3:uid="{BD249784-C12F-4B3B-8752-038CF2024DD9}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{E7140FF5-BE1A-4956-A3E4-A572C8619336}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="81" totalsRowDxfId="80">
+    <tableColumn id="7" xr3:uid="{AC2B6381-3A66-4370-B6B2-C3E9DCB6FA43}" name="10:00:00 AM" dataDxfId="100" totalsRowDxfId="99">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="79" totalsRowDxfId="78">
+    <tableColumn id="3" xr3:uid="{B16B187E-86E2-4252-8947-27912248E347}" name="Copilot" totalsRowFunction="custom" dataDxfId="98" totalsRowDxfId="97">
       <totalsRowFormula>COUNTIF(tuesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="77" totalsRowDxfId="76">
+    <tableColumn id="8" xr3:uid="{328999B8-FD8B-4839-8311-45FC5EB6D50E}" name="Claude" totalsRowFunction="custom" dataDxfId="96" totalsRowDxfId="95">
       <totalsRowFormula>COUNTIF(tuesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="75" totalsRowDxfId="74">
+    <tableColumn id="9" xr3:uid="{34EA6EBA-9872-4064-B9A2-2F4F1923665B}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="94" totalsRowDxfId="93">
       <totalsRowFormula>COUNTIF(tuesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="73" totalsRowDxfId="72">
+    <tableColumn id="10" xr3:uid="{A69DFCC9-26FD-4F9A-AE74-129C7FB342B4}" name="VS Code" totalsRowFunction="custom" dataDxfId="92" totalsRowDxfId="91">
       <totalsRowFormula>COUNTIF(tuesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="71" totalsRowDxfId="70">
+    <tableColumn id="11" xr3:uid="{A0474679-DF85-45F0-9952-0B19F3B91232}" name="GitHub" totalsRowFunction="custom" dataDxfId="90" totalsRowDxfId="89">
       <totalsRowFormula>COUNTIF(tuesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="69" totalsRowDxfId="68">
+    <tableColumn id="12" xr3:uid="{7CE7CEA0-1D58-4456-BEE3-FACC7BEBA621}" name="AzDO" totalsRowFunction="custom" dataDxfId="88" totalsRowDxfId="87">
       <totalsRowFormula>COUNTIF(tuesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="67" totalsRowDxfId="66">
+    <tableColumn id="13" xr3:uid="{1C626DD1-4625-488A-B7AC-16AA057A1A0F}" name="Agnostic" totalsRowFunction="custom" dataDxfId="86" totalsRowDxfId="85">
       <totalsRowFormula>COUNTIF(tuesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2809,33 +2811,33 @@
   <autoFilter ref="B2:O12" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{9E7625E1-2B56-4752-B6F8-BF1B9CB4F92C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="65" totalsRowDxfId="64"/>
+    <tableColumn id="4" xr3:uid="{DC994249-3F03-42D7-9369-8492F63A3609}" name="Start Time" dataDxfId="84" totalsRowDxfId="83"/>
     <tableColumn id="5" xr3:uid="{78218F89-BD58-4DD6-9B0D-DCE1B0CA5E74}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="63"/>
-    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="62"/>
+    <tableColumn id="6" xr3:uid="{9BF78A26-DFD1-4FA6-8A13-90E044BF9CF6}" name="Description" dataDxfId="82"/>
+    <tableColumn id="14" xr3:uid="{2A17624B-AB55-4881-A9E9-C5F0EB76662A}" name="Deck" dataDxfId="81"/>
     <tableColumn id="2" xr3:uid="{06859EAF-BB57-49A2-83C0-AA6CD01CE733}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="61" totalsRowDxfId="60">
+    <tableColumn id="7" xr3:uid="{5CB8B7F0-73B0-4AB6-8CAD-73AAC7120336}" name="10:00:00 AM" dataDxfId="80" totalsRowDxfId="79">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="59" totalsRowDxfId="58">
+    <tableColumn id="3" xr3:uid="{52C57E48-213E-4B1B-B6CB-F6F6B19597C6}" name="Copilot" totalsRowFunction="custom" dataDxfId="78" totalsRowDxfId="77">
       <totalsRowFormula>COUNTIF(wednesday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="57" totalsRowDxfId="56">
+    <tableColumn id="8" xr3:uid="{0D5BA76C-D529-453A-9FAA-BF02D249B691}" name="Claude" totalsRowFunction="custom" dataDxfId="76" totalsRowDxfId="75">
       <totalsRowFormula>COUNTIF(wednesday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="55" totalsRowDxfId="54">
+    <tableColumn id="9" xr3:uid="{153E0A8B-602A-4078-A22C-AA416D599897}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="74" totalsRowDxfId="73">
       <totalsRowFormula>COUNTIF(wednesday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="53" totalsRowDxfId="52">
+    <tableColumn id="10" xr3:uid="{03C0F805-9CE7-4D2A-998E-1F7DD639C9BE}" name="VS Code" totalsRowFunction="custom" dataDxfId="72" totalsRowDxfId="71">
       <totalsRowFormula>COUNTIF(wednesday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="51" totalsRowDxfId="50">
+    <tableColumn id="11" xr3:uid="{7C08E3F4-0D07-4067-8415-25B5EA773AA1}" name="GitHub" totalsRowFunction="custom" dataDxfId="70" totalsRowDxfId="69">
       <totalsRowFormula>COUNTIF(wednesday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="49" totalsRowDxfId="48">
+    <tableColumn id="12" xr3:uid="{47D5B1A8-5588-43F5-8363-ACE644E9CB39}" name="AzDO" totalsRowFunction="custom" dataDxfId="68" totalsRowDxfId="67">
       <totalsRowFormula>COUNTIF(wednesday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="47" totalsRowDxfId="46">
+    <tableColumn id="13" xr3:uid="{DB68B21D-4B3C-4D28-AA56-E23ED49750CA}" name="Agnostic" totalsRowFunction="custom" dataDxfId="66" totalsRowDxfId="65">
       <totalsRowFormula>COUNTIF(wednesday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2848,33 +2850,33 @@
   <autoFilter ref="B2:O15" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{D80C761D-4E7E-4D1A-862A-6769A723C40C}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="45" totalsRowDxfId="44"/>
+    <tableColumn id="4" xr3:uid="{7A86A47A-4F2B-4910-A4AF-BDDD69C8349B}" name="Start Time" dataDxfId="64" totalsRowDxfId="63"/>
     <tableColumn id="5" xr3:uid="{F640E5CE-B0CE-4586-AB64-2F877DC1D9FB}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="43"/>
-    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="42"/>
+    <tableColumn id="6" xr3:uid="{2594D38F-32AB-4663-AE35-3BC8F9A7567A}" name="Description" dataDxfId="62"/>
+    <tableColumn id="14" xr3:uid="{B8DD6DEA-7ABC-4794-9C00-21703D00F0B9}" name="Deck" dataDxfId="61"/>
     <tableColumn id="2" xr3:uid="{76D09C9B-F732-4E1C-945B-A497FD16EFDB}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="41" totalsRowDxfId="40">
+    <tableColumn id="7" xr3:uid="{A26CFC55-26C1-4F30-803D-BBF5981DFCA5}" name="10:00:00 AM" dataDxfId="60" totalsRowDxfId="59">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="39" totalsRowDxfId="38">
+    <tableColumn id="3" xr3:uid="{040567B8-43A2-489E-A9CC-73859959BD5C}" name="Copilot" totalsRowFunction="custom" dataDxfId="58" totalsRowDxfId="57">
       <totalsRowFormula>COUNTIF(thursday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="37" totalsRowDxfId="36">
+    <tableColumn id="8" xr3:uid="{8123314B-943D-472F-983B-8523B69999C0}" name="Claude" totalsRowFunction="custom" dataDxfId="56" totalsRowDxfId="55">
       <totalsRowFormula>COUNTIF(thursday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="34">
+    <tableColumn id="9" xr3:uid="{2498F0CF-6AFF-47E1-979B-DE081B427120}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="54" totalsRowDxfId="53">
       <totalsRowFormula>COUNTIF(thursday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="33" totalsRowDxfId="32">
+    <tableColumn id="10" xr3:uid="{913F6E6D-CD6B-4637-B962-BB89DDCA6740}" name="VS Code" totalsRowFunction="custom" dataDxfId="52" totalsRowDxfId="51">
       <totalsRowFormula>COUNTIF(thursday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
+    <tableColumn id="11" xr3:uid="{BC331ED4-BE71-4300-9771-6BE4E6F8E51C}" name="GitHub" totalsRowFunction="custom" dataDxfId="50" totalsRowDxfId="49">
       <totalsRowFormula>COUNTIF(thursday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
+    <tableColumn id="12" xr3:uid="{D1E8199D-E549-4A4D-AE32-B59854B704A5}" name="AzDO" totalsRowFunction="custom" dataDxfId="48" totalsRowDxfId="47">
       <totalsRowFormula>COUNTIF(thursday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
+    <tableColumn id="13" xr3:uid="{761C22D5-EF2F-4F87-9F85-B289C4EAFA34}" name="Agnostic" totalsRowFunction="custom" dataDxfId="46" totalsRowDxfId="45">
       <totalsRowFormula>COUNTIF(thursday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2883,37 +2885,37 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E7AA1501-B84A-474D-B2E1-AAA4E0FD1225}" name="friday" displayName="friday" ref="B2:O22" totalsRowCount="1">
-  <autoFilter ref="B2:O21" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{E7AA1501-B84A-474D-B2E1-AAA4E0FD1225}" name="friday" displayName="friday" ref="B2:O23" totalsRowCount="1">
+  <autoFilter ref="B2:O22" xr:uid="{A2A7F544-4367-4018-8DC9-81CA31EC2612}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{26906033-DBB1-4850-8A65-B0AABB8EB5B7}" name="Topic"/>
-    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="123" totalsRowDxfId="122"/>
+    <tableColumn id="4" xr3:uid="{BDBF7E0D-1B9B-4EA6-8393-3A73A6DB40AA}" name="Start Time" dataDxfId="18" totalsRowDxfId="8"/>
     <tableColumn id="5" xr3:uid="{B474477F-00C6-4EE7-A8CC-63E5347553DE}" name="Duration"/>
-    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="121"/>
+    <tableColumn id="6" xr3:uid="{0AB30286-B74F-4E70-B4F1-CBD65236A925}" name="Description" dataDxfId="17"/>
     <tableColumn id="14" xr3:uid="{DF3B0E26-BDAD-42AF-AA94-ECF071ABBC93}" name="Deck"/>
     <tableColumn id="2" xr3:uid="{FDADF079-31AD-4240-B382-130BDA5B792F}" name="Slides"/>
-    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="120" totalsRowDxfId="119">
+    <tableColumn id="7" xr3:uid="{17FCC81E-88B4-40C8-ABC1-B8AD7F02B4EA}" name="10:00:00 AM" dataDxfId="16" totalsRowDxfId="7">
       <calculatedColumnFormula>H2 + (D2/ 1440)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="118" totalsRowDxfId="117">
+    <tableColumn id="3" xr3:uid="{E3F3161D-9131-432E-959B-E6F0A1281AC5}" name="Copilot" totalsRowFunction="custom" dataDxfId="15" totalsRowDxfId="6">
       <totalsRowFormula>COUNTIF(friday[Copilot],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="116" totalsRowDxfId="115">
+    <tableColumn id="8" xr3:uid="{4141EF85-371E-4375-8C00-1C37E83D6E69}" name="Claude" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="5">
       <totalsRowFormula>COUNTIF(friday[Claude],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="114" totalsRowDxfId="113">
+    <tableColumn id="9" xr3:uid="{9E14D6DD-E032-4528-9C0C-58B736CC7A80}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="13" totalsRowDxfId="4">
       <totalsRowFormula>COUNTIF(friday[Visual Studio],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="112" totalsRowDxfId="111">
+    <tableColumn id="10" xr3:uid="{8F46D2CC-5CBC-48F4-9A4B-3CC4AEAEB311}" name="VS Code" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="3">
       <totalsRowFormula>COUNTIF(friday[VS Code],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="110" totalsRowDxfId="109">
+    <tableColumn id="11" xr3:uid="{D81D028C-428B-4074-8804-73407B951898}" name="GitHub" totalsRowFunction="custom" dataDxfId="11" totalsRowDxfId="2">
       <totalsRowFormula>COUNTIF(friday[GitHub],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="108" totalsRowDxfId="107">
+    <tableColumn id="12" xr3:uid="{4FF24485-BCF2-4202-B4EF-7AD6E0292975}" name="AzDO" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="1">
       <totalsRowFormula>COUNTIF(friday[AzDO],TRUE)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="106" totalsRowDxfId="105">
+    <tableColumn id="13" xr3:uid="{EF5A8DFC-6137-42BC-B9EE-012CF110EF5A}" name="Agnostic" totalsRowFunction="custom" dataDxfId="9" totalsRowDxfId="0">
       <totalsRowFormula>COUNTIF(friday[Agnostic],TRUE)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -2922,35 +2924,35 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}" name="Totals" displayName="Totals" ref="B3:I9" totalsRowCount="1" headerRowDxfId="44" dataDxfId="42" headerRowBorderDxfId="43" tableBorderDxfId="41" totalsRowBorderDxfId="40">
   <autoFilter ref="B3:I8" xr:uid="{7BE215E2-9049-4E20-81CC-83A554BF1101}"/>
   <tableColumns count="8">
-    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="20" totalsRowDxfId="19"/>
-    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="18" totalsRowDxfId="17">
+    <tableColumn id="8" xr3:uid="{C90FAB4F-EDD1-47CD-AEF9-BF085C892241}" name="DOW" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{0B80151C-6332-4045-885D-4147B93941CE}" name="Copilot" totalsRowFunction="custom" dataDxfId="37" totalsRowDxfId="36">
       <calculatedColumnFormula>COUNTIF(monday[Copilot],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Copilot])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="16" totalsRowDxfId="15">
+    <tableColumn id="2" xr3:uid="{C4207A88-8986-426B-BC78-867B36106C7E}" name="Claude" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="34">
       <calculatedColumnFormula>COUNTIF(monday[Claude],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Claude])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="14" totalsRowDxfId="13">
+    <tableColumn id="3" xr3:uid="{55899575-AD3C-46F5-A917-21CD0BF2F3C2}" name="Visual Studio" totalsRowFunction="custom" dataDxfId="33" totalsRowDxfId="32">
       <calculatedColumnFormula>COUNTIF(monday[Visual Studio],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Visual Studio])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="12" totalsRowDxfId="11">
+    <tableColumn id="4" xr3:uid="{5E38F5FE-B835-4536-AEC2-9829AF391F08}" name="VS Code" totalsRowFunction="custom" dataDxfId="31" totalsRowDxfId="30">
       <calculatedColumnFormula>COUNTIF(monday[VS Code],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[VS Code])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="10" totalsRowDxfId="9">
+    <tableColumn id="5" xr3:uid="{56DCFF07-860C-45E3-B43E-A327A8EAFDBD}" name="GitHub" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
       <calculatedColumnFormula>COUNTIF(monday[GitHub],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[GitHub])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="8" totalsRowDxfId="7">
+    <tableColumn id="6" xr3:uid="{F5088BF5-0F50-4520-95EA-55D8BA949BE7}" name="AzDO" totalsRowFunction="custom" dataDxfId="27" totalsRowDxfId="26">
       <calculatedColumnFormula>COUNTIF(monday[AzDO],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[AzDO])</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="6" totalsRowDxfId="5">
+    <tableColumn id="7" xr3:uid="{252AD14A-47C2-48BC-8B33-8D3A247588EF}" name="Agnostic" totalsRowFunction="custom" dataDxfId="25" totalsRowDxfId="24">
       <calculatedColumnFormula>COUNTIF(monday[Agnostic],TRUE)</calculatedColumnFormula>
       <totalsRowFormula>SUM(Totals[Agnostic])</totalsRowFormula>
     </tableColumn>
@@ -2960,12 +2962,12 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}" name="Table3" displayName="Table3" ref="C16:E23" totalsRowShown="0" headerRowDxfId="23">
   <autoFilter ref="C16:E23" xr:uid="{912E96BC-0A44-4EB1-8D25-1D93E5F52B1A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{591572D6-A8EA-493D-8473-133E4763BB61}" name="AIA" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{34DA7748-7B6D-4305-8183-2EF0146134B7}" name="IDE" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{F11CA94F-DD1D-4587-93E7-6E32450B9602}" name="SCC/WI/PR" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3299,7 +3301,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11BDF954-FF19-4C47-AD82-6E7FB7023B19}">
-  <dimension ref="C3:E60"/>
+  <dimension ref="C3:E62"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="3" max="3" width="64.53125" bestFit="1" customWidth="1"/>
@@ -3959,6 +3961,25 @@
       <c r="E60" s="2" t="s">
         <v>305</v>
       </c>
+    </row>
+    <row r="61" spans="3:5" x14ac:dyDescent="0.45">
+      <c r="C61" t="s">
+        <v>373</v>
+      </c>
+      <c r="D61" t="str">
+        <f>LOWER(Table11[[#This Row],[Name]])</f>
+        <v>implementation-with-vertical-slices.deck.md</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="62" spans="3:5" x14ac:dyDescent="0.45">
+      <c r="D62" t="str">
+        <f>LOWER(Table11[[#This Row],[Name]])</f>
+        <v/>
+      </c>
+      <c r="E62" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -7290,7 +7311,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD15E000-1B92-41C3-BF19-4CD4B65C581F}">
-  <dimension ref="B2:O22"/>
+  <dimension ref="B2:O23"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="40.06640625" customWidth="1"/>
@@ -7704,7 +7725,7 @@
         <v>357</v>
       </c>
       <c r="H12" s="1">
-        <f t="shared" ref="H12:H21" si="0">H11 + (D11/ 1440)</f>
+        <f t="shared" ref="H12:H22" si="0">H11 + (D11/ 1440)</f>
         <v>0.46527777777777779</v>
       </c>
       <c r="I12" s="5" t="b">
@@ -7920,95 +7941,89 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
-      <c r="B18" t="s">
+    <row r="18" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="E18" s="2"/>
+      <c r="F18" t="s">
+        <v>373</v>
+      </c>
+      <c r="H18" s="1" t="e">
+        <f>H17 + (D17/ 1440)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="I18" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L18" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M18" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N18" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="2:15" ht="42.75" x14ac:dyDescent="0.45">
+      <c r="B19" t="s">
         <v>84</v>
       </c>
-      <c r="D18">
+      <c r="D19">
         <v>10</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F19" t="s">
         <v>362</v>
       </c>
-      <c r="H18" s="1" t="e">
-        <f t="shared" si="0"/>
+      <c r="H19" s="1" t="e">
+        <f>H17 + (D17/ 1440)</f>
         <v>#REF!</v>
       </c>
-      <c r="I18" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K18" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L18" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M18" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="N18" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="O18" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="B19" t="s">
+      <c r="I19" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J19" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K19" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L19" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M19" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N19" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O19" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="2:15" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="B20" t="s">
         <v>85</v>
       </c>
-      <c r="D19">
+      <c r="D20">
         <v>20</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F20" t="s">
         <v>361</v>
       </c>
-      <c r="H19" s="1" t="e">
-        <f>#REF! + (#REF!/ 1440)</f>
-        <v>#REF!</v>
-      </c>
-      <c r="I19" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J19" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K19" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L19" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M19" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="N19" s="5" t="b">
-        <v>1</v>
-      </c>
-      <c r="O19" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:15" ht="57" x14ac:dyDescent="0.45">
-      <c r="B20" t="s">
-        <v>86</v>
-      </c>
-      <c r="D20">
-        <v>10</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F20"/>
       <c r="H20" s="1" t="e">
         <f>#REF! + (#REF!/ 1440)</f>
         <v>#REF!</v>
@@ -8035,71 +8050,108 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="2:15" ht="99.75" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:15" ht="57" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D21">
         <v>10</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F21"/>
       <c r="H21" s="1" t="e">
+        <f>#REF! + (#REF!/ 1440)</f>
+        <v>#REF!</v>
+      </c>
+      <c r="I21" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K21" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L21" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M21" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N21" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:15" ht="99.75" x14ac:dyDescent="0.45">
+      <c r="B22" t="s">
+        <v>87</v>
+      </c>
+      <c r="D22">
+        <v>10</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F22"/>
+      <c r="H22" s="1" t="e">
         <f t="shared" si="0"/>
         <v>#REF!</v>
       </c>
-      <c r="I21" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="J21" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K21" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="L21" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="M21" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="N21" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="O21" s="5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="F22"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="16">
+      <c r="I22" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K22" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="L22" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M22" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="N22" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O22" s="5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.45">
+      <c r="F23"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="16">
         <f>COUNTIF(friday[Copilot],TRUE)</f>
         <v>0</v>
       </c>
-      <c r="J22" s="16">
+      <c r="J23" s="16">
         <f>COUNTIF(friday[Claude],TRUE)</f>
         <v>0</v>
       </c>
-      <c r="K22" s="16">
+      <c r="K23" s="16">
         <f>COUNTIF(friday[Visual Studio],TRUE)</f>
         <v>0</v>
       </c>
-      <c r="L22" s="16">
+      <c r="L23" s="16">
         <f>COUNTIF(friday[VS Code],TRUE)</f>
         <v>0</v>
       </c>
-      <c r="M22" s="16">
+      <c r="M23" s="16">
         <f>COUNTIF(friday[GitHub],TRUE)</f>
         <v>3</v>
       </c>
-      <c r="N22" s="16">
+      <c r="N23" s="16">
         <f>COUNTIF(friday[AzDO],TRUE)</f>
         <v>3</v>
       </c>
-      <c r="O22" s="16">
+      <c r="O23" s="16">
         <f>COUNTIF(friday[Agnostic],TRUE)</f>
         <v>13</v>
       </c>

</xml_diff>